<commit_message>
Add LTE Spectrum Coordination sheet as the last workbook tab
Document UL/DL decoupling on CA UEs from CA FPD ref 55, related DSS/NSA
parameter text, and CloudAIR/Turkcell material. Cover index updated.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Carrier_Aggregation_Deployment.xlsx
+++ b/Carrier_Aggregation_Deployment.xlsx
@@ -14,6 +14,7 @@
     <sheet name="4. Step2 3CC Config" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="5. Step3 4CC Config" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="6. Step4 5CC Config" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="7. LTE Spectrum Coordination" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'0. Cover &amp; Index'!$1:$3</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'4. Step2 3CC Config'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'5. Step3 4CC Config'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'6. Step4 5CC Config'!$1:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'7. LTE Spectrum Coordination'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -98,7 +100,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -153,6 +155,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -226,7 +233,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -327,6 +334,21 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2261,6 +2283,61 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5810250" cy="3238500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5905500" cy="2190750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2551,7 +2628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2763,7 +2840,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Read sheets 1–2 for concepts. Deploy Step1 (2CC) first, then Step2–4. Each Step sheet is self-contained.</t>
+          <t>Read sheets 1–2 for concepts. Deploy Step1 (2CC) first, then Step2–4. After CA is green, use sheet 7 for LTE Spectrum Coordination (UL/DL decoupling on the CA UE).</t>
         </is>
       </c>
       <c r="C12" s="10" t="n"/>
@@ -2779,7 +2856,7 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Sheet map  (document sequence Ch.3 → Ch.8)</t>
+          <t>Sheet map  (document sequence Ch.3 → Ch.8, then LTE Spectrum Coordination)</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
@@ -3016,54 +3093,83 @@
       <c r="I22" s="10" t="n"/>
       <c r="J22" s="11" t="n"/>
     </row>
-    <row r="23" ht="8" customHeight="1"/>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>7. LTE Spectrum Coordination</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>CA FPD Ch.23 item 55 + related FPDs (DSS, NSA, CellCaAlgoSwitch) + CloudAIR/Turkcell</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Last sheet: UL/DL decoupling on a CA UE — principle, UL-quality PCell trigger, leave, params, MML, counters, KPI, licenses</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="10" t="n"/>
+      <c r="J23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="8" customHeight="1"/>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Recommended live-network sequence</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="6" t="n"/>
-    </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="110" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>•  Confirm overlapping coverage, neighbor relations (NoRmvFlag=FORBID_RMV_ENUM), licenses, UE Rel-10+ (2CC) / Rel-12+ (3CC+), EPC MBR.
 •  Choose Adaptive mode (recommended) unless the cluster is a small fixed co-coverage CA group.
 •  Activate Downlink 2CC, verify counters and KPI, then add 3CC → 4CC → 5CC by turning on CaDl3CCSwitch / CaDl4CCSwitch / CaDl5CCSwitch.
 •  Do not skip 2CC: 3CC/4CC/5CC list Downlink 2CC (and 3CC/4CC as applicable) as prerequisite functions.
+•  After CA is stable on a high/low (or TDD-high + FDD-low) pair, enable LTE Spectrum Coordination (sheet 7) so cell-edge UEs uplink on the coverage layer while DL stays aggregated. Dedicated FPD is CA ref 55 (not in this repo).
 •  Huawei note: this FPD is activation guidance. Feature gains depend on the live scenario; contact Huawei service for optimization.</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
+      <c r="B26" s="14" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="14" t="n"/>
+      <c r="G26" s="14" t="n"/>
+      <c r="H26" s="14" t="n"/>
+      <c r="I26" s="14" t="n"/>
+      <c r="J26" s="14" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="A14:J14"/>
     <mergeCell ref="D18:J18"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="B8:J8"/>
+    <mergeCell ref="D23:J23"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="D20:J20"/>
     <mergeCell ref="B9:J9"/>
-    <mergeCell ref="A24:J24"/>
     <mergeCell ref="D19:J19"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="A1:J1"/>
@@ -3073,6 +3179,7 @@
     <mergeCell ref="B7:J7"/>
     <mergeCell ref="D17:J17"/>
     <mergeCell ref="D16:J16"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="B12:J12"/>
   </mergeCells>
@@ -22953,4 +23060,4599 @@
   </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="000D7377"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:J192"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  7.  LTE Spectrum Coordination   —  UL/DL decoupling on a CA UE  (CloudAIR)</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="72" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Place in the CA FPD: Chapter 23 Reference Documents, item 55. “LTE Spectrum Coordination”.  The dedicated Feature Parameter Description is a separate eRAN document and is NOT attached to this repository.  This sheet therefore uses only statements that appear in the CA FPD, in related Huawei FPDs (DSS, NSA, CellCaAlgoSwitch), and in Huawei public CloudAIR / Turkcell trial material.  Rows marked “Reconstructed MML” use the same MOD CAMGTCFG bit-switch syntax as the CA FPD samples; they are not copied from a Spectrum Coordination MML example.  License models and dedicated counter IDs are not published in the sources below — see License Control Item Lists and the dedicated FPD.</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="n"/>
+      <c r="C2" s="17" t="n"/>
+      <c r="D2" s="17" t="n"/>
+      <c r="E2" s="17" t="n"/>
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="17" t="n"/>
+      <c r="H2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="17" t="n"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>A.  Principal  —  what the feature is and how it sits on Carrier Aggregation</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>A1.  One-sentence definition</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22" t="n"/>
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="22" t="n"/>
+    </row>
+    <row r="5" ht="41" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination is Huawei CloudAIR “channel cloudification” for LTE: it lifts the binding between the uplink channel and the downlink channel of a CA UE so that DL can stay on both the high band and the low band while UL is placed on the band that currently gives the better uplink experience.  Huawei’s published parameter meaning: when SpectrumCoordinationSwitch is selected, PCell changes are triggered based on uplink quality.  Applies to LTE FDD and LTE TDD.  Default of the switch is Off.</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="19" t="n"/>
+      <c r="H5" s="19" t="n"/>
+      <c r="I5" s="19" t="n"/>
+      <c r="J5" s="19" t="n"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>A2.  Why it exists (the coverage mismatch CA does not solve by itself)</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="22" t="n"/>
+      <c r="H6" s="22" t="n"/>
+      <c r="I6" s="22" t="n"/>
+      <c r="J6" s="22" t="n"/>
+    </row>
+    <row r="7" ht="130" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>•  High bands (1800 / 2100 / TDD mid-band) have more spectrum and higher DL peak, but worse UL coverage: UE Tx power is limited (~23 dBm) and path loss + penetration rise with frequency.
+•  Low bands (700 / 800 / 900) have excellent UL coverage but less bandwidth. A UE that camps on the high band as PCell keeps PUCCH/PUSCH on that high-band PCell (unless UL CA is also configured).
+•  Ordinary DL CA already gives the UE both carriers for downlink. It does not by itself move the UL control/data to the low band when the UE is at the cell edge — PCell is still chosen mainly by DL measurements / PCC anchoring.
+•  Spectrum Coordination adds UL-quality-triggered PCell change on top of CA, so the cell-edge UE can keep DL aggregation and still uplink on the coverage layer.
+•  Huawei commercial trial (Turkcell Antalya, eRAN 13.1, Jan 2018): DL hosted by both bands; cell-center UE selects high band as UL; cell-edge UE selects low band as UL. Reported cell-edge downlink data rate increase &gt; 30%.
+•  CloudAIR white paper: usable for FDD high+low, and also for TDD high band paired with FDD low band.</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="19" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1"/>
+    <row r="9" ht="15" customHeight="1"/>
+    <row r="10" ht="15" customHeight="1"/>
+    <row r="11" ht="15" customHeight="1"/>
+    <row r="12" ht="15" customHeight="1"/>
+    <row r="13" ht="15" customHeight="1"/>
+    <row r="14" ht="15" customHeight="1"/>
+    <row r="15" ht="15" customHeight="1"/>
+    <row r="16" ht="15" customHeight="1"/>
+    <row r="17" ht="15" customHeight="1"/>
+    <row r="18" ht="15" customHeight="1"/>
+    <row r="19" ht="15" customHeight="1"/>
+    <row r="20" ht="15" customHeight="1"/>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Figure SC-1  UL/DL decoupling on a CA UE  (schematic reconstructed from Huawei CloudAIR / Turkcell description — not a Huawei FPD original)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>A3.  Relationship to Carrier Aggregation (this workbook)</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+      <c r="F32" s="22" t="n"/>
+      <c r="G32" s="22" t="n"/>
+      <c r="H32" s="22" t="n"/>
+      <c r="I32" s="22" t="n"/>
+      <c r="J32" s="22" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>What CA already does (sheets 1–6)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>What Spectrum Coordination adds</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr"/>
+      <c r="E33" s="7" t="inlineStr"/>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="7" t="inlineStr"/>
+      <c r="I33" s="7" t="inlineStr"/>
+      <c r="J33" s="7" t="inlineStr"/>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>DL user-plane</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Aggregates 2–5 (up to 8) CCs after SCell activation (MAC CE). Peak = sum of CCs, capped by BBP and UE category.</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Does not replace CA. DL remains hosted by both high and low bands so cell-edge DL still uses the high-band SCell.</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="10" t="n"/>
+      <c r="I34" s="10" t="n"/>
+      <c r="J34" s="11" t="n"/>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>UL user-plane / control</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Default: UL on PCell/PCC. UL 2CC is a separate feature (CA FPD Ch.10, CaUl2CCSwitch).</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Chooses which cell is PCell according to UL quality, so UL rides the better uplink band without requiring UL CA.</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="10" t="n"/>
+      <c r="I35" s="10" t="n"/>
+      <c r="J35" s="11" t="n"/>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>PCell selection</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>PCC anchoring (A1 then A5) + preferred PCell priority / PccFreqCfg. Driven by DL RSRP/RSRQ.</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Additional PCell-change trigger: uplink quality. Can move PCell from high band (center) to low band (edge) and back.</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="10" t="n"/>
+      <c r="I36" s="10" t="n"/>
+      <c r="J36" s="11" t="n"/>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>SCell management</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Ch.4.6 A4 add / A6 change / A2 remove / traffic+CQI activate/deactivate. Unchanged as the state machine.</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>After a UL-quality PCell change, the previous PCell typically remains as SCell so DL CA continues. Do not reuse A1–A6 as the Spectrum Coordination trigger.</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="10" t="n"/>
+      <c r="I37" s="10" t="n"/>
+      <c r="J37" s="11" t="n"/>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Licensing</t>
+        </is>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>LAOFD / TDLAOFD / LEOFD CA licenses in Step1–4.</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Spectrum Coordination is a separate eRAN feature (FDD and TDD names appear on CellCaAlgoSwitch). CA licenses still required because DL CA is the vehicle.</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="10" t="n"/>
+      <c r="I38" s="10" t="n"/>
+      <c r="J38" s="11" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>A4.  What this feature is NOT  (do not mix these on the same change request)</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="22" t="n"/>
+      <c r="F39" s="22" t="n"/>
+      <c r="G39" s="22" t="n"/>
+      <c r="H39" s="22" t="n"/>
+      <c r="I39" s="22" t="n"/>
+      <c r="J39" s="22" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>Look-alike name</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>What it actually is</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Typical switch</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>This sheet?</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr"/>
+      <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="7" t="inlineStr"/>
+      <c r="I40" s="7" t="inlineStr"/>
+      <c r="J40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41" ht="44" customHeight="1">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination (this sheet)</t>
+        </is>
+      </c>
+      <c r="B41" s="29" t="inlineStr">
+        <is>
+          <t>UL/DL decoupling across LTE high/low bands on a CA UE; PCell change on UL quality.</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch → SpectrumCoordinationSwitch</t>
+        </is>
+      </c>
+      <c r="D41" s="29" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="10" t="n"/>
+      <c r="I41" s="10" t="n"/>
+      <c r="J41" s="11" t="n"/>
+    </row>
+    <row r="42" ht="44" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>LTE spectrum coordination enhancement</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>WBB / RRN enhancement of the above. NSA PCC anchoring takes precedence if both on.</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch → WbbCaMultiCarrierCoordSw</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>YES (section D/E)</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="10" t="n"/>
+      <c r="I42" s="10" t="n"/>
+      <c r="J42" s="11" t="n"/>
+    </row>
+    <row r="43" ht="44" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>LTE FDD and NR Flash DSS / Hybrid DSS / SUL DSS</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>4G and 5G share the SAME carrier’s RBs over time. Reduces LTE UL RBs → fewer UEs get Spectrum Coordination.</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>SpectrumCloud.SpectrumCloudSwitch = LTE_NR_SPECTRUM_SHR (or SUL variant)</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Impact only</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="10" t="n"/>
+      <c r="I43" s="10" t="n"/>
+      <c r="J43" s="11" t="n"/>
+    </row>
+    <row r="44" ht="44" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>GSM and LTE Spectrum Concurrency / UMTS–LTE Spectrum Sharing</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>CloudAIR spectrum cloudification between RATs on one band. CA FPD: do not use 5 MHz / GL-concurrency cells as PCell (PUCCH vs SRS).</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>SpectrumCloudSwitch = GL_SPECTRUM_CONCURRENCY or UL_SPECTRUM_SHARING</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>Impact only</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="10" t="n"/>
+      <c r="I44" s="10" t="n"/>
+      <c r="J44" s="11" t="n"/>
+    </row>
+    <row r="45" ht="44" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>2019 “LTE&amp;NR Spectrum Coordination” press note</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Dynamic 4G/5G spectrum allocation on C-band / 2.6 GHz and FDD 2.1 GHz sharing. Different product story from LTE high/low UL decoupling.</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>LTE–NR DSS / sharing family — not SpectrumCoordinationSwitch</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>NO — related but different</t>
+        </is>
+      </c>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="10" t="n"/>
+      <c r="H45" s="10" t="n"/>
+      <c r="I45" s="10" t="n"/>
+      <c r="J45" s="11" t="n"/>
+    </row>
+    <row r="46" ht="44" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>5G UL/DL decoupling (NR SUL / NR FPD item 75 in CA refs)</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>NR uplink on a supplementary or low band while NR DL stays on C-band. Different RAT, different FPD.</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>NR feature documentation “UL and DL Decoupling in 5G RAN”</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+      <c r="H46" s="10" t="n"/>
+      <c r="I46" s="10" t="n"/>
+      <c r="J46" s="11" t="n"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>B.  Triggering conditions  (UL-quality PCell change — not CA A1–A6)</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="6" t="n"/>
+    </row>
+    <row r="48" ht="28" customHeight="1">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>The dedicated FPD’s UL-quality threshold table is not in this repository. What is documented: “Spectrum coordination is enabled only if this option is selected. With spectrum coordination enabled, PCell changes are triggered based on uplink quality. This option applies only to LTE FDD and LTE TDD.”  Default: Off.  Worked numbers below are radio-propagation illustrations so the operations team can see the size of the UL gap; they are not Huawei factory defaults.</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="n"/>
+      <c r="C48" s="17" t="n"/>
+      <c r="D48" s="17" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="17" t="n"/>
+      <c r="G48" s="17" t="n"/>
+      <c r="H48" s="17" t="n"/>
+      <c r="I48" s="17" t="n"/>
+      <c r="J48" s="17" t="n"/>
+    </row>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>Figure SC-2  Enablement and UL-quality PCell change  (reconstructed from CellCaAlgoSwitch meaning + CloudAIR; not a Huawei original figure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="21" t="inlineStr">
+        <is>
+          <t>B1.  Preconditions before the UL-quality trigger can fire</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="n"/>
+      <c r="C66" s="22" t="n"/>
+      <c r="D66" s="22" t="n"/>
+      <c r="E66" s="22" t="n"/>
+      <c r="F66" s="22" t="n"/>
+      <c r="G66" s="22" t="n"/>
+      <c r="H66" s="22" t="n"/>
+      <c r="I66" s="22" t="n"/>
+      <c r="J66" s="22" t="n"/>
+    </row>
+    <row r="67" ht="120" customHeight="1">
+      <c r="A67" s="18" t="inlineStr">
+        <is>
+          <t>•  Downlink CA is already working on the high/low pair (this workbook Step1 as a minimum). Spectrum Coordination does not aggregate carriers by itself.
+•  The two cells overlap in coverage. Neighbors exist (CA FPD: NoRmvFlag = FORBID_RMV_ENUM on CA neighbors).
+•  UE is CA-capable (Rel-10+ for 2CC). Same UE-attribute exclusions as CA still apply (emergency call, eMBMS, eMTC, high-speed rules — see Step1 B1).
+•  SpectrumCoordinationSwitch = On on the cells that will participate (PCell and the partner band). Default is Off, so nothing happens until this bit is selected.
+•  Enough LTE uplink RBs remain on the cell. DSS and UL multi-cluster each reduce the LTE UL RB pool and therefore reduce the proportion of UEs for which Spectrum Coordination takes effect (DSS FPD).
+•  For NSA DC UEs: if RsvdSwPara6_bit20 is selected after Spectrum Coordination is on, the feature is disabled for those UEs (NSA FPD) — they will not be HO’d from PCC to a non-candidate PCC.</t>
+        </is>
+      </c>
+      <c r="B67" s="19" t="n"/>
+      <c r="C67" s="19" t="n"/>
+      <c r="D67" s="19" t="n"/>
+      <c r="E67" s="19" t="n"/>
+      <c r="F67" s="19" t="n"/>
+      <c r="G67" s="19" t="n"/>
+      <c r="H67" s="19" t="n"/>
+      <c r="I67" s="19" t="n"/>
+      <c r="J67" s="19" t="n"/>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="26" t="inlineStr">
+        <is>
+          <t>B2.  Size of the UL problem  —  extra path loss of the high band vs the low band</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="6" t="n"/>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="6" t="n"/>
+      <c r="I68" s="6" t="n"/>
+      <c r="J68" s="6" t="n"/>
+    </row>
+    <row r="69" ht="89" customHeight="1">
+      <c r="A69" s="27" t="inlineStr">
+        <is>
+          <t>3GPP / Huawei condition:
+ΔPL_freq (dB) ≈ 20 · log10(f_high / f_low)     (same distance, free-space / Okumura-style frequency term)
+ΔPL_total ≈ ΔPL_freq + ΔPL_penetration + ΔPL_clutter
+UL SNR_high ≈ (P_UE − PL_high − N) ;   UL SNR_low ≈ (P_UE − PL_low − N)
+With P_UE capped (typically 23 dBm), the high band runs out of UL SNR first. That is the cell-edge trigger region.</t>
+        </is>
+      </c>
+      <c r="B69" s="28" t="n"/>
+      <c r="C69" s="28" t="n"/>
+      <c r="D69" s="28" t="n"/>
+      <c r="E69" s="28" t="n"/>
+      <c r="F69" s="28" t="n"/>
+      <c r="G69" s="28" t="n"/>
+      <c r="H69" s="28" t="n"/>
+      <c r="I69" s="28" t="n"/>
+      <c r="J69" s="28" t="n"/>
+    </row>
+    <row r="70" ht="90" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>Worked example (sample values from the document or typical live-network settings):
+Sample pair used on many LTE CA networks (not a Huawei MML value):
+  High UL ≈ Band 3  1747.5 MHz     Low UL ≈ Band 8  897.5 MHz
+  ΔPL_freq = 20 · log10(1747.5 / 897.5) = 20 · log10(1.947) ≈ 5.8 dB
+  Extra building penetration 1800 vs 900 is typically another ~5 to 10 dB  →  ΔPL_total ≈ 11 to 16 dB at the same location.
+  If a cell-edge UE has UL SINR = −2 dB on the high-band PCell, the same UE on the low band is in the order of +9 to +14 dB, all else equal.
+Result: Spectrum Coordination’s job is to change PCell to the low-band cell in this region so PUCCH/PUSCH ride the coverage layer, while the high-band cell stays as SCell and continues to carry DL. When the UE walks back to the center and high-band UL recovers, PCell can return to the high band.</t>
+        </is>
+      </c>
+      <c r="B70" s="14" t="n"/>
+      <c r="C70" s="14" t="n"/>
+      <c r="D70" s="14" t="n"/>
+      <c r="E70" s="14" t="n"/>
+      <c r="F70" s="14" t="n"/>
+      <c r="G70" s="14" t="n"/>
+      <c r="H70" s="14" t="n"/>
+      <c r="I70" s="14" t="n"/>
+      <c r="J70" s="14" t="n"/>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="21" t="inlineStr">
+        <is>
+          <t>B3.  Worked examples  (operator illustration — not Huawei factory thresholds)</t>
+        </is>
+      </c>
+      <c r="B71" s="22" t="n"/>
+      <c r="C71" s="22" t="n"/>
+      <c r="D71" s="22" t="n"/>
+      <c r="E71" s="22" t="n"/>
+      <c r="F71" s="22" t="n"/>
+      <c r="G71" s="22" t="n"/>
+      <c r="H71" s="22" t="n"/>
+      <c r="I71" s="22" t="n"/>
+      <c r="J71" s="22" t="n"/>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>UE location</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>High-band UL SINR (sample)</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Low-band UL SINR (sample)</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Expected PCell after coordination</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>DL CA state</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr"/>
+      <c r="I72" s="7" t="inlineStr"/>
+      <c r="J72" s="7" t="inlineStr"/>
+    </row>
+    <row r="73" ht="52" customHeight="1">
+      <c r="A73" s="29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>Cell center</t>
+        </is>
+      </c>
+      <c r="C73" s="29" t="inlineStr">
+        <is>
+          <t>+18 dB (good)</t>
+        </is>
+      </c>
+      <c r="D73" s="29" t="inlineStr">
+        <is>
+          <t>+22 dB (also good)</t>
+        </is>
+      </c>
+      <c r="E73" s="29" t="inlineStr">
+        <is>
+          <t>HIGH band (capacity layer)</t>
+        </is>
+      </c>
+      <c r="F73" s="29" t="inlineStr">
+        <is>
+          <t>Both CCs active</t>
+        </is>
+      </c>
+      <c r="G73" s="29" t="inlineStr">
+        <is>
+          <t>UL does not need the coverage layer. Keep PCell on high band so UL uses the typically wider high-band PUSCH.</t>
+        </is>
+      </c>
+      <c r="H73" s="10" t="n"/>
+      <c r="I73" s="10" t="n"/>
+      <c r="J73" s="11" t="n"/>
+    </row>
+    <row r="74" ht="52" customHeight="1">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t>Mid cell</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t>+6 dB</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t>+14 dB</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>Depends on live UL-quality criterion in the dedicated FPD</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Both CCs active</t>
+        </is>
+      </c>
+      <c r="G74" s="12" t="inlineStr">
+        <is>
+          <t>Do not invent a dB threshold. Confirm hysteresis / time-to-trigger in LTE Spectrum Coordination FPD / Parameter Reference to avoid PCell ping-pong.</t>
+        </is>
+      </c>
+      <c r="H74" s="10" t="n"/>
+      <c r="I74" s="10" t="n"/>
+      <c r="J74" s="11" t="n"/>
+    </row>
+    <row r="75" ht="52" customHeight="1">
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B75" s="29" t="inlineStr">
+        <is>
+          <t>Cell edge (Turkcell-class)</t>
+        </is>
+      </c>
+      <c r="C75" s="29" t="inlineStr">
+        <is>
+          <t>−2 dB (UL limited)</t>
+        </is>
+      </c>
+      <c r="D75" s="29" t="inlineStr">
+        <is>
+          <t>+10 dB (usable)</t>
+        </is>
+      </c>
+      <c r="E75" s="29" t="inlineStr">
+        <is>
+          <t>LOW band (coverage layer)</t>
+        </is>
+      </c>
+      <c r="F75" s="29" t="inlineStr">
+        <is>
+          <t>Both CCs active — high band remains SCell for DL</t>
+        </is>
+      </c>
+      <c r="G75" s="29" t="inlineStr">
+        <is>
+          <t>This is the gain region: cell-edge DL rate rose &gt;30% in the 2018 commercial trial because DL still used the high-band SCell while UL survived on low band.</t>
+        </is>
+      </c>
+      <c r="H75" s="10" t="n"/>
+      <c r="I75" s="10" t="n"/>
+      <c r="J75" s="11" t="n"/>
+    </row>
+    <row r="76" ht="52" customHeight="1">
+      <c r="A76" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="inlineStr">
+        <is>
+          <t>Cell edge, CA not configured</t>
+        </is>
+      </c>
+      <c r="C76" s="12" t="inlineStr">
+        <is>
+          <t>−2 dB</t>
+        </is>
+      </c>
+      <c r="D76" s="12" t="inlineStr">
+        <is>
+          <t>+10 dB</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>Idle/connected reselection or coverage HO only — no SC</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>Single carrier</t>
+        </is>
+      </c>
+      <c r="G76" s="12" t="inlineStr">
+        <is>
+          <t>Without CA, moving PCell to low band also loses high-band DL. Spectrum Coordination is not a substitute for 2CC.</t>
+        </is>
+      </c>
+      <c r="H76" s="10" t="n"/>
+      <c r="I76" s="10" t="n"/>
+      <c r="J76" s="11" t="n"/>
+    </row>
+    <row r="77" ht="52" customHeight="1">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>NSA DC UE, bit20 = 1</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>PCC not moved by Spectrum Coordination</t>
+        </is>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>LTE CA + NR SCG as NSA allows</t>
+        </is>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>NSA FPD: RsvdSwPara6_bit20 disables spectrum coordination for NSA DC UEs to prevent HO from PCC to a non-candidate PCC.</t>
+        </is>
+      </c>
+      <c r="H77" s="10" t="n"/>
+      <c r="I77" s="10" t="n"/>
+      <c r="J77" s="11" t="n"/>
+    </row>
+    <row r="78" ht="52" customHeight="1">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t>NSA DC PCC anchoring ON + WbbCaMultiCarrierCoordSw ON</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="D78" s="12" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>NSA PCC anchoring wins</t>
+        </is>
+      </c>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>NSA DC</t>
+        </is>
+      </c>
+      <c r="G78" s="12" t="inlineStr">
+        <is>
+          <t>NSA FPD: NSA DC PCC anchoring takes precedence over LTE spectrum coordination enhancement. Only NSA anchoring takes effect.</t>
+        </is>
+      </c>
+      <c r="H78" s="10" t="n"/>
+      <c r="I78" s="10" t="n"/>
+      <c r="J78" s="11" t="n"/>
+    </row>
+    <row r="79" ht="52" customHeight="1">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>DSS cell, few LTE UL RBs left</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>measured</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>Feature may not take effect for this UE</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>CA may still run on remaining LTE RBs</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>DSS FPD: fewer uplink RBs available for LTE reduces the proportion of UEs for which LTE Spectrum Coordination takes effect.</t>
+        </is>
+      </c>
+      <c r="H79" s="10" t="n"/>
+      <c r="I79" s="10" t="n"/>
+      <c r="J79" s="11" t="n"/>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="21" t="inlineStr">
+        <is>
+          <t>B4.  After the PCell change  —  CA state machine continues</t>
+        </is>
+      </c>
+      <c r="B80" s="22" t="n"/>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
+      <c r="E80" s="22" t="n"/>
+      <c r="F80" s="22" t="n"/>
+      <c r="G80" s="22" t="n"/>
+      <c r="H80" s="22" t="n"/>
+      <c r="I80" s="22" t="n"/>
+      <c r="J80" s="22" t="n"/>
+    </row>
+    <row r="81" ht="49" customHeight="1">
+      <c r="A81" s="18" t="inlineStr">
+        <is>
+          <t>Once the low-band cell is PCell, ordinary CA Ch.4.6 still applies: the high-band neighbor should already be a candidate SCell (group CaGroupSCellCfg or adaptive SccFreqCfg), A4/blind add can keep it configured, and MAC CE activation keeps DL on both CCs.  Event A5 Thresh1 remains −43 dBm / −3 dB for CA PCC anchoring; A6 Hys remains 1 dB. Those constants are CA FPD facts and are not Spectrum Coordination thresholds.  If the operations team also has Enhanced PCC anchoring ON, both DL-based anchoring and UL-quality PCell change can request a PCell change. The dedicated Spectrum Coordination FPD is the place that states the exact precedence; this repository does not. Known documented precedence: NSA DC PCC anchoring &gt; LTE spectrum coordination enhancement.</t>
+        </is>
+      </c>
+      <c r="B81" s="19" t="n"/>
+      <c r="C81" s="19" t="n"/>
+      <c r="D81" s="19" t="n"/>
+      <c r="E81" s="19" t="n"/>
+      <c r="F81" s="19" t="n"/>
+      <c r="G81" s="19" t="n"/>
+      <c r="H81" s="19" t="n"/>
+      <c r="I81" s="19" t="n"/>
+      <c r="J81" s="19" t="n"/>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>C.  Leaving / rollback</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
+      <c r="I82" s="6" t="n"/>
+      <c r="J82" s="6" t="n"/>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Leave path</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>How to do it / what to watch</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr"/>
+      <c r="F83" s="7" t="inlineStr"/>
+      <c r="G83" s="7" t="inlineStr"/>
+      <c r="H83" s="7" t="inlineStr"/>
+      <c r="I83" s="7" t="inlineStr"/>
+      <c r="J83" s="7" t="inlineStr"/>
+    </row>
+    <row r="84" ht="48" customHeight="1">
+      <c r="A84" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>UE moves back to cell center</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>High-band UL quality recovers → PCell can return to high band; low band stays as SCell for DL.</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Watch PCell HO counters (L.HHO.*.CAUser.PCC). Confirm no ping-pong (HO prep ≫ HO success). Dedicated hysteresis is in the Spectrum Coordination FPD.</t>
+        </is>
+      </c>
+      <c r="E84" s="10" t="n"/>
+      <c r="F84" s="10" t="n"/>
+      <c r="G84" s="10" t="n"/>
+      <c r="H84" s="10" t="n"/>
+      <c r="I84" s="10" t="n"/>
+      <c r="J84" s="11" t="n"/>
+    </row>
+    <row r="85" ht="48" customHeight="1">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>SCell (high band) radio quality collapses</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>Ordinary CA A2 / traffic / CQI deactivation / RRC remove. UE may keep low-band PCell as a single carrier.</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>Same leaving package as Step1 section C. Not Spectrum Coordination-specific.</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="n"/>
+      <c r="F85" s="10" t="n"/>
+      <c r="G85" s="10" t="n"/>
+      <c r="H85" s="10" t="n"/>
+      <c r="I85" s="10" t="n"/>
+      <c r="J85" s="11" t="n"/>
+    </row>
+    <row r="86" ht="48" customHeight="1">
+      <c r="A86" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>Operator turns the feature off</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>UL-quality PCell changes stop. Existing CA continues with DL-based PCC anchoring / A4–A6 only.</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG CellCaAlgoSwitch=SpectrumCoordinationSwitch-0 on every cell where it was enabled. Then re-check PCell distribution vs band.</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="n"/>
+      <c r="F86" s="10" t="n"/>
+      <c r="G86" s="10" t="n"/>
+      <c r="H86" s="10" t="n"/>
+      <c r="I86" s="10" t="n"/>
+      <c r="J86" s="11" t="n"/>
+    </row>
+    <row r="87" ht="48" customHeight="1">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>NSA DC UE, bit20 selected</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>Spectrum Coordination does not move that UE’s PCC.</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>MOD ENBCELLRSVDPARA RsvdSwPara6_bit20-1. Confirm exact bit MML in eNodeBFunction Used Reserved Parameter List.</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="n"/>
+      <c r="F87" s="10" t="n"/>
+      <c r="G87" s="10" t="n"/>
+      <c r="H87" s="10" t="n"/>
+      <c r="I87" s="10" t="n"/>
+      <c r="J87" s="11" t="n"/>
+    </row>
+    <row r="88" ht="48" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>DSS / UL multi-cluster shrinks LTE UL RBs</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>Feature takes effect for a smaller fraction of UEs — looks like “leaving” in KPI even though the switch is still On.</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>Check remaining LTE UL RB count and DSS sharing ratio before blaming Spectrum Coordination.</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="n"/>
+      <c r="F88" s="10" t="n"/>
+      <c r="G88" s="10" t="n"/>
+      <c r="H88" s="10" t="n"/>
+      <c r="I88" s="10" t="n"/>
+      <c r="J88" s="11" t="n"/>
+    </row>
+    <row r="89" ht="48" customHeight="1">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t>Load-balance inter-CC transfer vs enhancement</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>CA FPD: inter-CC load transfer does not take effect for WBB CA UEs or RRNs on which LTE spectrum coordination enhancement has taken effect.</t>
+        </is>
+      </c>
+      <c r="D89" s="12" t="inlineStr">
+        <is>
+          <t>If you need DlCaLbAlgoSwitch / CaLoadBalancePreAllocSwitch on those WBB/RRN UEs, do not expect both to win.</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="n"/>
+      <c r="F89" s="10" t="n"/>
+      <c r="G89" s="10" t="n"/>
+      <c r="H89" s="10" t="n"/>
+      <c r="I89" s="10" t="n"/>
+      <c r="J89" s="11" t="n"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>D.  Prerequisite / exclusive / impacted features  (one feature per row; related parameters grouped)</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
+      <c r="I90" s="6" t="n"/>
+      <c r="J90" s="6" t="n"/>
+    </row>
+    <row r="91" ht="28" customHeight="1">
+      <c r="A91" s="16" t="inlineStr">
+        <is>
+          <t>CA FPD function-impact tables (Ch.5 / Ch.13 CloudAIR rows) plus DSS FPD and NSA FPD. Related parameters of the same feature are grouped in the Parameter column.</t>
+        </is>
+      </c>
+      <c r="B91" s="17" t="n"/>
+      <c r="C91" s="17" t="n"/>
+      <c r="D91" s="17" t="n"/>
+      <c r="E91" s="17" t="n"/>
+      <c r="F91" s="17" t="n"/>
+      <c r="G91" s="17" t="n"/>
+      <c r="H91" s="17" t="n"/>
+      <c r="I91" s="17" t="n"/>
+      <c r="J91" s="17" t="n"/>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Relation</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>RAT</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Related parameter(s)</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>Impact / rule</t>
+        </is>
+      </c>
+      <c r="G92" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H92" s="7" t="inlineStr"/>
+      <c r="I92" s="7" t="inlineStr"/>
+      <c r="J92" s="7" t="inlineStr"/>
+    </row>
+    <row r="93" ht="62" customHeight="1">
+      <c r="A93" s="29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B93" s="38" t="inlineStr">
+        <is>
+          <t>Prerequisite</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D93" s="38" t="inlineStr">
+        <is>
+          <t>Downlink 2CC CA (this workbook Step1)</t>
+        </is>
+      </c>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch (2CC bits); ENodeBAlgoSwitch.CaAlgoSwitch FreqCfgSwitch/AdpCaSwitch; CaGroup or PccFreqCfg+SccFreqCfg</t>
+        </is>
+      </c>
+      <c r="F93" s="29" t="inlineStr">
+        <is>
+          <t>DL must already be aggregatable on the high+low pair. Spectrum Coordination does not create CA.</t>
+        </is>
+      </c>
+      <c r="G93" s="29" t="inlineStr">
+        <is>
+          <t>3CC/4CC/5CC optional; they increase DL after the UL PCell is correct.</t>
+        </is>
+      </c>
+      <c r="H93" s="10" t="n"/>
+      <c r="I93" s="10" t="n"/>
+      <c r="J93" s="11" t="n"/>
+    </row>
+    <row r="94" ht="62" customHeight="1">
+      <c r="A94" s="29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B94" s="38" t="inlineStr">
+        <is>
+          <t>Prerequisite</t>
+        </is>
+      </c>
+      <c r="C94" s="29" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D94" s="38" t="inlineStr">
+        <is>
+          <t>Overlapping high/low coverage + CA neighbor</t>
+        </is>
+      </c>
+      <c r="E94" s="29" t="inlineStr">
+        <is>
+          <t>EutranInterNFreq.AggregationAttribute FREQ_MEAS_FLAG; EutranCellMeasurement.NoRmvFlag=FORBID_RMV_ENUM</t>
+        </is>
+      </c>
+      <c r="F94" s="29" t="inlineStr">
+        <is>
+          <t>Without overlap, a PCell change to the other band drops the UE out of coverage of the original DL CC.</t>
+        </is>
+      </c>
+      <c r="G94" s="29" t="inlineStr">
+        <is>
+          <t>Same coverage rule as CA Ch.5.3.5.</t>
+        </is>
+      </c>
+      <c r="H94" s="10" t="n"/>
+      <c r="I94" s="10" t="n"/>
+      <c r="J94" s="11" t="n"/>
+    </row>
+    <row r="95" ht="62" customHeight="1">
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B95" s="35" t="inlineStr">
+        <is>
+          <t>This function</t>
+        </is>
+      </c>
+      <c r="C95" s="31" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D95" s="35" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination</t>
+        </is>
+      </c>
+      <c r="E95" s="31" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch → SpectrumCoordinationSwitch</t>
+        </is>
+      </c>
+      <c r="F95" s="31" t="inlineStr">
+        <is>
+          <t>Master enable. Default Off. PCell changes based on uplink quality when selected.</t>
+        </is>
+      </c>
+      <c r="G95" s="31" t="inlineStr">
+        <is>
+          <t>CellCaAlgoSwitch description in related eRAN FPDs. Dedicated FPD = CA ref 55.</t>
+        </is>
+      </c>
+      <c r="H95" s="10" t="n"/>
+      <c r="I95" s="10" t="n"/>
+      <c r="J95" s="11" t="n"/>
+    </row>
+    <row r="96" ht="62" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B96" s="37" t="inlineStr">
+        <is>
+          <t>Enhancement</t>
+        </is>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>TDD (documented in CA FPD CloudAIR rows); listed generally on CellCaAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="D96" s="37" t="inlineStr">
+        <is>
+          <t>LTE spectrum coordination enhancement</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch → WbbCaMultiCarrierCoordSw</t>
+        </is>
+      </c>
+      <c r="F96" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD Ch.5 / Ch.13: inter-CC load transfer triggered by cell load (DlCaLbAlgoSwitch) or by cell-load differences (CaLoadBalancePreAllocSwitch) does NOT take effect for WBB CA UEs or RRNs on which this enhancement has taken effect.</t>
+        </is>
+      </c>
+      <c r="G96" s="9" t="inlineStr">
+        <is>
+          <t>NSA FPD: NSA DC PCC anchoring takes precedence over this enhancement.</t>
+        </is>
+      </c>
+      <c r="H96" s="10" t="n"/>
+      <c r="I96" s="10" t="n"/>
+      <c r="J96" s="11" t="n"/>
+    </row>
+    <row r="97" ht="62" customHeight="1">
+      <c r="A97" s="39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B97" s="40" t="inlineStr">
+        <is>
+          <t>Impacted by</t>
+        </is>
+      </c>
+      <c r="C97" s="39" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="D97" s="40" t="inlineStr">
+        <is>
+          <t>LTE FDD and NR Flash / Hybrid / SUL Dynamic Spectrum Sharing</t>
+        </is>
+      </c>
+      <c r="E97" s="39" t="inlineStr">
+        <is>
+          <t>SpectrumCloud.SpectrumCloudSwitch = LTE_NR_SPECTRUM_SHR or LTE_NR_UPLINK_SPECTRUM_SHR; CaMgtCfg.CellCaAlgoSwitch → SpectrumCoordinationSwitch</t>
+        </is>
+      </c>
+      <c r="F97" s="39" t="inlineStr">
+        <is>
+          <t>DSS FPD: the number of uplink RBs available for LTE decreases, which reduces the proportion of UEs for which LTE Spectrum Coordination takes effect.</t>
+        </is>
+      </c>
+      <c r="G97" s="39" t="inlineStr">
+        <is>
+          <t>CA FPD also: DSS cells not recommended as PCell (PUCCH so large SRS cannot be configured).</t>
+        </is>
+      </c>
+      <c r="H97" s="10" t="n"/>
+      <c r="I97" s="10" t="n"/>
+      <c r="J97" s="11" t="n"/>
+    </row>
+    <row r="98" ht="62" customHeight="1">
+      <c r="A98" s="39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B98" s="40" t="inlineStr">
+        <is>
+          <t>Impacted by</t>
+        </is>
+      </c>
+      <c r="C98" s="39" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D98" s="40" t="inlineStr">
+        <is>
+          <t>UL Multi-Cluster Scheduling</t>
+        </is>
+      </c>
+      <c r="E98" s="39" t="inlineStr">
+        <is>
+          <t>CellAlgoSwitch.UlSchExtSwitch → UlMultiClusterSwitch</t>
+        </is>
+      </c>
+      <c r="F98" s="39" t="inlineStr">
+        <is>
+          <t>DSS FPD lists this next to Spectrum Coordination: fewer LTE UL RBs → fewer UEs get Spectrum Coordination, and UL frequency-selective / multi-cluster gain also drops.</t>
+        </is>
+      </c>
+      <c r="G98" s="39" t="inlineStr">
+        <is>
+          <t>Review this bit on DSS-sharing cells.</t>
+        </is>
+      </c>
+      <c r="H98" s="10" t="n"/>
+      <c r="I98" s="10" t="n"/>
+      <c r="J98" s="11" t="n"/>
+    </row>
+    <row r="99" ht="62" customHeight="1">
+      <c r="A99" s="39" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B99" s="40" t="inlineStr">
+        <is>
+          <t>Impacted by / exception</t>
+        </is>
+      </c>
+      <c r="C99" s="39" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D99" s="40" t="inlineStr">
+        <is>
+          <t>EPC-based NSA DC</t>
+        </is>
+      </c>
+      <c r="E99" s="39" t="inlineStr">
+        <is>
+          <t>ENBCELLRSVDPARA.RsvdSwPara6 → RsvdSwPara6_bit20; CaMgtCfg.CellCaAlgoSwitch → WbbCaMultiCarrierCoordSw; NSA PCC-anchoring switches (see NSA FPD)</t>
+        </is>
+      </c>
+      <c r="F99" s="39" t="inlineStr">
+        <is>
+          <t>After Spectrum Coordination is enabled, select bit20 to disable it for NSA DC UEs (prevents HO from PCC to non-candidate PCC). NSA PCC anchoring &gt; coordination enhancement.</t>
+        </is>
+      </c>
+      <c r="G99" s="39" t="inlineStr">
+        <is>
+          <t>Reserved-parameter details: eNodeBFunction Used Reserved Parameter List.</t>
+        </is>
+      </c>
+      <c r="H99" s="10" t="n"/>
+      <c r="I99" s="10" t="n"/>
+      <c r="J99" s="11" t="n"/>
+    </row>
+    <row r="100" ht="62" customHeight="1">
+      <c r="A100" s="39" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B100" s="40" t="inlineStr">
+        <is>
+          <t>Impact (does not take effect together)</t>
+        </is>
+      </c>
+      <c r="C100" s="39" t="inlineStr">
+        <is>
+          <t>TDD WBB/RRN</t>
+        </is>
+      </c>
+      <c r="D100" s="40" t="inlineStr">
+        <is>
+          <t>Inter-CC load transfer</t>
+        </is>
+      </c>
+      <c r="E100" s="39" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch.CaLbAlgoSwitch → DlCaLbAlgoSwitch; ENodeBAlgoSwitch.CaAlgoSwitch → CaLoadBalancePreAllocSwitch; WbbCaMultiCarrierCoordSw</t>
+        </is>
+      </c>
+      <c r="F100" s="39" t="inlineStr">
+        <is>
+          <t>Load-triggered inter-CC transfer does not take effect on WBB CA UEs / RRNs where spectrum coordination enhancement has taken effect.</t>
+        </is>
+      </c>
+      <c r="G100" s="39" t="inlineStr">
+        <is>
+          <t>CA FPD CloudAIR impact rows, DL 2CC and FDD+TDD CA chapters.</t>
+        </is>
+      </c>
+      <c r="H100" s="10" t="n"/>
+      <c r="I100" s="10" t="n"/>
+      <c r="J100" s="11" t="n"/>
+    </row>
+    <row r="101" ht="62" customHeight="1">
+      <c r="A101" s="12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B101" s="33" t="inlineStr">
+        <is>
+          <t>Related CloudAIR (different feature)</t>
+        </is>
+      </c>
+      <c r="C101" s="12" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="D101" s="33" t="inlineStr">
+        <is>
+          <t>GSM and LTE Spectrum Concurrency</t>
+        </is>
+      </c>
+      <c r="E101" s="12" t="inlineStr">
+        <is>
+          <t>SpectrumCloud.SpectrumCloudSwitch = GL_SPECTRUM_CONCURRENCY</t>
+        </is>
+      </c>
+      <c r="F101" s="12" t="inlineStr">
+        <is>
+          <t>CA FPD: such LTE cells are not recommended as PCells (PUCCH vs SRS). Relaxed-backhaul: if they are SCells, pre-scheduling RB estimate can be stale.</t>
+        </is>
+      </c>
+      <c r="G101" s="12" t="inlineStr">
+        <is>
+          <t>Do not confuse with SpectrumCoordinationSwitch.</t>
+        </is>
+      </c>
+      <c r="H101" s="10" t="n"/>
+      <c r="I101" s="10" t="n"/>
+      <c r="J101" s="11" t="n"/>
+    </row>
+    <row r="102" ht="62" customHeight="1">
+      <c r="A102" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B102" s="37" t="inlineStr">
+        <is>
+          <t>Related CloudAIR (different feature)</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="D102" s="37" t="inlineStr">
+        <is>
+          <t>UMTS and LTE Spectrum Sharing (and DC-HSDPA variant)</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>SpectrumCloud.SpectrumCloudSwitch = UL_SPECTRUM_SHARING or DC_HSDPA_BASED_UL_SPECTRUM_SHR</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD: 5 MHz cells not recommended as PCell. Massive CA not recommended on sharing cells.</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>Spectrum cloudification, not channel cloudification.</t>
+        </is>
+      </c>
+      <c r="H102" s="10" t="n"/>
+      <c r="I102" s="10" t="n"/>
+      <c r="J102" s="11" t="n"/>
+    </row>
+    <row r="103" ht="62" customHeight="1">
+      <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B103" s="33" t="inlineStr">
+        <is>
+          <t>Related CA (still required)</t>
+        </is>
+      </c>
+      <c r="C103" s="12" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D103" s="33" t="inlineStr">
+        <is>
+          <t>Enhanced PCC anchoring / A5 HO events</t>
+        </is>
+      </c>
+      <c r="E103" s="12" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch.CaAlgoSwitch → EnhancedPccAnchorSwitch; CaAlgoExtSwitch → CaA5HoEventSwitch + CaA5HoEventEnhSwitch</t>
+        </is>
+      </c>
+      <c r="F103" s="12" t="inlineStr">
+        <is>
+          <t>DL-based PCell steering remains. Spectrum Coordination adds UL-quality PCell change on top. Keep A5 HO switches so a UE can HO from PCell to its SCell (CA Ch.4.3 recommendation).</t>
+        </is>
+      </c>
+      <c r="G103" s="12" t="inlineStr">
+        <is>
+          <t>Do not turn CA PCC anchoring off unless the dedicated FPD says so — it is not stated here.</t>
+        </is>
+      </c>
+      <c r="H103" s="10" t="n"/>
+      <c r="I103" s="10" t="n"/>
+      <c r="J103" s="11" t="n"/>
+    </row>
+    <row r="104" ht="62" customHeight="1">
+      <c r="A104" s="9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B104" s="37" t="inlineStr">
+        <is>
+          <t>Hardware / product</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="D104" s="37" t="inlineStr">
+        <is>
+          <t>3900 / 5900 series eNodeB (same family as CA)</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD hardware chapters apply to the CA vehicle. Dedicated Spectrum Coordination hardware notes are in its own FPD (not in repo).</t>
+        </is>
+      </c>
+      <c r="G104" s="9" t="inlineStr">
+        <is>
+          <t>Contact Huawei service for board combination if activating on LampSite / RRU-only sites.</t>
+        </is>
+      </c>
+      <c r="H104" s="10" t="n"/>
+      <c r="I104" s="10" t="n"/>
+      <c r="J104" s="11" t="n"/>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>E.  Parameters  (SN, MO, name, default, recommended, description, notes)</t>
+        </is>
+      </c>
+      <c r="B105" s="6" t="n"/>
+      <c r="C105" s="6" t="n"/>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="6" t="n"/>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+    </row>
+    <row r="106" ht="28" customHeight="1">
+      <c r="A106" s="16" t="inlineStr">
+        <is>
+          <t>Only parameters that appear in the sources listed in section L. Factory defaults that the source actually prints are used; otherwise “See Parameter Reference”. Recommended values are operational, not Huawei-confidential tuning.</t>
+        </is>
+      </c>
+      <c r="B106" s="17" t="n"/>
+      <c r="C106" s="17" t="n"/>
+      <c r="D106" s="17" t="n"/>
+      <c r="E106" s="17" t="n"/>
+      <c r="F106" s="17" t="n"/>
+      <c r="G106" s="17" t="n"/>
+      <c r="H106" s="17" t="n"/>
+      <c r="I106" s="17" t="n"/>
+      <c r="J106" s="17" t="n"/>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>MO Name</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>Parameter name</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>Default value</t>
+        </is>
+      </c>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Recommended value</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>Parameter description</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr"/>
+      <c r="I107" s="7" t="inlineStr"/>
+      <c r="J107" s="7" t="inlineStr"/>
+    </row>
+    <row r="108" ht="52" customHeight="1">
+      <c r="A108" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B108" s="33" t="inlineStr">
+        <is>
+          <t>CaMgtCfg</t>
+        </is>
+      </c>
+      <c r="C108" s="33" t="inlineStr">
+        <is>
+          <t>CellCaAlgoSwitch / SpectrumCoordinationSwitch</t>
+        </is>
+      </c>
+      <c r="D108" s="12" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E108" s="33" t="inlineStr">
+        <is>
+          <t>1 on every high-band and low-band cell that should participate, after Step1 CA is verified</t>
+        </is>
+      </c>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>Spectrum coordination is enabled only if this option is selected. With spectrum coordination enabled, PCell changes are triggered based on uplink quality. Applies to LTE FDD and LTE TDD.</t>
+        </is>
+      </c>
+      <c r="G108" s="12" t="inlineStr">
+        <is>
+          <t>Master switch. Same MO as CaDl3CCSwitch / CaUl2CCSwitch / … Default Off is printed in related FPD CellCaAlgoSwitch listing.</t>
+        </is>
+      </c>
+      <c r="H108" s="10" t="n"/>
+      <c r="I108" s="10" t="n"/>
+      <c r="J108" s="11" t="n"/>
+    </row>
+    <row r="109" ht="40" customHeight="1">
+      <c r="A109" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="B109" s="35" t="inlineStr">
+        <is>
+          <t>CaMgtCfg</t>
+        </is>
+      </c>
+      <c r="C109" s="35" t="inlineStr">
+        <is>
+          <t>CellCaAlgoSwitch / WbbCaMultiCarrierCoordSw</t>
+        </is>
+      </c>
+      <c r="D109" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E109" s="35" t="inlineStr">
+        <is>
+          <t>1 only if WBB/RRN coordination enhancement is required AND NSA PCC anchoring is not supposed to win</t>
+        </is>
+      </c>
+      <c r="F109" s="31" t="inlineStr">
+        <is>
+          <t>LTE spectrum coordination enhancement. Referenced from CA FPD CloudAIR impact rows and from NSA FPD (“coordination enhancement”).</t>
+        </is>
+      </c>
+      <c r="G109" s="31" t="inlineStr">
+        <is>
+          <t>Related: DlCaLbAlgoSwitch, CaLoadBalancePreAllocSwitch (load transfer does not take effect on WBB CA UEs/RRNs once enhancement has taken effect). Related: NSA PCC anchoring takes precedence.</t>
+        </is>
+      </c>
+      <c r="H109" s="10" t="n"/>
+      <c r="I109" s="10" t="n"/>
+      <c r="J109" s="11" t="n"/>
+    </row>
+    <row r="110" ht="52" customHeight="1">
+      <c r="A110" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B110" s="35" t="inlineStr">
+        <is>
+          <t>ENBCELLRSVDPARA</t>
+        </is>
+      </c>
+      <c r="C110" s="35" t="inlineStr">
+        <is>
+          <t>RsvdSwPara6 / RsvdSwPara6_bit20</t>
+        </is>
+      </c>
+      <c r="D110" s="31" t="inlineStr">
+        <is>
+          <t>See reserved-parameter list (typically 0 = not selected)</t>
+        </is>
+      </c>
+      <c r="E110" s="35" t="inlineStr">
+        <is>
+          <t>1 on NSA sites if NSA DC UEs must NOT be moved by Spectrum Coordination</t>
+        </is>
+      </c>
+      <c r="F110" s="31" t="inlineStr">
+        <is>
+          <t>After LTE spectrum coordination is enabled, this bit can be selected to disable spectrum coordination for NSA DC UEs, i.e. to prevent NSA DC UEs from being handed over from PCCs to non-candidate PCCs.</t>
+        </is>
+      </c>
+      <c r="G110" s="31" t="inlineStr">
+        <is>
+          <t>Source: EPC-based NSA FPD. Confirm meaning, version, and MML in 3900 &amp; 5900 eNodeBFunction Used Reserved Parameter List. Related: SpectrumCoordinationSwitch must already be On.</t>
+        </is>
+      </c>
+      <c r="H110" s="10" t="n"/>
+      <c r="I110" s="10" t="n"/>
+      <c r="J110" s="11" t="n"/>
+    </row>
+    <row r="111" ht="52" customHeight="1">
+      <c r="A111" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="B111" s="35" t="inlineStr">
+        <is>
+          <t>CellAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="C111" s="35" t="inlineStr">
+        <is>
+          <t>UlSchExtSwitch / UlMultiClusterSwitch</t>
+        </is>
+      </c>
+      <c r="D111" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E111" s="35" t="inlineStr">
+        <is>
+          <t>Review on DSS / tight-UL cells; do not assume Off</t>
+        </is>
+      </c>
+      <c r="F111" s="31" t="inlineStr">
+        <is>
+          <t>UL multi-cluster scheduling. DSS FPD: fewer LTE UL RBs reduces the proportion of UEs for which Spectrum Coordination takes effect, and reduces UL multi-cluster / frequency-selective gain.</t>
+        </is>
+      </c>
+      <c r="G111" s="31" t="inlineStr">
+        <is>
+          <t>Related to SpectrumCoordinationSwitch only through the shared UL RB pool — not an alias of it.</t>
+        </is>
+      </c>
+      <c r="H111" s="10" t="n"/>
+      <c r="I111" s="10" t="n"/>
+      <c r="J111" s="11" t="n"/>
+    </row>
+    <row r="112" ht="64" customHeight="1">
+      <c r="A112" s="34" t="n">
+        <v>5</v>
+      </c>
+      <c r="B112" s="35" t="inlineStr">
+        <is>
+          <t>SpectrumCloud</t>
+        </is>
+      </c>
+      <c r="C112" s="35" t="inlineStr">
+        <is>
+          <t>SpectrumCloudSwitch</t>
+        </is>
+      </c>
+      <c r="D112" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference (DSS Off unless DSS is the job)</t>
+        </is>
+      </c>
+      <c r="E112" s="35" t="inlineStr">
+        <is>
+          <t>Keep DSS and Spectrum Coordination planning coupled if both are on the same LTE cell</t>
+        </is>
+      </c>
+      <c r="F112" s="31" t="inlineStr">
+        <is>
+          <t>LTE_NR_SPECTRUM_SHR / LTE_NR_UPLINK_SPECTRUM_SHR / GL_SPECTRUM_CONCURRENCY / UL_SPECTRUM_SHARING are different CloudAIR functions. Flash DSS reduces LTE UL RBs (Spectrum Coordination UE proportion ↓). GL concurrency / UMTS sharing: CA FPD says do not use those cells as PCell if PUCCH kills SRS.</t>
+        </is>
+      </c>
+      <c r="G112" s="31" t="inlineStr">
+        <is>
+          <t>Do not set SpectrumCloudSwitch to enable LTE Spectrum Coordination — that is CellCaAlgoSwitch.</t>
+        </is>
+      </c>
+      <c r="H112" s="10" t="n"/>
+      <c r="I112" s="10" t="n"/>
+      <c r="J112" s="11" t="n"/>
+    </row>
+    <row r="113" ht="40" customHeight="1">
+      <c r="A113" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="B113" s="35" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="C113" s="35" t="inlineStr">
+        <is>
+          <t>CaLbAlgoSwitch / DlCaLbAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="D113" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E113" s="35" t="inlineStr">
+        <is>
+          <t>Know the conflict on WBB/RRN if WbbCaMultiCarrierCoordSw is On</t>
+        </is>
+      </c>
+      <c r="F113" s="31" t="inlineStr">
+        <is>
+          <t>Inter-CC load transfer triggered by cell load. CA FPD: does not take effect for WBB CA UEs or RRNs on which LTE spectrum coordination enhancement has taken effect.</t>
+        </is>
+      </c>
+      <c r="G113" s="31" t="inlineStr">
+        <is>
+          <t>Related: WbbCaMultiCarrierCoordSw.</t>
+        </is>
+      </c>
+      <c r="H113" s="10" t="n"/>
+      <c r="I113" s="10" t="n"/>
+      <c r="J113" s="11" t="n"/>
+    </row>
+    <row r="114" ht="40" customHeight="1">
+      <c r="A114" s="34" t="n">
+        <v>7</v>
+      </c>
+      <c r="B114" s="35" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="C114" s="35" t="inlineStr">
+        <is>
+          <t>CaAlgoSwitch / CaLoadBalancePreAllocSwitch</t>
+        </is>
+      </c>
+      <c r="D114" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E114" s="35" t="inlineStr">
+        <is>
+          <t>Same awareness as DlCaLbAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="F114" s="31" t="inlineStr">
+        <is>
+          <t>Inter-CC load transfer triggered by cell-load differences. Same CA FPD exclusion versus spectrum coordination enhancement on WBB CA UEs / RRNs.</t>
+        </is>
+      </c>
+      <c r="G114" s="31" t="inlineStr">
+        <is>
+          <t>Related: WbbCaMultiCarrierCoordSw, DlCaLbAlgoSwitch.</t>
+        </is>
+      </c>
+      <c r="H114" s="10" t="n"/>
+      <c r="I114" s="10" t="n"/>
+      <c r="J114" s="11" t="n"/>
+    </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B115" s="35" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="C115" s="35" t="inlineStr">
+        <is>
+          <t>CaAlgoSwitch / EnhancedPccAnchorSwitch</t>
+        </is>
+      </c>
+      <c r="D115" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference (CA Step1 recommends select)</t>
+        </is>
+      </c>
+      <c r="E115" s="35" t="inlineStr">
+        <is>
+          <t>Keep as in Step1 unless dedicated FPD says otherwise</t>
+        </is>
+      </c>
+      <c r="F115" s="31" t="inlineStr">
+        <is>
+          <t>DL-measurement PCC anchoring (A1/A5). Still the CA way of choosing a better PCell. Spectrum Coordination adds a UL-quality reason to change PCell.</t>
+        </is>
+      </c>
+      <c r="G115" s="31" t="inlineStr">
+        <is>
+          <t>Related CA: PccAnchorSwitch (ignored if Enhanced is On), PccFreqCfg.PccA4RsrpThd, CaGroup PreferredPCellPriority.</t>
+        </is>
+      </c>
+      <c r="H115" s="10" t="n"/>
+      <c r="I115" s="10" t="n"/>
+      <c r="J115" s="11" t="n"/>
+    </row>
+    <row r="116" ht="52" customHeight="1">
+      <c r="A116" s="34" t="n">
+        <v>9</v>
+      </c>
+      <c r="B116" s="35" t="inlineStr">
+        <is>
+          <t>ENodeBAlgoSwitch</t>
+        </is>
+      </c>
+      <c r="C116" s="35" t="inlineStr">
+        <is>
+          <t>CaAlgoExtSwitch / CaA5HoEventSwitch + CaA5HoEventEnhSwitch</t>
+        </is>
+      </c>
+      <c r="D116" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E116" s="35" t="inlineStr">
+        <is>
+          <t>Select BOTH (CA FPD Ch.4.3 recommendation)</t>
+        </is>
+      </c>
+      <c r="F116" s="31" t="inlineStr">
+        <is>
+          <t>Changes HO event A4 to A5 when SCells exist so the UE can be handed over from its PCell to its SCell. Spectrum Coordination’s PCell change between high and low bands needs this HO path to be legal.</t>
+        </is>
+      </c>
+      <c r="G116" s="31" t="inlineStr">
+        <is>
+          <t>Related: InterFreqHoGroup A5 thresholds. A5 Thresh1 is always −43 dBm / −3 dB (CA FPD).</t>
+        </is>
+      </c>
+      <c r="H116" s="10" t="n"/>
+      <c r="I116" s="10" t="n"/>
+      <c r="J116" s="11" t="n"/>
+    </row>
+    <row r="117" ht="40" customHeight="1">
+      <c r="A117" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="B117" s="35" t="inlineStr">
+        <is>
+          <t>CaMgtCfg</t>
+        </is>
+      </c>
+      <c r="C117" s="35" t="inlineStr">
+        <is>
+          <t>CellCaAlgoSwitch / CaUl2CCSwitch</t>
+        </is>
+      </c>
+      <c r="D117" s="31" t="inlineStr">
+        <is>
+          <t>Off</t>
+        </is>
+      </c>
+      <c r="E117" s="35" t="inlineStr">
+        <is>
+          <t>Independent — enable only if UL 2CC is planned</t>
+        </is>
+      </c>
+      <c r="F117" s="31" t="inlineStr">
+        <is>
+          <t>Uplink 2CC aggregation (CA FPD Ch.10). Spectrum Coordination is an alternative/complement for UL coverage, not a substitute for UL 2CC peak rate.</t>
+        </is>
+      </c>
+      <c r="G117" s="31" t="inlineStr">
+        <is>
+          <t>If both are on, the dedicated FPDs must be read together. Not described further here.</t>
+        </is>
+      </c>
+      <c r="H117" s="10" t="n"/>
+      <c r="I117" s="10" t="n"/>
+      <c r="J117" s="11" t="n"/>
+    </row>
+    <row r="118" ht="40" customHeight="1">
+      <c r="A118" s="34" t="n">
+        <v>11</v>
+      </c>
+      <c r="B118" s="35" t="inlineStr">
+        <is>
+          <t>EutranInterNFreq</t>
+        </is>
+      </c>
+      <c r="C118" s="35" t="inlineStr">
+        <is>
+          <t>AggregationAttribute / FREQ_MEAS_FLAG</t>
+        </is>
+      </c>
+      <c r="D118" s="31" t="inlineStr">
+        <is>
+          <t>Site-planned</t>
+        </is>
+      </c>
+      <c r="E118" s="35" t="inlineStr">
+        <is>
+          <t>Selected on the partner-band frequency</t>
+        </is>
+      </c>
+      <c r="F118" s="31" t="inlineStr">
+        <is>
+          <t>Frequency is a CA candidate. If deselected, the other band cannot be SCell after a PCell change.</t>
+        </is>
+      </c>
+      <c r="G118" s="31" t="inlineStr">
+        <is>
+          <t>CA Step1 prerequisite, still required here.</t>
+        </is>
+      </c>
+      <c r="H118" s="10" t="n"/>
+      <c r="I118" s="10" t="n"/>
+      <c r="J118" s="11" t="n"/>
+    </row>
+    <row r="119" ht="28" customHeight="1">
+      <c r="A119" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="B119" s="35" t="inlineStr">
+        <is>
+          <t>EutranCellMeasurement</t>
+        </is>
+      </c>
+      <c r="C119" s="35" t="inlineStr">
+        <is>
+          <t>NoRmvFlag</t>
+        </is>
+      </c>
+      <c r="D119" s="31" t="inlineStr">
+        <is>
+          <t>See Parameter Reference</t>
+        </is>
+      </c>
+      <c r="E119" s="35" t="inlineStr">
+        <is>
+          <t>FORBID_RMV_ENUM on CA neighbors of the pair</t>
+        </is>
+      </c>
+      <c r="F119" s="31" t="inlineStr">
+        <is>
+          <t>Stops ANR from deleting the high/low neighbor used for CA and for PCell swap.</t>
+        </is>
+      </c>
+      <c r="G119" s="31" t="inlineStr">
+        <is>
+          <t>CA FPD neighbor rule.</t>
+        </is>
+      </c>
+      <c r="H119" s="10" t="n"/>
+      <c r="I119" s="10" t="n"/>
+      <c r="J119" s="11" t="n"/>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="21" t="inlineStr">
+        <is>
+          <t>E2.  Parameters that exist only in the dedicated FPD  —  not printed here</t>
+        </is>
+      </c>
+      <c r="B120" s="22" t="n"/>
+      <c r="C120" s="22" t="n"/>
+      <c r="D120" s="22" t="n"/>
+      <c r="E120" s="22" t="n"/>
+      <c r="F120" s="22" t="n"/>
+      <c r="G120" s="22" t="n"/>
+      <c r="H120" s="22" t="n"/>
+      <c r="I120" s="22" t="n"/>
+      <c r="J120" s="22" t="n"/>
+    </row>
+    <row r="121" ht="72" customHeight="1">
+      <c r="A121" s="41" t="inlineStr">
+        <is>
+          <t>•  UL-quality metric, entering/leaving thresholds, hysteresis, time-to-trigger, and any blacklist (VoLTE / high-speed / QCI) for Spectrum Coordination PCell change.
+•  Whether the feature requires group-based CA, adaptive CA, or both.
+•  Dedicated performance counters and license models (Feature ID / Model / sales unit).
+•  Action: open eRAN Feature Documentation → LTE Spectrum Coordination, then filter eNodeBFunction Parameter Reference by that feature ID (CA FPD Ch.20 FAQ).</t>
+        </is>
+      </c>
+      <c r="B121" s="42" t="n"/>
+      <c r="C121" s="42" t="n"/>
+      <c r="D121" s="42" t="n"/>
+      <c r="E121" s="42" t="n"/>
+      <c r="F121" s="42" t="n"/>
+      <c r="G121" s="42" t="n"/>
+      <c r="H121" s="42" t="n"/>
+      <c r="I121" s="42" t="n"/>
+      <c r="J121" s="42" t="n"/>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>F.  MML  (reconstructed from documented switches; not a dedicated-FPD sample)</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="n"/>
+      <c r="C122" s="6" t="n"/>
+      <c r="D122" s="6" t="n"/>
+      <c r="E122" s="6" t="n"/>
+      <c r="F122" s="6" t="n"/>
+      <c r="G122" s="6" t="n"/>
+      <c r="H122" s="6" t="n"/>
+      <c r="I122" s="6" t="n"/>
+      <c r="J122" s="6" t="n"/>
+    </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="16" t="inlineStr">
+        <is>
+          <t>Bit-switch syntax matches CA FPD samples (CellCaAlgoSwitch=Name-1). Replace LocalCellId and confirm reserved-parameter MML on the live version. Doc example eNodeBId=1234 is not required here.</t>
+        </is>
+      </c>
+      <c r="B123" s="17" t="n"/>
+      <c r="C123" s="17" t="n"/>
+      <c r="D123" s="17" t="n"/>
+      <c r="E123" s="17" t="n"/>
+      <c r="F123" s="17" t="n"/>
+      <c r="G123" s="17" t="n"/>
+      <c r="H123" s="17" t="n"/>
+      <c r="I123" s="17" t="n"/>
+      <c r="J123" s="17" t="n"/>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t>Seq</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t>Mode</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr">
+        <is>
+          <t>RAT</t>
+        </is>
+      </c>
+      <c r="E124" s="7" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="F124" s="7" t="inlineStr">
+        <is>
+          <t>MML command (verbatim from document)</t>
+        </is>
+      </c>
+      <c r="G124" s="7" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="H124" s="7" t="inlineStr"/>
+      <c r="I124" s="7" t="inlineStr"/>
+      <c r="J124" s="7" t="inlineStr"/>
+    </row>
+    <row r="125" ht="24" customHeight="1">
+      <c r="A125" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B125" s="32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C125" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E125" s="12" t="inlineStr">
+        <is>
+          <t>Pre-check</t>
+        </is>
+      </c>
+      <c r="F125" s="33" t="inlineStr">
+        <is>
+          <t>DSP CELLCA; DSP CAMGTCFG: LocalCellId=0; LST CAMGTCFG: LocalCellId=0;</t>
+        </is>
+      </c>
+      <c r="G125" s="12" t="inlineStr">
+        <is>
+          <t>Confirm Step1 CA is already producing SCell add/act counters before enabling Spectrum Coordination.</t>
+        </is>
+      </c>
+      <c r="H125" s="10" t="n"/>
+      <c r="I125" s="10" t="n"/>
+      <c r="J125" s="11" t="n"/>
+    </row>
+    <row r="126" ht="24" customHeight="1">
+      <c r="A126" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B126" s="36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>Enable SC</t>
+        </is>
+      </c>
+      <c r="F126" s="37" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>Reconstructed MML. Run on each participating high-band and low-band cell (repeat LocalCellId). Default was Off.</t>
+        </is>
+      </c>
+      <c r="H126" s="10" t="n"/>
+      <c r="I126" s="10" t="n"/>
+      <c r="J126" s="11" t="n"/>
+    </row>
+    <row r="127" ht="24" customHeight="1">
+      <c r="A127" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B127" s="32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C127" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E127" s="12" t="inlineStr">
+        <is>
+          <t>Enable SC</t>
+        </is>
+      </c>
+      <c r="F127" s="33" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
+        </is>
+      </c>
+      <c r="G127" s="12" t="inlineStr">
+        <is>
+          <t>Partner-band cell. Use live LocalCellId (doc 2CC TDD examples used 0 and 1).</t>
+        </is>
+      </c>
+      <c r="H127" s="10" t="n"/>
+      <c r="I127" s="10" t="n"/>
+      <c r="J127" s="11" t="n"/>
+    </row>
+    <row r="128" ht="24" customHeight="1">
+      <c r="A128" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="B128" s="36" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>TDD WBB/RRN</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr">
+        <is>
+          <t>Optional enhancement</t>
+        </is>
+      </c>
+      <c r="F128" s="37" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-1;</t>
+        </is>
+      </c>
+      <c r="G128" s="9" t="inlineStr">
+        <is>
+          <t>Reconstructed. Only if enhancement is required. Conflicts with inter-CC load transfer on WBB CA UEs/RRNs. NSA PCC anchoring will override it.</t>
+        </is>
+      </c>
+      <c r="H128" s="10" t="n"/>
+      <c r="I128" s="10" t="n"/>
+      <c r="J128" s="11" t="n"/>
+    </row>
+    <row r="129" ht="24" customHeight="1">
+      <c r="A129" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B129" s="32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C129" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="inlineStr">
+        <is>
+          <t>FDD/TDD NSA</t>
+        </is>
+      </c>
+      <c r="E129" s="12" t="inlineStr">
+        <is>
+          <t>NSA exception</t>
+        </is>
+      </c>
+      <c r="F129" s="33" t="inlineStr">
+        <is>
+          <t>MOD ENBCELLRSVDPARA: LocalCellId=0, RsvdSwPara6=RsvdSwPara6_bit20-1;</t>
+        </is>
+      </c>
+      <c r="G129" s="12" t="inlineStr">
+        <is>
+          <t>Reconstructed from NSA FPD wording. Confirm bit name and command in Used Reserved Parameter List before live use.</t>
+        </is>
+      </c>
+      <c r="H129" s="10" t="n"/>
+      <c r="I129" s="10" t="n"/>
+      <c r="J129" s="11" t="n"/>
+    </row>
+    <row r="130" ht="24" customHeight="1">
+      <c r="A130" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="B130" s="36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>UL RB awareness</t>
+        </is>
+      </c>
+      <c r="F130" s="37" t="inlineStr">
+        <is>
+          <t>LST CELLALGOSWITCH: LocalCellId=0;</t>
+        </is>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>Inspect UlSchExtSwitch / UlMultiClusterSwitch. Do not toggle blindly; DSS FPD only states the RB-pool impact.</t>
+        </is>
+      </c>
+      <c r="H130" s="10" t="n"/>
+      <c r="I130" s="10" t="n"/>
+      <c r="J130" s="11" t="n"/>
+    </row>
+    <row r="131" ht="24" customHeight="1">
+      <c r="A131" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B131" s="32" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C131" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D131" s="12" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="E131" s="12" t="inlineStr">
+        <is>
+          <t>DSS coexistence check</t>
+        </is>
+      </c>
+      <c r="F131" s="33" t="inlineStr">
+        <is>
+          <t>LST SPECTRUMCLOUD: LocalCellId=0;</t>
+        </is>
+      </c>
+      <c r="G131" s="12" t="inlineStr">
+        <is>
+          <t>If SpectrumCloudSwitch is LTE_NR_SPECTRUM_SHR (or SUL), expect a smaller Spectrum Coordination UE proportion.</t>
+        </is>
+      </c>
+      <c r="H131" s="10" t="n"/>
+      <c r="I131" s="10" t="n"/>
+      <c r="J131" s="11" t="n"/>
+    </row>
+    <row r="132" ht="24" customHeight="1">
+      <c r="A132" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="B132" s="36" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>HO path</t>
+        </is>
+      </c>
+      <c r="F132" s="37" t="inlineStr">
+        <is>
+          <t>LST ENODEBALGOSWITCH:;</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>Confirm CaA5HoEventSwitch and CaA5HoEventEnhSwitch remain selected (CA Ch.4.3) so PCell↔SCell HO is possible.</t>
+        </is>
+      </c>
+      <c r="H132" s="10" t="n"/>
+      <c r="I132" s="10" t="n"/>
+      <c r="J132" s="11" t="n"/>
+    </row>
+    <row r="133" ht="24" customHeight="1">
+      <c r="A133" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B133" s="32" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C133" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E133" s="12" t="inlineStr">
+        <is>
+          <t>Verify</t>
+        </is>
+      </c>
+      <c r="F133" s="33" t="inlineStr">
+        <is>
+          <t>DSP CAMGTCFG: LocalCellId=0;</t>
+        </is>
+      </c>
+      <c r="G133" s="12" t="inlineStr">
+        <is>
+          <t>SpectrumCoordinationSwitch should show selected. Then watch CA PCell HO counters (section G).</t>
+        </is>
+      </c>
+      <c r="H133" s="10" t="n"/>
+      <c r="I133" s="10" t="n"/>
+      <c r="J133" s="11" t="n"/>
+    </row>
+    <row r="134" ht="24" customHeight="1">
+      <c r="A134" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="B134" s="36" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr">
+        <is>
+          <t>Rollback</t>
+        </is>
+      </c>
+      <c r="F134" s="37" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;</t>
+        </is>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>Stops UL-quality PCell changes. Repeat on every cell. Enhancement bit and reserved bit20 are independent rollbacks.</t>
+        </is>
+      </c>
+      <c r="H134" s="10" t="n"/>
+      <c r="I134" s="10" t="n"/>
+      <c r="J134" s="11" t="n"/>
+    </row>
+    <row r="135" ht="24" customHeight="1">
+      <c r="A135" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B135" s="32" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C135" s="12" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D135" s="12" t="inlineStr">
+        <is>
+          <t>TDD WBB/RRN</t>
+        </is>
+      </c>
+      <c r="E135" s="12" t="inlineStr">
+        <is>
+          <t>Rollback enhancement</t>
+        </is>
+      </c>
+      <c r="F135" s="33" t="inlineStr">
+        <is>
+          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-0;</t>
+        </is>
+      </c>
+      <c r="G135" s="12" t="inlineStr">
+        <is>
+          <t>Restores the possibility of inter-CC load transfer on those WBB/RRN UEs (subject to DlCaLbAlgoSwitch / CaLoadBalancePreAllocSwitch).</t>
+        </is>
+      </c>
+      <c r="H135" s="10" t="n"/>
+      <c r="I135" s="10" t="n"/>
+      <c r="J135" s="11" t="n"/>
+    </row>
+    <row r="136" ht="24" customHeight="1">
+      <c r="A136" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B136" s="36" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD NSA</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr">
+        <is>
+          <t>Rollback NSA exception</t>
+        </is>
+      </c>
+      <c r="F136" s="37" t="inlineStr">
+        <is>
+          <t>MOD ENBCELLRSVDPARA: LocalCellId=0, RsvdSwPara6=RsvdSwPara6_bit20-0;</t>
+        </is>
+      </c>
+      <c r="G136" s="9" t="inlineStr">
+        <is>
+          <t>Re-enables Spectrum Coordination for NSA DC UEs if the master switch is still On. Confirm MML.</t>
+        </is>
+      </c>
+      <c r="H136" s="10" t="n"/>
+      <c r="I136" s="10" t="n"/>
+      <c r="J136" s="11" t="n"/>
+    </row>
+    <row r="137" ht="22" customHeight="1">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>G.  Counters  (CA FPD set used as the live monitor — dedicated SC counters not in repo)</t>
+        </is>
+      </c>
+      <c r="B137" s="6" t="n"/>
+      <c r="C137" s="6" t="n"/>
+      <c r="D137" s="6" t="n"/>
+      <c r="E137" s="6" t="n"/>
+      <c r="F137" s="6" t="n"/>
+      <c r="G137" s="6" t="n"/>
+      <c r="H137" s="6" t="n"/>
+      <c r="I137" s="6" t="n"/>
+      <c r="J137" s="6" t="n"/>
+    </row>
+    <row r="138" ht="28" customHeight="1">
+      <c r="A138" s="16" t="inlineStr">
+        <is>
+          <t>CA FPD Ch.21 says to filter eNodeBFunction Performance Counter Summary by the feature ID of LTE Spectrum Coordination. That ID is not printed in the CA FPD. Until the dedicated FPD is available, use the CA PCell HO / SCell / throughput counters below to see whether PCells are moving and whether cell-edge DL bits rise.</t>
+        </is>
+      </c>
+      <c r="B138" s="17" t="n"/>
+      <c r="C138" s="17" t="n"/>
+      <c r="D138" s="17" t="n"/>
+      <c r="E138" s="17" t="n"/>
+      <c r="F138" s="17" t="n"/>
+      <c r="G138" s="17" t="n"/>
+      <c r="H138" s="17" t="n"/>
+      <c r="I138" s="17" t="n"/>
+      <c r="J138" s="17" t="n"/>
+    </row>
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>Counter ID</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t>Counter Name</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>Function / what it measures</t>
+        </is>
+      </c>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+      <c r="F139" s="7" t="inlineStr"/>
+      <c r="G139" s="7" t="inlineStr"/>
+      <c r="H139" s="7" t="inlineStr"/>
+      <c r="I139" s="7" t="inlineStr"/>
+      <c r="J139" s="7" t="inlineStr"/>
+    </row>
+    <row r="140" ht="32" customHeight="1">
+      <c r="A140" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t>1526728993</t>
+        </is>
+      </c>
+      <c r="C140" s="33" t="inlineStr">
+        <is>
+          <t>L.HHO.ExecAttOut.CAUser.PCC</t>
+        </is>
+      </c>
+      <c r="D140" s="12" t="inlineStr">
+        <is>
+          <t>CA UE PCell HO execution attempts</t>
+        </is>
+      </c>
+      <c r="E140" s="12" t="inlineStr">
+        <is>
+          <t>Expect a rise when SC starts swapping high↔low PCell. Compare with non-SC cluster.</t>
+        </is>
+      </c>
+      <c r="F140" s="10" t="n"/>
+      <c r="G140" s="10" t="n"/>
+      <c r="H140" s="10" t="n"/>
+      <c r="I140" s="10" t="n"/>
+      <c r="J140" s="11" t="n"/>
+    </row>
+    <row r="141" ht="32" customHeight="1">
+      <c r="A141" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>1526728994</t>
+        </is>
+      </c>
+      <c r="C141" s="37" t="inlineStr">
+        <is>
+          <t>L.HHO.ExecSuccOut.CAUser.PCC</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>CA UE PCell HO execution success</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Numerator of PCell HO success. Ping-pong if Att ≫ Succ or Att spikes with no KPI gain.</t>
+        </is>
+      </c>
+      <c r="F141" s="10" t="n"/>
+      <c r="G141" s="10" t="n"/>
+      <c r="H141" s="10" t="n"/>
+      <c r="I141" s="10" t="n"/>
+      <c r="J141" s="11" t="n"/>
+    </row>
+    <row r="142" ht="32" customHeight="1">
+      <c r="A142" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B142" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C142" s="33" t="inlineStr">
+        <is>
+          <t>L.HHO.PrepAttOut.CAUser.PCC (CA FPD HO family)</t>
+        </is>
+      </c>
+      <c r="D142" s="12" t="inlineStr">
+        <is>
+          <t>CA UE PCell HO preparations</t>
+        </is>
+      </c>
+      <c r="E142" s="12" t="inlineStr">
+        <is>
+          <t>Preparations without executions → measurement/threshold issue, not necessarily SC.</t>
+        </is>
+      </c>
+      <c r="F142" s="10" t="n"/>
+      <c r="G142" s="10" t="n"/>
+      <c r="H142" s="10" t="n"/>
+      <c r="I142" s="10" t="n"/>
+      <c r="J142" s="11" t="n"/>
+    </row>
+    <row r="143" ht="32" customHeight="1">
+      <c r="A143" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
+        <is>
+          <t>1526729045 / 9046</t>
+        </is>
+      </c>
+      <c r="C143" s="37" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Add.Att / .Succ</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>DL SCell add</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>After PCell moves to low band, high band must still add as SCell. If add fails, you get coverage-layer UL but lose high-band DL.</t>
+        </is>
+      </c>
+      <c r="F143" s="10" t="n"/>
+      <c r="G143" s="10" t="n"/>
+      <c r="H143" s="10" t="n"/>
+      <c r="I143" s="10" t="n"/>
+      <c r="J143" s="11" t="n"/>
+    </row>
+    <row r="144" ht="32" customHeight="1">
+      <c r="A144" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t>1526728999 / 9000</t>
+        </is>
+      </c>
+      <c r="C144" s="33" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Act.Att / .Succ</t>
+        </is>
+      </c>
+      <c r="D144" s="12" t="inlineStr">
+        <is>
+          <t>SCell MAC activation</t>
+        </is>
+      </c>
+      <c r="E144" s="12" t="inlineStr">
+        <is>
+          <t>DL decoupling only exists while the high-band SCell is active.</t>
+        </is>
+      </c>
+      <c r="F144" s="10" t="n"/>
+      <c r="G144" s="10" t="n"/>
+      <c r="H144" s="10" t="n"/>
+      <c r="I144" s="10" t="n"/>
+      <c r="J144" s="11" t="n"/>
+    </row>
+    <row r="145" ht="32" customHeight="1">
+      <c r="A145" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>1526732658 / 1526729259</t>
+        </is>
+      </c>
+      <c r="C145" s="37" t="inlineStr">
+        <is>
+          <t>L.CA.Traffic.bits.DL.PCell / .SCell</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>DL bits on PCell vs SCell of CA UEs</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Cell-edge: more bits should appear on the high-band SCell while PCell is the low band.</t>
+        </is>
+      </c>
+      <c r="F145" s="10" t="n"/>
+      <c r="G145" s="10" t="n"/>
+      <c r="H145" s="10" t="n"/>
+      <c r="I145" s="10" t="n"/>
+      <c r="J145" s="11" t="n"/>
+    </row>
+    <row r="146" ht="32" customHeight="1">
+      <c r="A146" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t>1526729003 / 9004</t>
+        </is>
+      </c>
+      <c r="C146" s="33" t="inlineStr">
+        <is>
+          <t>L.CA.DL.PCell.Act.Dur / SCell.Act.Dur</t>
+        </is>
+      </c>
+      <c r="D146" s="12" t="inlineStr">
+        <is>
+          <t>Active duration</t>
+        </is>
+      </c>
+      <c r="E146" s="12" t="inlineStr">
+        <is>
+          <t>Duration share high-as-SCell vs low-as-PCell is the operational fingerprint of SC.</t>
+        </is>
+      </c>
+      <c r="F146" s="10" t="n"/>
+      <c r="G146" s="10" t="n"/>
+      <c r="H146" s="10" t="n"/>
+      <c r="I146" s="10" t="n"/>
+      <c r="J146" s="11" t="n"/>
+    </row>
+    <row r="147" ht="32" customHeight="1">
+      <c r="A147" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C147" s="37" t="inlineStr">
+        <is>
+          <t>L.Thrp.bits.DL.CAUser / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>CA UE DL throughput ingredients</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Cell-edge bins (RSRP/SINR) should move if Turkcell-class gain is present.</t>
+        </is>
+      </c>
+      <c r="F147" s="10" t="n"/>
+      <c r="G147" s="10" t="n"/>
+      <c r="H147" s="10" t="n"/>
+      <c r="I147" s="10" t="n"/>
+      <c r="J147" s="11" t="n"/>
+    </row>
+    <row r="148" ht="32" customHeight="1">
+      <c r="A148" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>1526729047 / 9048</t>
+        </is>
+      </c>
+      <c r="C148" s="33" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Rmv.Att / .Succ</t>
+        </is>
+      </c>
+      <c r="D148" s="12" t="inlineStr">
+        <is>
+          <t>SCell remove</t>
+        </is>
+      </c>
+      <c r="E148" s="12" t="inlineStr">
+        <is>
+          <t>If SC PCell swap is followed by immediate SCell remove, overlap or A2 is too aggressive (Step1 leaving).</t>
+        </is>
+      </c>
+      <c r="F148" s="10" t="n"/>
+      <c r="G148" s="10" t="n"/>
+      <c r="H148" s="10" t="n"/>
+      <c r="I148" s="10" t="n"/>
+      <c r="J148" s="11" t="n"/>
+    </row>
+    <row r="149" ht="32" customHeight="1">
+      <c r="A149" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C149" s="37" t="inlineStr">
+        <is>
+          <t>UL: PUSCH SINR / UL MCS / UL IBLER (cell performance / UE trace)</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>UL quality of the current PCell</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>This is the actual trigger family. Use MAE-Access UE trace on the same IMSI before/after the PCell swap.</t>
+        </is>
+      </c>
+      <c r="F149" s="10" t="n"/>
+      <c r="G149" s="10" t="n"/>
+      <c r="H149" s="10" t="n"/>
+      <c r="I149" s="10" t="n"/>
+      <c r="J149" s="11" t="n"/>
+    </row>
+    <row r="150" ht="32" customHeight="1">
+      <c r="A150" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="C150" s="33" t="inlineStr">
+        <is>
+          <t>DSP UEONLINEINFO / RRC_CONN_RECFG</t>
+        </is>
+      </c>
+      <c r="D150" s="12" t="inlineStr">
+        <is>
+          <t>sCellToAddModList after PCell band change; non-zero RB/TBS on both CCs</t>
+        </is>
+      </c>
+      <c r="E150" s="12" t="inlineStr">
+        <is>
+          <t>Same verification style as CA Ch.5.4.2.</t>
+        </is>
+      </c>
+      <c r="F150" s="10" t="n"/>
+      <c r="G150" s="10" t="n"/>
+      <c r="H150" s="10" t="n"/>
+      <c r="I150" s="10" t="n"/>
+      <c r="J150" s="11" t="n"/>
+    </row>
+    <row r="151" ht="32" customHeight="1">
+      <c r="A151" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C151" s="37" t="inlineStr">
+        <is>
+          <t>Dedicated LTE Spectrum Coordination counters</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>Not published in this repository</t>
+        </is>
+      </c>
+      <c r="E151" s="9" t="inlineStr">
+        <is>
+          <t>Filter Performance Counter Summary by the feature ID from the dedicated FPD / License Control Item Lists.</t>
+        </is>
+      </c>
+      <c r="F151" s="10" t="n"/>
+      <c r="G151" s="10" t="n"/>
+      <c r="H151" s="10" t="n"/>
+      <c r="I151" s="10" t="n"/>
+      <c r="J151" s="11" t="n"/>
+    </row>
+    <row r="152" ht="22" customHeight="1">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>H.  KPI formulas</t>
+        </is>
+      </c>
+      <c r="B152" s="6" t="n"/>
+      <c r="C152" s="6" t="n"/>
+      <c r="D152" s="6" t="n"/>
+      <c r="E152" s="6" t="n"/>
+      <c r="F152" s="6" t="n"/>
+      <c r="G152" s="6" t="n"/>
+      <c r="H152" s="6" t="n"/>
+      <c r="I152" s="6" t="n"/>
+      <c r="J152" s="6" t="n"/>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B153" s="7" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="D153" s="7" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>Source / how to use</t>
+        </is>
+      </c>
+      <c r="F153" s="7" t="inlineStr"/>
+      <c r="G153" s="7" t="inlineStr"/>
+      <c r="H153" s="7" t="inlineStr"/>
+      <c r="I153" s="7" t="inlineStr"/>
+      <c r="J153" s="7" t="inlineStr"/>
+    </row>
+    <row r="154" ht="48" customHeight="1">
+      <c r="A154" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>CA UE PCell HO success rate</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>L.HHO.ExecSuccOut.CAUser.PCC / L.HHO.ExecAttOut.CAUser.PCC × 100%</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E154" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD Ch.5.4.3. Must stay healthy after SC is turned on; a drop means UL-quality PCell change is too aggressive or neighbors are missing.</t>
+        </is>
+      </c>
+      <c r="F154" s="10" t="n"/>
+      <c r="G154" s="10" t="n"/>
+      <c r="H154" s="10" t="n"/>
+      <c r="I154" s="10" t="n"/>
+      <c r="J154" s="11" t="n"/>
+    </row>
+    <row r="155" ht="48" customHeight="1">
+      <c r="A155" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B155" s="12" t="inlineStr">
+        <is>
+          <t>DL SCell add success (post-swap)</t>
+        </is>
+      </c>
+      <c r="C155" s="12" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Add.Succ / L.CA.DLSCell.Add.Att × 100%</t>
+        </is>
+      </c>
+      <c r="D155" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E155" s="12" t="inlineStr">
+        <is>
+          <t>CA FPD. After PCell moves to low band this is the rate at which high-band DL is recovered as SCell.</t>
+        </is>
+      </c>
+      <c r="F155" s="10" t="n"/>
+      <c r="G155" s="10" t="n"/>
+      <c r="H155" s="10" t="n"/>
+      <c r="I155" s="10" t="n"/>
+      <c r="J155" s="11" t="n"/>
+    </row>
+    <row r="156" ht="48" customHeight="1">
+      <c r="A156" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B156" s="9" t="inlineStr">
+        <is>
+          <t>SCell activation success</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Act.Succ / L.CA.DLSCell.Act.Att × 100%</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E156" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD. Decoupling is real only while both CCs are active.</t>
+        </is>
+      </c>
+      <c r="F156" s="10" t="n"/>
+      <c r="G156" s="10" t="n"/>
+      <c r="H156" s="10" t="n"/>
+      <c r="I156" s="10" t="n"/>
+      <c r="J156" s="11" t="n"/>
+    </row>
+    <row r="157" ht="48" customHeight="1">
+      <c r="A157" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B157" s="12" t="inlineStr">
+        <is>
+          <t>CA UE average DL data rate (last-TTI removed)</t>
+        </is>
+      </c>
+      <c r="C157" s="12" t="inlineStr">
+        <is>
+          <t>(L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D157" s="12" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E157" s="12" t="inlineStr">
+        <is>
+          <t>CA FPD. Split by RSRP band (cell-edge vs center) on the OSS. Cell-edge bin is the SC target.</t>
+        </is>
+      </c>
+      <c r="F157" s="10" t="n"/>
+      <c r="G157" s="10" t="n"/>
+      <c r="H157" s="10" t="n"/>
+      <c r="I157" s="10" t="n"/>
+      <c r="J157" s="11" t="n"/>
+    </row>
+    <row r="158" ht="48" customHeight="1">
+      <c r="A158" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B158" s="9" t="inlineStr">
+        <is>
+          <t>PCell vs SCell DL traffic share</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
+        <is>
+          <t>SCell bits / (PCell bits + SCell bits) = L.CA.Traffic.bits.DL.SCell / (L.CA.Traffic.bits.DL.PCell + L.CA.Traffic.bits.DL.SCell) × 100%</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E158" s="9" t="inlineStr">
+        <is>
+          <t>Operator identity from CA counters. On a low-band PCell + high-band SCell edge UE this share should be high.</t>
+        </is>
+      </c>
+      <c r="F158" s="10" t="n"/>
+      <c r="G158" s="10" t="n"/>
+      <c r="H158" s="10" t="n"/>
+      <c r="I158" s="10" t="n"/>
+      <c r="J158" s="11" t="n"/>
+    </row>
+    <row r="159" ht="48" customHeight="1">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B159" s="12" t="inlineStr">
+        <is>
+          <t>Cell-edge DL rate gain (trial KPI)</t>
+        </is>
+      </c>
+      <c r="C159" s="12" t="inlineStr">
+        <is>
+          <t>(R_edge_after − R_edge_before) / R_edge_before × 100%</t>
+        </is>
+      </c>
+      <c r="D159" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E159" s="12" t="inlineStr">
+        <is>
+          <t>Huawei/Turkcell commercial trial reported &gt; 30% cell-edge downlink data rate. Use the same cell-edge definition (e.g. RSRP &lt; −110 dBm or UL SINR &lt; 0 dB) before and after. Not a Huawei counter formula.</t>
+        </is>
+      </c>
+      <c r="F159" s="10" t="n"/>
+      <c r="G159" s="10" t="n"/>
+      <c r="H159" s="10" t="n"/>
+      <c r="I159" s="10" t="n"/>
+      <c r="J159" s="11" t="n"/>
+    </row>
+    <row r="160" ht="48" customHeight="1">
+      <c r="A160" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>CA UE E-RAB drop rate</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr">
+        <is>
+          <t>L.E-RAB.AbnormRel.CAUser / (L.E-RAB.AbnormRel.CAUser + L.E-RAB.NormRel.CAUser) × 100%</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E160" s="9" t="inlineStr">
+        <is>
+          <t>CA FPD. PCell ping-pong from SC must not raise drop.</t>
+        </is>
+      </c>
+      <c r="F160" s="10" t="n"/>
+      <c r="G160" s="10" t="n"/>
+      <c r="H160" s="10" t="n"/>
+      <c r="I160" s="10" t="n"/>
+      <c r="J160" s="11" t="n"/>
+    </row>
+    <row r="161" ht="48" customHeight="1">
+      <c r="A161" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B161" s="12" t="inlineStr">
+        <is>
+          <t>Spectrum Coordination take-effect ratio (qualitative)</t>
+        </is>
+      </c>
+      <c r="C161" s="12" t="inlineStr">
+        <is>
+          <t>UEs with UL-quality PCell swap / CA UEs on the pair   —  exact counter not in repo</t>
+        </is>
+      </c>
+      <c r="D161" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E161" s="12" t="inlineStr">
+        <is>
+          <t>DSS FPD states this ratio falls when LTE UL RBs shrink. Track via PCell band distribution of CA UEs (high-band PCell % in center vs edge).</t>
+        </is>
+      </c>
+      <c r="F161" s="10" t="n"/>
+      <c r="G161" s="10" t="n"/>
+      <c r="H161" s="10" t="n"/>
+      <c r="I161" s="10" t="n"/>
+      <c r="J161" s="11" t="n"/>
+    </row>
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="21" t="inlineStr">
+        <is>
+          <t>H2.  Sample arithmetic  (cell-edge gain)</t>
+        </is>
+      </c>
+      <c r="B162" s="22" t="n"/>
+      <c r="C162" s="22" t="n"/>
+      <c r="D162" s="22" t="n"/>
+      <c r="E162" s="22" t="n"/>
+      <c r="F162" s="22" t="n"/>
+      <c r="G162" s="22" t="n"/>
+      <c r="H162" s="22" t="n"/>
+      <c r="I162" s="22" t="n"/>
+      <c r="J162" s="22" t="n"/>
+    </row>
+    <row r="163" ht="20" customHeight="1">
+      <c r="A163" s="26" t="inlineStr">
+        <is>
+          <t>Turkcell-class cell-edge DL gain  (public trial, not an MML output)</t>
+        </is>
+      </c>
+      <c r="B163" s="6" t="n"/>
+      <c r="C163" s="6" t="n"/>
+      <c r="D163" s="6" t="n"/>
+      <c r="E163" s="6" t="n"/>
+      <c r="F163" s="6" t="n"/>
+      <c r="G163" s="6" t="n"/>
+      <c r="H163" s="6" t="n"/>
+      <c r="I163" s="6" t="n"/>
+      <c r="J163" s="6" t="n"/>
+    </row>
+    <row r="164" ht="42" customHeight="1">
+      <c r="A164" s="27" t="inlineStr">
+        <is>
+          <t>3GPP / Huawei condition:
+Gain% = (R_after − R_before) / R_before × 100%</t>
+        </is>
+      </c>
+      <c r="B164" s="28" t="n"/>
+      <c r="C164" s="28" t="n"/>
+      <c r="D164" s="28" t="n"/>
+      <c r="E164" s="28" t="n"/>
+      <c r="F164" s="28" t="n"/>
+      <c r="G164" s="28" t="n"/>
+      <c r="H164" s="28" t="n"/>
+      <c r="I164" s="28" t="n"/>
+      <c r="J164" s="28" t="n"/>
+    </row>
+    <row r="165" ht="90" customHeight="1">
+      <c r="A165" s="13" t="inlineStr">
+        <is>
+          <t>Worked example (sample values from the document or typical live-network settings):
+Suppose a cell-edge CA UE (high-band PCell, UL limited) had R_before = 8 Mbit/s DL because UL ACK/NACK and UL traffic collapsed.
+After SC the same location uses low-band PCell + high-band SCell: R_after = 10.5 Mbit/s.
+Gain% = (10.5 − 8) / 8 × 100% = 31.25%.
+Result: This matches the order of the published “over 30% at cell edges” result. If your after-rate does not move, first check SCell add/act success and remaining LTE UL RBs (DSS), not the 30% figure itself.</t>
+        </is>
+      </c>
+      <c r="B165" s="14" t="n"/>
+      <c r="C165" s="14" t="n"/>
+      <c r="D165" s="14" t="n"/>
+      <c r="E165" s="14" t="n"/>
+      <c r="F165" s="14" t="n"/>
+      <c r="G165" s="14" t="n"/>
+      <c r="H165" s="14" t="n"/>
+      <c r="I165" s="14" t="n"/>
+      <c r="J165" s="14" t="n"/>
+    </row>
+    <row r="166" ht="22" customHeight="1">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>I.  Licenses — FDD and TDD</t>
+        </is>
+      </c>
+      <c r="B166" s="6" t="n"/>
+      <c r="C166" s="6" t="n"/>
+      <c r="D166" s="6" t="n"/>
+      <c r="E166" s="6" t="n"/>
+      <c r="F166" s="6" t="n"/>
+      <c r="G166" s="6" t="n"/>
+      <c r="H166" s="6" t="n"/>
+      <c r="I166" s="6" t="n"/>
+      <c r="J166" s="6" t="n"/>
+    </row>
+    <row r="167" ht="22" customHeight="1">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>RAT</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>Feature ID</t>
+        </is>
+      </c>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t>Feature name</t>
+        </is>
+      </c>
+      <c r="E167" s="7" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="F167" s="7" t="inlineStr">
+        <is>
+          <t>Sales unit</t>
+        </is>
+      </c>
+      <c r="G167" s="7" t="inlineStr">
+        <is>
+          <t>When consumed</t>
+        </is>
+      </c>
+      <c r="H167" s="7" t="inlineStr"/>
+      <c r="I167" s="7" t="inlineStr"/>
+      <c r="J167" s="7" t="inlineStr"/>
+    </row>
+    <row r="168" ht="52" customHeight="1">
+      <c r="A168" s="30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B168" s="30" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="C168" s="30" t="inlineStr">
+        <is>
+          <t>Not printed in CA FPD</t>
+        </is>
+      </c>
+      <c r="D168" s="30" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination (LTE FDD)</t>
+        </is>
+      </c>
+      <c r="E168" s="30" t="inlineStr">
+        <is>
+          <t>Not in repo — open License Control Item Lists (FDD) (CA FPD ref 91)</t>
+        </is>
+      </c>
+      <c r="F168" s="30" t="inlineStr">
+        <is>
+          <t>See list (typically per cell)</t>
+        </is>
+      </c>
+      <c r="G168" s="30" t="inlineStr">
+        <is>
+          <t>Related FPD CellCaAlgoSwitch listing names this feature on the same MO as CA bits. Do not assume a CA license (LAOFD-*) covers it.</t>
+        </is>
+      </c>
+      <c r="H168" s="10" t="n"/>
+      <c r="I168" s="10" t="n"/>
+      <c r="J168" s="11" t="n"/>
+    </row>
+    <row r="169" ht="52" customHeight="1">
+      <c r="A169" s="30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B169" s="30" t="inlineStr">
+        <is>
+          <t>TDD</t>
+        </is>
+      </c>
+      <c r="C169" s="30" t="inlineStr">
+        <is>
+          <t>Not printed in CA FPD</t>
+        </is>
+      </c>
+      <c r="D169" s="30" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination (LTE TDD)</t>
+        </is>
+      </c>
+      <c r="E169" s="30" t="inlineStr">
+        <is>
+          <t>Not in repo — open License Control Item Lists (TDD) (CA FPD ref 93)</t>
+        </is>
+      </c>
+      <c r="F169" s="30" t="inlineStr">
+        <is>
+          <t>See list (typically per cell)</t>
+        </is>
+      </c>
+      <c r="G169" s="30" t="inlineStr">
+        <is>
+          <t>Same as FDD: separate from TDLAOFD CA licenses. Enhancement (WbbCaMultiCarrierCoordSw) may share or add a WBB license — confirm in WBB FPD (CA ref 54).</t>
+        </is>
+      </c>
+      <c r="H169" s="10" t="n"/>
+      <c r="I169" s="10" t="n"/>
+      <c r="J169" s="11" t="n"/>
+    </row>
+    <row r="170" ht="52" customHeight="1">
+      <c r="A170" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B170" s="9" t="inlineStr">
+        <is>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>LAOFD-001001 / TDLAOFD-001001 (and 40 MHz / 3CC / 4CC+5CC as deployed)</t>
+        </is>
+      </c>
+      <c r="D170" s="9" t="inlineStr">
+        <is>
+          <t>Downlink CA (this workbook Steps 1–4)</t>
+        </is>
+      </c>
+      <c r="E170" s="9" t="inlineStr">
+        <is>
+          <t>See Step1–4 license tables</t>
+        </is>
+      </c>
+      <c r="F170" s="9" t="inlineStr">
+        <is>
+          <t>per cell</t>
+        </is>
+      </c>
+      <c r="G170" s="9" t="inlineStr">
+        <is>
+          <t>Still required. Spectrum Coordination rides on CA. License insufficiency of CA items can block CELL ACTIVATION.</t>
+        </is>
+      </c>
+      <c r="H170" s="10" t="n"/>
+      <c r="I170" s="10" t="n"/>
+      <c r="J170" s="11" t="n"/>
+    </row>
+    <row r="171" ht="52" customHeight="1">
+      <c r="A171" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B171" s="12" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="C171" s="12" t="inlineStr">
+        <is>
+          <t>MRFD160222 family (DSS) — only if DSS is also on</t>
+        </is>
+      </c>
+      <c r="D171" s="12" t="inlineStr">
+        <is>
+          <t>LTE FDD and NR Flash Dynamic Spectrum Sharing</t>
+        </is>
+      </c>
+      <c r="E171" s="12" t="inlineStr">
+        <is>
+          <t>LT1S0LFNSS00 (DSS FPD, not SC)</t>
+        </is>
+      </c>
+      <c r="F171" s="12" t="inlineStr">
+        <is>
+          <t>per cell</t>
+        </is>
+      </c>
+      <c r="G171" s="12" t="inlineStr">
+        <is>
+          <t>Listed so planners do not confuse DSS licenses with Spectrum Coordination. DSS reduces SC take-effect ratio.</t>
+        </is>
+      </c>
+      <c r="H171" s="10" t="n"/>
+      <c r="I171" s="10" t="n"/>
+      <c r="J171" s="11" t="n"/>
+    </row>
+    <row r="172" ht="28" customHeight="1">
+      <c r="A172" s="16" t="inlineStr">
+        <is>
+          <t>No Feature ID / Model for LTE Spectrum Coordination is printed in the CA FPD, DSS FPD extract, or NSA FPD extract used here. Do not copy guessed IDs into a license request. Use License Control Item Lists (FDD/TDD) and the dedicated FPD.</t>
+        </is>
+      </c>
+      <c r="B172" s="17" t="n"/>
+      <c r="C172" s="17" t="n"/>
+      <c r="D172" s="17" t="n"/>
+      <c r="E172" s="17" t="n"/>
+      <c r="F172" s="17" t="n"/>
+      <c r="G172" s="17" t="n"/>
+      <c r="H172" s="17" t="n"/>
+      <c r="I172" s="17" t="n"/>
+      <c r="J172" s="17" t="n"/>
+    </row>
+    <row r="173" ht="22" customHeight="1">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>J.  Deployment checklist  (after Step1 CA is green)</t>
+        </is>
+      </c>
+      <c r="B173" s="6" t="n"/>
+      <c r="C173" s="6" t="n"/>
+      <c r="D173" s="6" t="n"/>
+      <c r="E173" s="6" t="n"/>
+      <c r="F173" s="6" t="n"/>
+      <c r="G173" s="6" t="n"/>
+      <c r="H173" s="6" t="n"/>
+      <c r="I173" s="6" t="n"/>
+      <c r="J173" s="6" t="n"/>
+    </row>
+    <row r="174" ht="22" customHeight="1">
+      <c r="A174" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D174" s="7" t="inlineStr">
+        <is>
+          <t>Pass criteria</t>
+        </is>
+      </c>
+      <c r="E174" s="7" t="inlineStr"/>
+      <c r="F174" s="7" t="inlineStr"/>
+      <c r="G174" s="7" t="inlineStr"/>
+      <c r="H174" s="7" t="inlineStr"/>
+      <c r="I174" s="7" t="inlineStr"/>
+      <c r="J174" s="7" t="inlineStr"/>
+    </row>
+    <row r="175" ht="32" customHeight="1">
+      <c r="A175" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
+        <is>
+          <t>Cluster</t>
+        </is>
+      </c>
+      <c r="C175" s="9" t="inlineStr">
+        <is>
+          <t>High + low (or TDD high + FDD low) co-coverage pair chosen</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>Overlap plot; CA neighbors exist; FREQ_MEAS_FLAG selected</t>
+        </is>
+      </c>
+      <c r="E175" s="10" t="n"/>
+      <c r="F175" s="10" t="n"/>
+      <c r="G175" s="10" t="n"/>
+      <c r="H175" s="10" t="n"/>
+      <c r="I175" s="10" t="n"/>
+      <c r="J175" s="11" t="n"/>
+    </row>
+    <row r="176" ht="32" customHeight="1">
+      <c r="A176" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>CA baseline</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="inlineStr">
+        <is>
+          <t>Step1 2CC counters non-zero for a week</t>
+        </is>
+      </c>
+      <c r="D176" s="12" t="inlineStr">
+        <is>
+          <t>SCell add/act success high; CA UE rate &gt; non-CA</t>
+        </is>
+      </c>
+      <c r="E176" s="10" t="n"/>
+      <c r="F176" s="10" t="n"/>
+      <c r="G176" s="10" t="n"/>
+      <c r="H176" s="10" t="n"/>
+      <c r="I176" s="10" t="n"/>
+      <c r="J176" s="11" t="n"/>
+    </row>
+    <row r="177" ht="32" customHeight="1">
+      <c r="A177" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B177" s="9" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
+        <is>
+          <t>Spectrum Coordination + CA licenses on both cells</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>LST LICENSE / License Control Item Lists — do not guess models</t>
+        </is>
+      </c>
+      <c r="E177" s="10" t="n"/>
+      <c r="F177" s="10" t="n"/>
+      <c r="G177" s="10" t="n"/>
+      <c r="H177" s="10" t="n"/>
+      <c r="I177" s="10" t="n"/>
+      <c r="J177" s="11" t="n"/>
+    </row>
+    <row r="178" ht="32" customHeight="1">
+      <c r="A178" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B178" s="12" t="inlineStr">
+        <is>
+          <t>Conflicts</t>
+        </is>
+      </c>
+      <c r="C178" s="12" t="inlineStr">
+        <is>
+          <t>DSS UL RB share, UlMultiClusterSwitch, NSA bit20, WBB load-transfer</t>
+        </is>
+      </c>
+      <c r="D178" s="12" t="inlineStr">
+        <is>
+          <t>Documented coexistence: fewer UL RBs → fewer SC UEs; bit20 if NSA PCC must stay</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="n"/>
+      <c r="F178" s="10" t="n"/>
+      <c r="G178" s="10" t="n"/>
+      <c r="H178" s="10" t="n"/>
+      <c r="I178" s="10" t="n"/>
+      <c r="J178" s="11" t="n"/>
+    </row>
+    <row r="179" ht="32" customHeight="1">
+      <c r="A179" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>HO path</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="inlineStr">
+        <is>
+          <t>CaA5HoEventSwitch + CaA5HoEventEnhSwitch</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>PCell can HO to SCell</t>
+        </is>
+      </c>
+      <c r="E179" s="10" t="n"/>
+      <c r="F179" s="10" t="n"/>
+      <c r="G179" s="10" t="n"/>
+      <c r="H179" s="10" t="n"/>
+      <c r="I179" s="10" t="n"/>
+      <c r="J179" s="11" t="n"/>
+    </row>
+    <row r="180" ht="32" customHeight="1">
+      <c r="A180" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B180" s="12" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="C180" s="12" t="inlineStr">
+        <is>
+          <t>SpectrumCoordinationSwitch-1 on both cells of the pair</t>
+        </is>
+      </c>
+      <c r="D180" s="12" t="inlineStr">
+        <is>
+          <t>DSP CAMGTCFG shows selected</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="n"/>
+      <c r="F180" s="10" t="n"/>
+      <c r="G180" s="10" t="n"/>
+      <c r="H180" s="10" t="n"/>
+      <c r="I180" s="10" t="n"/>
+      <c r="J180" s="11" t="n"/>
+    </row>
+    <row r="181" ht="32" customHeight="1">
+      <c r="A181" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>Monitor 24–72 h</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
+          <t>PCell HO, SCell add/act, cell-edge DL rate, drop</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>HO success stable; cell-edge DL up; no ping-pong</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="n"/>
+      <c r="F181" s="10" t="n"/>
+      <c r="G181" s="10" t="n"/>
+      <c r="H181" s="10" t="n"/>
+      <c r="I181" s="10" t="n"/>
+      <c r="J181" s="11" t="n"/>
+    </row>
+    <row r="182" ht="32" customHeight="1">
+      <c r="A182" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B182" s="12" t="inlineStr">
+        <is>
+          <t>Optimize or roll back</t>
+        </is>
+      </c>
+      <c r="C182" s="12" t="inlineStr">
+        <is>
+          <t>If ping-pong or drop, switch-0 and open dedicated FPD for hysteresis</t>
+        </is>
+      </c>
+      <c r="D182" s="12" t="inlineStr">
+        <is>
+          <t>Rollback MML in section F seq 9</t>
+        </is>
+      </c>
+      <c r="E182" s="10" t="n"/>
+      <c r="F182" s="10" t="n"/>
+      <c r="G182" s="10" t="n"/>
+      <c r="H182" s="10" t="n"/>
+      <c r="I182" s="10" t="n"/>
+      <c r="J182" s="11" t="n"/>
+    </row>
+    <row r="183" ht="22" customHeight="1">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>K.  Sources  (every claim on this sheet traces to one of these)</t>
+        </is>
+      </c>
+      <c r="B183" s="6" t="n"/>
+      <c r="C183" s="6" t="n"/>
+      <c r="D183" s="6" t="n"/>
+      <c r="E183" s="6" t="n"/>
+      <c r="F183" s="6" t="n"/>
+      <c r="G183" s="6" t="n"/>
+      <c r="H183" s="6" t="n"/>
+      <c r="I183" s="6" t="n"/>
+      <c r="J183" s="6" t="n"/>
+    </row>
+    <row r="184" ht="22" customHeight="1">
+      <c r="A184" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B184" s="7" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C184" s="7" t="inlineStr">
+        <is>
+          <t>What was taken from it</t>
+        </is>
+      </c>
+      <c r="D184" s="7" t="inlineStr"/>
+      <c r="E184" s="7" t="inlineStr"/>
+      <c r="F184" s="7" t="inlineStr"/>
+      <c r="G184" s="7" t="inlineStr"/>
+      <c r="H184" s="7" t="inlineStr"/>
+      <c r="I184" s="7" t="inlineStr"/>
+      <c r="J184" s="7" t="inlineStr"/>
+    </row>
+    <row r="185" ht="52" customHeight="1">
+      <c r="A185" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
+        <is>
+          <t>Huawei eRAN Carrier Aggregation FPD, eRAN21.1 Issue 11 (2026-06-30), Ch.23 item 55</t>
+        </is>
+      </c>
+      <c r="C185" s="9" t="inlineStr">
+        <is>
+          <t>Identifies LTE Spectrum Coordination as a related eRAN FPD. CloudAIR impact rows: WbbCaMultiCarrierCoordSw vs DlCaLbAlgoSwitch / CaLoadBalancePreAllocSwitch on WBB CA UEs/RRNs (Ch.5 and Ch.13).</t>
+        </is>
+      </c>
+      <c r="D185" s="10" t="n"/>
+      <c r="E185" s="10" t="n"/>
+      <c r="F185" s="10" t="n"/>
+      <c r="G185" s="10" t="n"/>
+      <c r="H185" s="10" t="n"/>
+      <c r="I185" s="10" t="n"/>
+      <c r="J185" s="11" t="n"/>
+    </row>
+    <row r="186" ht="52" customHeight="1">
+      <c r="A186" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t>CaMgtCfg.CellCaAlgoSwitch option text in related eRAN FPDs (CoMP / parameter listing)</t>
+        </is>
+      </c>
+      <c r="C186" s="12" t="inlineStr">
+        <is>
+          <t>SpectrumCoordinationSwitch: enabled only if selected; PCell changes triggered based on uplink quality; FDD and TDD; default Off. Feature names “LTE Spectrum Coordination (LTE FDD/TDD)” appear on that MO.</t>
+        </is>
+      </c>
+      <c r="D186" s="10" t="n"/>
+      <c r="E186" s="10" t="n"/>
+      <c r="F186" s="10" t="n"/>
+      <c r="G186" s="10" t="n"/>
+      <c r="H186" s="10" t="n"/>
+      <c r="I186" s="10" t="n"/>
+      <c r="J186" s="11" t="n"/>
+    </row>
+    <row r="187" ht="52" customHeight="1">
+      <c r="A187" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B187" s="9" t="inlineStr">
+        <is>
+          <t>SingleRAN LTE FDD and NR Spectrum Sharing FPD (Flash DSS) function-impact table</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>SpectrumCoordinationSwitch identity. Fewer LTE UL RBs → smaller proportion of UEs for which Spectrum Coordination takes effect. UlMultiClusterSwitch listed on the same impact.</t>
+        </is>
+      </c>
+      <c r="D187" s="10" t="n"/>
+      <c r="E187" s="10" t="n"/>
+      <c r="F187" s="10" t="n"/>
+      <c r="G187" s="10" t="n"/>
+      <c r="H187" s="10" t="n"/>
+      <c r="I187" s="10" t="n"/>
+      <c r="J187" s="11" t="n"/>
+    </row>
+    <row r="188" ht="52" customHeight="1">
+      <c r="A188" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B188" s="12" t="inlineStr">
+        <is>
+          <t>EPC-based NSA Performance Enhancement FPD</t>
+        </is>
+      </c>
+      <c r="C188" s="12" t="inlineStr">
+        <is>
+          <t>RsvdSwPara6_bit20 disables Spectrum Coordination for NSA DC UEs. WbbCaMultiCarrierCoordSw = coordination enhancement. NSA DC PCC anchoring takes precedence over the enhancement.</t>
+        </is>
+      </c>
+      <c r="D188" s="10" t="n"/>
+      <c r="E188" s="10" t="n"/>
+      <c r="F188" s="10" t="n"/>
+      <c r="G188" s="10" t="n"/>
+      <c r="H188" s="10" t="n"/>
+      <c r="I188" s="10" t="n"/>
+      <c r="J188" s="11" t="n"/>
+    </row>
+    <row r="189" ht="52" customHeight="1">
+      <c r="A189" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>Huawei press: Turkcell Antalya, 22 Jan 2018, eRAN 13.1 commercial network</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="inlineStr">
+        <is>
+          <t>DL always on high+low; UL selected high (center) or low (edge); cell-edge DL rate +30%+. CloudAIR key technology; lifts UL/DL channel binding.</t>
+        </is>
+      </c>
+      <c r="D189" s="10" t="n"/>
+      <c r="E189" s="10" t="n"/>
+      <c r="F189" s="10" t="n"/>
+      <c r="G189" s="10" t="n"/>
+      <c r="H189" s="10" t="n"/>
+      <c r="I189" s="10" t="n"/>
+      <c r="J189" s="11" t="n"/>
+    </row>
+    <row r="190" ht="52" customHeight="1">
+      <c r="A190" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B190" s="12" t="inlineStr">
+        <is>
+          <t>Huawei CloudAIR white paper (Jan 2018)</t>
+        </is>
+      </c>
+      <c r="C190" s="12" t="inlineStr">
+        <is>
+          <t>Channel cloudification example: LTE spectrum coordination uses high and low bands; FDD high+low and TDD high + FDD low.</t>
+        </is>
+      </c>
+      <c r="D190" s="10" t="n"/>
+      <c r="E190" s="10" t="n"/>
+      <c r="F190" s="10" t="n"/>
+      <c r="G190" s="10" t="n"/>
+      <c r="H190" s="10" t="n"/>
+      <c r="I190" s="10" t="n"/>
+      <c r="J190" s="11" t="n"/>
+    </row>
+    <row r="191" ht="52" customHeight="1">
+      <c r="A191" s="30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B191" s="30" t="inlineStr">
+        <is>
+          <t>This repository — not present</t>
+        </is>
+      </c>
+      <c r="C191" s="30" t="inlineStr">
+        <is>
+          <t>Dedicated “LTE Spectrum Coordination” Feature Parameter Description (thresholds, MML examples, counters, license models). Obtain from 3900 &amp; 5900 Series Base Station Product Documentation (CA FPD ref 100).</t>
+        </is>
+      </c>
+      <c r="D191" s="10" t="n"/>
+      <c r="E191" s="10" t="n"/>
+      <c r="F191" s="10" t="n"/>
+      <c r="G191" s="10" t="n"/>
+      <c r="H191" s="10" t="n"/>
+      <c r="I191" s="10" t="n"/>
+      <c r="J191" s="11" t="n"/>
+    </row>
+    <row r="192" ht="33" customHeight="1">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>If the dedicated LTE Spectrum Coordination FPD is added to this repository later, this sheet should be extended with its trigger/leave charts, full parameter list, verbatim MML, counters, KPI, and FDD/TDD licenses — the same depth as Step1 2CC.</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="n"/>
+      <c r="C192" s="4" t="n"/>
+      <c r="D192" s="4" t="n"/>
+      <c r="E192" s="4" t="n"/>
+      <c r="F192" s="4" t="n"/>
+      <c r="G192" s="4" t="n"/>
+      <c r="H192" s="4" t="n"/>
+      <c r="I192" s="4" t="n"/>
+      <c r="J192" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="143">
+    <mergeCell ref="E143:J143"/>
+    <mergeCell ref="D176:J176"/>
+    <mergeCell ref="A91:J91"/>
+    <mergeCell ref="G109:J109"/>
+    <mergeCell ref="G135:J135"/>
+    <mergeCell ref="D177:J177"/>
+    <mergeCell ref="E149:J149"/>
+    <mergeCell ref="A165:J165"/>
+    <mergeCell ref="G119:J119"/>
+    <mergeCell ref="C35:J35"/>
+    <mergeCell ref="G111:J111"/>
+    <mergeCell ref="D88:J88"/>
+    <mergeCell ref="A173:J173"/>
+    <mergeCell ref="G96:J96"/>
+    <mergeCell ref="G136:J136"/>
+    <mergeCell ref="A49:J49"/>
+    <mergeCell ref="A138:J138"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="E159:J159"/>
+    <mergeCell ref="A69:J69"/>
+    <mergeCell ref="E145:J145"/>
+    <mergeCell ref="A183:J183"/>
+    <mergeCell ref="G128:J128"/>
+    <mergeCell ref="A66:J66"/>
+    <mergeCell ref="G171:J171"/>
+    <mergeCell ref="E142:J142"/>
+    <mergeCell ref="D179:J179"/>
+    <mergeCell ref="A120:J120"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="C38:J38"/>
+    <mergeCell ref="G74:J74"/>
+    <mergeCell ref="G108:J108"/>
+    <mergeCell ref="D181:J181"/>
+    <mergeCell ref="E140:J140"/>
+    <mergeCell ref="G114:J114"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="G110:J110"/>
+    <mergeCell ref="E155:J155"/>
+    <mergeCell ref="D180:J180"/>
+    <mergeCell ref="G168:J168"/>
+    <mergeCell ref="A106:J106"/>
+    <mergeCell ref="G113:J113"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="G100:J100"/>
+    <mergeCell ref="A81:J81"/>
+    <mergeCell ref="G94:J94"/>
+    <mergeCell ref="C187:J187"/>
+    <mergeCell ref="A121:J121"/>
+    <mergeCell ref="E157:J157"/>
+    <mergeCell ref="G75:J75"/>
+    <mergeCell ref="D89:J89"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="G102:J102"/>
+    <mergeCell ref="A67:J67"/>
+    <mergeCell ref="G77:J77"/>
+    <mergeCell ref="A82:J82"/>
+    <mergeCell ref="A123:J123"/>
+    <mergeCell ref="G97:J97"/>
+    <mergeCell ref="C36:J36"/>
+    <mergeCell ref="A7:J7"/>
+    <mergeCell ref="G125:J125"/>
+    <mergeCell ref="A172:J172"/>
+    <mergeCell ref="G112:J112"/>
+    <mergeCell ref="G127:J127"/>
+    <mergeCell ref="C190:J190"/>
+    <mergeCell ref="C37:J37"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="G104:J104"/>
+    <mergeCell ref="C186:J186"/>
+    <mergeCell ref="E147:J147"/>
+    <mergeCell ref="A47:J47"/>
+    <mergeCell ref="E156:J156"/>
+    <mergeCell ref="A122:J122"/>
+    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="C185:J185"/>
+    <mergeCell ref="C191:J191"/>
+    <mergeCell ref="G76:J76"/>
+    <mergeCell ref="G99:J99"/>
+    <mergeCell ref="E148:J148"/>
+    <mergeCell ref="A152:J152"/>
+    <mergeCell ref="D85:J85"/>
+    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="D182:J182"/>
+    <mergeCell ref="E154:J154"/>
+    <mergeCell ref="G115:J115"/>
+    <mergeCell ref="G130:J130"/>
+    <mergeCell ref="G117:J117"/>
+    <mergeCell ref="G169:J169"/>
+    <mergeCell ref="D46:J46"/>
+    <mergeCell ref="G126:J126"/>
+    <mergeCell ref="G132:J132"/>
+    <mergeCell ref="C188:J188"/>
+    <mergeCell ref="A70:J70"/>
+    <mergeCell ref="A162:J162"/>
+    <mergeCell ref="E146:J146"/>
+    <mergeCell ref="G101:J101"/>
+    <mergeCell ref="G116:J116"/>
+    <mergeCell ref="A137:J137"/>
+    <mergeCell ref="G103:J103"/>
+    <mergeCell ref="A90:J90"/>
+    <mergeCell ref="E151:J151"/>
+    <mergeCell ref="A164:J164"/>
+    <mergeCell ref="D41:J41"/>
+    <mergeCell ref="G78:J78"/>
+    <mergeCell ref="E160:J160"/>
+    <mergeCell ref="G118:J118"/>
+    <mergeCell ref="E150:J150"/>
+    <mergeCell ref="A163:J163"/>
+    <mergeCell ref="D87:J87"/>
+    <mergeCell ref="C189:J189"/>
+    <mergeCell ref="D43:J43"/>
+    <mergeCell ref="G95:J95"/>
+    <mergeCell ref="C34:J34"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="E161:J161"/>
+    <mergeCell ref="G79:J79"/>
+    <mergeCell ref="G73:J73"/>
+    <mergeCell ref="E158:J158"/>
+    <mergeCell ref="D42:J42"/>
+    <mergeCell ref="G134:J134"/>
+    <mergeCell ref="A68:J68"/>
+    <mergeCell ref="D44:J44"/>
+    <mergeCell ref="A39:J39"/>
+    <mergeCell ref="D178:J178"/>
+    <mergeCell ref="A166:J166"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="E144:J144"/>
+    <mergeCell ref="G98:J98"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="D84:J84"/>
+    <mergeCell ref="G170:J170"/>
+    <mergeCell ref="D45:J45"/>
+    <mergeCell ref="A65:J65"/>
+    <mergeCell ref="D86:J86"/>
+    <mergeCell ref="G93:J93"/>
+    <mergeCell ref="A80:J80"/>
+    <mergeCell ref="D175:J175"/>
+    <mergeCell ref="A192:J192"/>
+    <mergeCell ref="A105:J105"/>
+    <mergeCell ref="E141:J141"/>
+    <mergeCell ref="G133:J133"/>
+    <mergeCell ref="A71:J71"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.25" footer="0.25"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;LCarrier Aggregation Deployment Guide&amp;R&amp;A</oddHeader>
+    <oddFooter>&amp;LSource: Huawei eRAN CA Feature Parameter Description, eRAN21.1 Issue 11 (2026-06-30)&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify Spectrum Coordination MML to LocalCellId=1 and add meeting brief
Keep one cell in the MML samples and add a final-summary block for
meeting talking points (benefit, trigger/leave, UL/DL CA limits, GPS).

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Carrier_Aggregation_Deployment.xlsx
+++ b/Carrier_Aggregation_Deployment.xlsx
@@ -100,7 +100,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -160,6 +160,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9A227"/>
       </patternFill>
     </fill>
   </fills>
@@ -233,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -348,6 +353,10 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23041,7 +23050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J189"/>
+  <dimension ref="A1:J186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -23075,7 +23084,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="16" t="inlineStr">
         <is>
-          <t>Huawei eRAN LTE Spectrum Coordination Feature Parameter Description, eRAN21.1 Issue 01 (2025-03-10).  Applies to FDD/TDD (no FDD↔TDD principle difference, §2.4).  MML, counter IDs, license models, and Figure 4-1 are taken from this FPD.  Doc example uses downlink 3CC (LocalCellId=0/1/2).  Where the FPD does not print a factory default, Default = “See Parameter Reference”; Recommended = Table 4-1/4-2 setting or the MML sample.</t>
+          <t>Huawei eRAN LTE Spectrum Coordination Feature Parameter Description, eRAN21.1 Issue 01 (2025-03-10).  Applies to FDD/TDD (no FDD↔TDD principle difference, §2.4).  MML, counter IDs, license models, and Figure 4-1 are taken from this FPD.  Cell-level MML in this sheet uses LocalCellId=1 only (repeat on the partner cell in live network).  Where the FPD does not print a factory default, Default = “See Parameter Reference”; Recommended = Table 4-1/4-2 setting or the MML sample.</t>
         </is>
       </c>
       <c r="B2" s="17" t="n"/>
@@ -23462,7 +23471,7 @@
       <c r="A36" s="13" t="inlineStr">
         <is>
           <t>Worked example (sample values from the document or typical live-network settings):
-Doc MML: MOD CAMGTCFG: LocalCellId=0/1/2, SpectrumCoordSinrThld=-2;
+Doc MML (this sheet: LocalCellId=1): MOD CAMGTCFG: LocalCellId=1, SpectrumCoordSinrThld=-2;
 Sample UE at high-frequency PCell: UL SINR used in scheduling = −3 dB, threshold = −2 dB.
 Compare: −3 &lt; −2  → TRUE.
 Result: LTE Spectrum Coordination evaluation STARTS. If UL SINR = 0 dB: 0 &lt; −2 is FALSE → no SC handover from this trigger.</t>
@@ -23932,7 +23941,7 @@
     <row r="61" ht="33" customHeight="1">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=0/1/2, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;  stops UL-SINR-triggered PCell swaps. CA itself is unchanged. Doc example is the 3CC set of three cells.</t>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;  stops UL-SINR-triggered PCell swaps. CA itself is unchanged. Repeat on every participating cell in live network.</t>
         </is>
       </c>
       <c r="B61" s="19" t="n"/>
@@ -24763,7 +24772,7 @@
       </c>
       <c r="G84" s="12" t="inlineStr">
         <is>
-          <t>Doc MML: CellCaAlgoSwitch=SpectrumCoordinationSwitch-1 on LocalCellId=0,1,2 (3CC example).</t>
+          <t>Doc MML in this sheet: CellCaAlgoSwitch=SpectrumCoordinationSwitch-1 on LocalCellId=1.</t>
         </is>
       </c>
       <c r="H84" s="10" t="n"/>
@@ -24953,7 +24962,7 @@
       </c>
       <c r="G89" s="31" t="inlineStr">
         <is>
-          <t>Doc MML on LocalCellId=0,1,2.</t>
+          <t>Doc MML in this sheet: LocalCellId=1.</t>
         </is>
       </c>
       <c r="H89" s="10" t="n"/>
@@ -25343,7 +25352,7 @@
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>F.  MML  (verbatim from Ch.4.4.1.2 and Ch.5.4.1.2)</t>
+          <t>F.  MML  (from Ch.4.4.1.2 and Ch.5.4.1.2  —  LocalCellId=1 only)</t>
         </is>
       </c>
       <c r="B100" s="6" t="n"/>
@@ -25359,7 +25368,7 @@
     <row r="101" ht="28" customHeight="1">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t>Ch.4 example is downlink 3CC (LocalCellId=0,1,2; EARFCN 123/567/890). Ch.5 example: low-frequency LocalCellId=0 as MBBSERCELL, EARFCN 123 PCC + 456 SCC. Replace IDs with live-network values.</t>
+          <t>FPD sample used three cells (0/1/2). This sheet keeps one cell: LocalCellId=1. Repeat the same cell-level command on every participating high/low cell in the live network. eNodeB-level commands have no LocalCellId. EARFCN 123/567 are FPD examples — replace with live EARFCNs.</t>
         </is>
       </c>
       <c r="B101" s="17" t="n"/>
@@ -25438,12 +25447,12 @@
       </c>
       <c r="F103" s="33" t="inlineStr">
         <is>
-          <t>MOD CELLMLBHO: LocalCellId=0, MlbMatchOtherFeatureMode=HoAdmitSwitch-0;</t>
+          <t>MOD CELLMLBHO: LocalCellId=1, MlbMatchOtherFeatureMode=HoAdmitSwitch-0;</t>
         </is>
       </c>
       <c r="G103" s="12" t="inlineStr">
         <is>
-          <t>Doc: Enabling LTE spectrum coordination (taking downlink 3CC as an example). Repeat 0,1,2.</t>
+          <t>Deselect MLB unnecessary-HO admission on the cell (original PCell/SCell). Repeat on partner cell in live network.</t>
         </is>
       </c>
       <c r="H103" s="10" t="n"/>
@@ -25476,19 +25485,19 @@
       </c>
       <c r="F104" s="37" t="inlineStr">
         <is>
-          <t>MOD CELLMLBHO: LocalCellId=1, MlbMatchOtherFeatureMode=HoAdmitSwitch-0;</t>
+          <t>MOD CELLALGOSWITCH: LocalCellId=1, PucchAlgoSwitch=Dl2CCAckResShareSw-1;</t>
         </is>
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>Original PCell/SCell set.</t>
+          <t>With CaEnhancedPreAllocSwitch, prevents low-frequency cell traffic from increasing.</t>
         </is>
       </c>
       <c r="H104" s="10" t="n"/>
       <c r="I104" s="10" t="n"/>
       <c r="J104" s="11" t="n"/>
     </row>
-    <row r="105" ht="24" customHeight="1">
+    <row r="105" ht="36" customHeight="1">
       <c r="A105" s="32" t="n">
         <v>3</v>
       </c>
@@ -25514,12 +25523,12 @@
       </c>
       <c r="F105" s="33" t="inlineStr">
         <is>
-          <t>MOD CELLMLBHO: LocalCellId=2, MlbMatchOtherFeatureMode=HoAdmitSwitch-0;</t>
+          <t>MOD ENODEBALGOSWITCH: CaAlgoSwitch=HoWithSccCfgSwitch-1&amp;SccA2RmvSwitch-1, CaAlgoExtSwitch=CaEnhancedPreAllocSwitch-1;</t>
         </is>
       </c>
       <c r="G105" s="12" t="inlineStr">
         <is>
-          <t>Original PCell/SCell set.</t>
+          <t>eNodeB-level (no LocalCellId): SCell-during-HO + A2 remove + enhanced pre-alloc.</t>
         </is>
       </c>
       <c r="H105" s="10" t="n"/>
@@ -25552,12 +25561,12 @@
       </c>
       <c r="F106" s="37" t="inlineStr">
         <is>
-          <t>MOD CELLALGOSWITCH: LocalCellId=0, PucchAlgoSwitch=Dl2CCAckResShareSw-1;</t>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
         </is>
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>Prevents low-frequency traffic increase (with CaEnhancedPreAllocSwitch).</t>
+          <t>Master switch. Repeat on every participating cell.</t>
         </is>
       </c>
       <c r="H106" s="10" t="n"/>
@@ -25585,15 +25594,19 @@
       </c>
       <c r="E107" s="12" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Optimize SC</t>
         </is>
       </c>
       <c r="F107" s="33" t="inlineStr">
         <is>
-          <t>MOD CELLALGOSWITCH: LocalCellId=1, PucchAlgoSwitch=Dl2CCAckResShareSw-1;</t>
-        </is>
-      </c>
-      <c r="G107" s="12" t="inlineStr"/>
+          <t>MOD CAMGTCFG: LocalCellId=1, SpectrumCoordSinrThld=-2;</t>
+        </is>
+      </c>
+      <c r="G107" s="12" t="inlineStr">
+        <is>
+          <t>Doc recommended SINR threshold on original PCells.</t>
+        </is>
+      </c>
       <c r="H107" s="10" t="n"/>
       <c r="I107" s="10" t="n"/>
       <c r="J107" s="11" t="n"/>
@@ -25609,7 +25622,7 @@
       </c>
       <c r="C108" s="9" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
@@ -25619,20 +25632,24 @@
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Optimize SC</t>
         </is>
       </c>
       <c r="F108" s="37" t="inlineStr">
         <is>
-          <t>MOD CELLALGOSWITCH: LocalCellId=2, PucchAlgoSwitch=Dl2CCAckResShareSw-1;</t>
-        </is>
-      </c>
-      <c r="G108" s="9" t="inlineStr"/>
+          <t>MOD SCCFREQCFG: PccDlEarfcn=123, SccDlEarfcn=567, SccA2RsrpThldExtendedOfs=-10;</t>
+        </is>
+      </c>
+      <c r="G108" s="9" t="inlineStr">
+        <is>
+          <t>Doc A2 extended offset. One PCC↔SCC pair shown; apply to each live pair.</t>
+        </is>
+      </c>
       <c r="H108" s="10" t="n"/>
       <c r="I108" s="10" t="n"/>
       <c r="J108" s="11" t="n"/>
     </row>
-    <row r="109" ht="36" customHeight="1">
+    <row r="109" ht="24" customHeight="1">
       <c r="A109" s="32" t="n">
         <v>7</v>
       </c>
@@ -25653,17 +25670,17 @@
       </c>
       <c r="E109" s="12" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Deactivate SC</t>
         </is>
       </c>
       <c r="F109" s="33" t="inlineStr">
         <is>
-          <t>MOD ENODEBALGOSWITCH: CaAlgoSwitch=HoWithSccCfgSwitch-1&amp;SccA2RmvSwitch-1, CaAlgoExtSwitch=CaEnhancedPreAllocSwitch-1;</t>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;</t>
         </is>
       </c>
       <c r="G109" s="12" t="inlineStr">
         <is>
-          <t>Doc single eNodeB-level command (HO-with-SCell + A2 remove + enhanced pre-alloc).</t>
+          <t>Stops UL-SINR PCell swaps. CA stays as configured.</t>
         </is>
       </c>
       <c r="H109" s="10" t="n"/>
@@ -25691,17 +25708,17 @@
       </c>
       <c r="E110" s="9" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Activate enhancement</t>
         </is>
       </c>
       <c r="F110" s="37" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
+          <t>MOD ENODEBALGOSWITCH: CaAlgoSwitch=HoWithSccCfgSwitch-1;</t>
         </is>
       </c>
       <c r="G110" s="9" t="inlineStr">
         <is>
-          <t>Master bit on each of the three cells.</t>
+          <t>Ch.5 WBB/RRN enhancement. eNodeB-level.</t>
         </is>
       </c>
       <c r="H110" s="10" t="n"/>
@@ -25729,15 +25746,19 @@
       </c>
       <c r="E111" s="12" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Activate enhancement</t>
         </is>
       </c>
       <c r="F111" s="33" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
-        </is>
-      </c>
-      <c r="G111" s="12" t="inlineStr"/>
+          <t>MOD CELL: LocalCellId=1, SpecifiedCellFlag=MBBSERCELL;</t>
+        </is>
+      </c>
+      <c r="G111" s="12" t="inlineStr">
+        <is>
+          <t>Mark the low-frequency cell as MBB service cell.</t>
+        </is>
+      </c>
       <c r="H111" s="10" t="n"/>
       <c r="I111" s="10" t="n"/>
       <c r="J111" s="11" t="n"/>
@@ -25763,15 +25784,19 @@
       </c>
       <c r="E112" s="9" t="inlineStr">
         <is>
-          <t>Activate SC</t>
+          <t>Activate enhancement</t>
         </is>
       </c>
       <c r="F112" s="37" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=2, CellCaAlgoSwitch=SpectrumCoordinationSwitch-1;</t>
-        </is>
-      </c>
-      <c r="G112" s="9" t="inlineStr"/>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-1;</t>
+        </is>
+      </c>
+      <c r="G112" s="9" t="inlineStr">
+        <is>
+          <t>Enhancement bit on the participating cell.</t>
+        </is>
+      </c>
       <c r="H112" s="10" t="n"/>
       <c r="I112" s="10" t="n"/>
       <c r="J112" s="11" t="n"/>
@@ -25797,17 +25822,17 @@
       </c>
       <c r="E113" s="12" t="inlineStr">
         <is>
-          <t>Optimize SC</t>
+          <t>Optimize enhancement</t>
         </is>
       </c>
       <c r="F113" s="33" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=0, SpectrumCoordSinrThld=-2;</t>
+          <t>MOD CELLWTTXPARACFG: LocalCellId=1, WbbMultiCarrierCoordA2Ofs=2;</t>
         </is>
       </c>
       <c r="G113" s="12" t="inlineStr">
         <is>
-          <t>Doc: Setting the SINR threshold (3CC example). Repeat 0,1,2.</t>
+          <t>Doc WBB A2 offset (low-frequency cells).</t>
         </is>
       </c>
       <c r="H113" s="10" t="n"/>
@@ -25825,7 +25850,7 @@
       </c>
       <c r="C114" s="9" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Adaptive</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
@@ -25835,15 +25860,19 @@
       </c>
       <c r="E114" s="9" t="inlineStr">
         <is>
-          <t>Optimize SC</t>
+          <t>Optimize enhancement</t>
         </is>
       </c>
       <c r="F114" s="37" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=1, SpectrumCoordSinrThld=-2;</t>
-        </is>
-      </c>
-      <c r="G114" s="9" t="inlineStr"/>
+          <t>MOD SCCFREQCFG: PccDlEarfcn=123, SccDlEarfcn=456, SccA2RsrpThldExtendedOfs=-10;</t>
+        </is>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>Doc: low-freq PCC 123 + high-freq WBB SCC 456.</t>
+        </is>
+      </c>
       <c r="H114" s="10" t="n"/>
       <c r="I114" s="10" t="n"/>
       <c r="J114" s="11" t="n"/>
@@ -25869,733 +25898,633 @@
       </c>
       <c r="E115" s="12" t="inlineStr">
         <is>
-          <t>Optimize SC</t>
+          <t>Deactivate enhancement</t>
         </is>
       </c>
       <c r="F115" s="33" t="inlineStr">
         <is>
-          <t>MOD CAMGTCFG: LocalCellId=2, SpectrumCoordSinrThld=-2;</t>
-        </is>
-      </c>
-      <c r="G115" s="12" t="inlineStr"/>
+          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-0;</t>
+        </is>
+      </c>
+      <c r="G115" s="12" t="inlineStr">
+        <is>
+          <t>Turns off WBB/RRN enhancement only.</t>
+        </is>
+      </c>
       <c r="H115" s="10" t="n"/>
       <c r="I115" s="10" t="n"/>
       <c r="J115" s="11" t="n"/>
     </row>
-    <row r="116" ht="24" customHeight="1">
-      <c r="A116" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="B116" s="36" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C116" s="9" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D116" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E116" s="9" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F116" s="37" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=123, SccDlEarfcn=567, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G116" s="9" t="inlineStr">
-        <is>
-          <t>Doc: extended A2 offset on every PCC↔SCC pair of {123,567,890}.</t>
-        </is>
-      </c>
-      <c r="H116" s="10" t="n"/>
-      <c r="I116" s="10" t="n"/>
-      <c r="J116" s="11" t="n"/>
-    </row>
-    <row r="117" ht="24" customHeight="1">
-      <c r="A117" s="32" t="n">
-        <v>15</v>
-      </c>
-      <c r="B117" s="32" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="C117" s="12" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D117" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E117" s="12" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F117" s="33" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=123, SccDlEarfcn=890, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G117" s="12" t="inlineStr"/>
-      <c r="H117" s="10" t="n"/>
-      <c r="I117" s="10" t="n"/>
-      <c r="J117" s="11" t="n"/>
-    </row>
-    <row r="118" ht="24" customHeight="1">
-      <c r="A118" s="36" t="n">
-        <v>16</v>
-      </c>
-      <c r="B118" s="36" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C118" s="9" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D118" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E118" s="9" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F118" s="37" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=567, SccDlEarfcn=123, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G118" s="9" t="inlineStr"/>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>G.  Counters  (Tables 4-3, 4-4, 5-4–5-8, 5.4.2)</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="n"/>
+      <c r="D116" s="6" t="n"/>
+      <c r="E116" s="6" t="n"/>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="H116" s="6" t="n"/>
+      <c r="I116" s="6" t="n"/>
+      <c r="J116" s="6" t="n"/>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>Counter ID</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t>Counter Name</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>Function / what it measures</t>
+        </is>
+      </c>
+      <c r="E117" s="7" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+      <c r="F117" s="7" t="inlineStr"/>
+      <c r="G117" s="7" t="inlineStr"/>
+      <c r="H117" s="7" t="inlineStr"/>
+      <c r="I117" s="7" t="inlineStr"/>
+      <c r="J117" s="7" t="inlineStr"/>
+    </row>
+    <row r="118" ht="32" customHeight="1">
+      <c r="A118" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B118" s="12" t="inlineStr">
+        <is>
+          <t>1526729994</t>
+        </is>
+      </c>
+      <c r="C118" s="33" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.PrepAttOut</t>
+        </is>
+      </c>
+      <c r="D118" s="12" t="inlineStr">
+        <is>
+          <t>UL-quality inter-freq HO preparations</t>
+        </is>
+      </c>
+      <c r="E118" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-3 activation: values increase ⇒ SC has taken effect</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="n"/>
+      <c r="G118" s="10" t="n"/>
       <c r="H118" s="10" t="n"/>
       <c r="I118" s="10" t="n"/>
       <c r="J118" s="11" t="n"/>
     </row>
-    <row r="119" ht="24" customHeight="1">
-      <c r="A119" s="32" t="n">
-        <v>17</v>
-      </c>
-      <c r="B119" s="32" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="C119" s="12" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D119" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E119" s="12" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F119" s="33" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=567, SccDlEarfcn=890, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G119" s="12" t="inlineStr"/>
+    <row r="119" ht="32" customHeight="1">
+      <c r="A119" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>1526729996</t>
+        </is>
+      </c>
+      <c r="C119" s="37" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.ExecAttOut</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>UL-quality inter-freq HO executions</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-3</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="n"/>
+      <c r="G119" s="10" t="n"/>
       <c r="H119" s="10" t="n"/>
       <c r="I119" s="10" t="n"/>
       <c r="J119" s="11" t="n"/>
     </row>
-    <row r="120" ht="24" customHeight="1">
-      <c r="A120" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="B120" s="36" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="C120" s="9" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D120" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E120" s="9" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F120" s="37" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=890, SccDlEarfcn=123, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G120" s="9" t="inlineStr"/>
+    <row r="120" ht="32" customHeight="1">
+      <c r="A120" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B120" s="12" t="inlineStr">
+        <is>
+          <t>1526729998</t>
+        </is>
+      </c>
+      <c r="C120" s="33" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.ExecSuccOut</t>
+        </is>
+      </c>
+      <c r="D120" s="12" t="inlineStr">
+        <is>
+          <t>UL-quality inter-freq HO success</t>
+        </is>
+      </c>
+      <c r="E120" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-3; success rate KPI</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="n"/>
+      <c r="G120" s="10" t="n"/>
       <c r="H120" s="10" t="n"/>
       <c r="I120" s="10" t="n"/>
       <c r="J120" s="11" t="n"/>
     </row>
-    <row r="121" ht="24" customHeight="1">
-      <c r="A121" s="32" t="n">
-        <v>19</v>
-      </c>
-      <c r="B121" s="32" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C121" s="12" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D121" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E121" s="12" t="inlineStr">
-        <is>
-          <t>Optimize SC</t>
-        </is>
-      </c>
-      <c r="F121" s="33" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=890, SccDlEarfcn=567, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G121" s="12" t="inlineStr"/>
+    <row r="121" ht="32" customHeight="1">
+      <c r="A121" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>1526729995</t>
+        </is>
+      </c>
+      <c r="C121" s="37" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFddTdd.ULquality.PrepAttOut</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>UL-quality FDD↔TDD HO preparations</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-3</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="n"/>
+      <c r="G121" s="10" t="n"/>
       <c r="H121" s="10" t="n"/>
       <c r="I121" s="10" t="n"/>
       <c r="J121" s="11" t="n"/>
     </row>
-    <row r="122" ht="24" customHeight="1">
-      <c r="A122" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="B122" s="36" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C122" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D122" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E122" s="9" t="inlineStr">
-        <is>
-          <t>Deactivate SC</t>
-        </is>
-      </c>
-      <c r="F122" s="37" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;</t>
-        </is>
-      </c>
-      <c r="G122" s="9" t="inlineStr">
-        <is>
-          <t>Doc deactivation (3CC). Repeat 1 and 2.</t>
-        </is>
-      </c>
+    <row r="122" ht="32" customHeight="1">
+      <c r="A122" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B122" s="12" t="inlineStr">
+        <is>
+          <t>1526729997</t>
+        </is>
+      </c>
+      <c r="C122" s="33" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFddTdd.ULquality.ExecAttOut</t>
+        </is>
+      </c>
+      <c r="D122" s="12" t="inlineStr">
+        <is>
+          <t>UL-quality FDD↔TDD HO executions</t>
+        </is>
+      </c>
+      <c r="E122" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-3</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="n"/>
+      <c r="G122" s="10" t="n"/>
       <c r="H122" s="10" t="n"/>
       <c r="I122" s="10" t="n"/>
       <c r="J122" s="11" t="n"/>
     </row>
-    <row r="123" ht="24" customHeight="1">
-      <c r="A123" s="32" t="n">
-        <v>21</v>
-      </c>
-      <c r="B123" s="32" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="C123" s="12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D123" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E123" s="12" t="inlineStr">
-        <is>
-          <t>Deactivate SC</t>
-        </is>
-      </c>
-      <c r="F123" s="33" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;</t>
-        </is>
-      </c>
-      <c r="G123" s="12" t="inlineStr"/>
+    <row r="123" ht="32" customHeight="1">
+      <c r="A123" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>1526729999</t>
+        </is>
+      </c>
+      <c r="C123" s="37" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFddTdd.ULquality.ExecSuccOut</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>UL-quality FDD↔TDD HO success</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-3</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="n"/>
+      <c r="G123" s="10" t="n"/>
       <c r="H123" s="10" t="n"/>
       <c r="I123" s="10" t="n"/>
       <c r="J123" s="11" t="n"/>
     </row>
-    <row r="124" ht="24" customHeight="1">
-      <c r="A124" s="36" t="n">
-        <v>22</v>
-      </c>
-      <c r="B124" s="36" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="C124" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D124" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E124" s="9" t="inlineStr">
-        <is>
-          <t>Deactivate SC</t>
-        </is>
-      </c>
-      <c r="F124" s="37" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=2, CellCaAlgoSwitch=SpectrumCoordinationSwitch-0;</t>
-        </is>
-      </c>
-      <c r="G124" s="9" t="inlineStr"/>
+    <row r="124" ht="32" customHeight="1">
+      <c r="A124" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B124" s="12" t="inlineStr">
+        <is>
+          <t>1526728426</t>
+        </is>
+      </c>
+      <c r="C124" s="33" t="inlineStr">
+        <is>
+          <t>L.Traffic.User.PCell.DL.Avg</t>
+        </is>
+      </c>
+      <c r="D124" s="12" t="inlineStr">
+        <is>
+          <t>Avg CA UEs using this cell as PCell</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8; Ch.4.2.2 says this moves after PCell swap</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="n"/>
+      <c r="G124" s="10" t="n"/>
       <c r="H124" s="10" t="n"/>
       <c r="I124" s="10" t="n"/>
       <c r="J124" s="11" t="n"/>
     </row>
-    <row r="125" ht="24" customHeight="1">
-      <c r="A125" s="32" t="n">
-        <v>23</v>
-      </c>
-      <c r="B125" s="32" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="C125" s="12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D125" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E125" s="12" t="inlineStr">
-        <is>
-          <t>Activate enhancement</t>
-        </is>
-      </c>
-      <c r="F125" s="33" t="inlineStr">
-        <is>
-          <t>MOD ENODEBALGOSWITCH: CaAlgoSwitch=HoWithSccCfgSwitch-1;</t>
-        </is>
-      </c>
-      <c r="G125" s="12" t="inlineStr">
-        <is>
-          <t>Ch.5.4.1.2 Activating LTE spectrum coordination enhancement.</t>
-        </is>
-      </c>
+    <row r="125" ht="32" customHeight="1">
+      <c r="A125" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>1526728427</t>
+        </is>
+      </c>
+      <c r="C125" s="37" t="inlineStr">
+        <is>
+          <t>L.Traffic.User.SCell.DL.Avg</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>Avg CA UEs using this cell as SCell</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="n"/>
+      <c r="G125" s="10" t="n"/>
       <c r="H125" s="10" t="n"/>
       <c r="I125" s="10" t="n"/>
       <c r="J125" s="11" t="n"/>
     </row>
-    <row r="126" ht="24" customHeight="1">
-      <c r="A126" s="36" t="n">
-        <v>24</v>
-      </c>
-      <c r="B126" s="36" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="C126" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D126" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E126" s="9" t="inlineStr">
-        <is>
-          <t>Activate enhancement</t>
-        </is>
-      </c>
-      <c r="F126" s="37" t="inlineStr">
-        <is>
-          <t>MOD CELL: LocalCellId=0, SpecifiedCellFlag=MBBSERCELL;</t>
-        </is>
-      </c>
-      <c r="G126" s="9" t="inlineStr">
-        <is>
-          <t>Low-frequency cell as MBB service cell.</t>
-        </is>
-      </c>
+    <row r="126" ht="32" customHeight="1">
+      <c r="A126" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B126" s="12" t="inlineStr">
+        <is>
+          <t>1526732658</t>
+        </is>
+      </c>
+      <c r="C126" s="33" t="inlineStr">
+        <is>
+          <t>L.CA.Traffic.bits.DL.PCell</t>
+        </is>
+      </c>
+      <c r="D126" s="12" t="inlineStr">
+        <is>
+          <t>DL bits on PCell of CA UEs</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8</t>
+        </is>
+      </c>
+      <c r="F126" s="10" t="n"/>
+      <c r="G126" s="10" t="n"/>
       <c r="H126" s="10" t="n"/>
       <c r="I126" s="10" t="n"/>
       <c r="J126" s="11" t="n"/>
     </row>
-    <row r="127" ht="24" customHeight="1">
-      <c r="A127" s="32" t="n">
-        <v>25</v>
-      </c>
-      <c r="B127" s="32" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C127" s="12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D127" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E127" s="12" t="inlineStr">
-        <is>
-          <t>Activate enhancement</t>
-        </is>
-      </c>
-      <c r="F127" s="33" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-1;</t>
-        </is>
-      </c>
-      <c r="G127" s="12" t="inlineStr">
-        <is>
-          <t>Low- and high-frequency cells (doc 0 and 1).</t>
-        </is>
-      </c>
+    <row r="127" ht="32" customHeight="1">
+      <c r="A127" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>1526729259</t>
+        </is>
+      </c>
+      <c r="C127" s="37" t="inlineStr">
+        <is>
+          <t>L.CA.Traffic.bits.DL.SCell</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>DL bits on SCell of CA UEs</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8</t>
+        </is>
+      </c>
+      <c r="F127" s="10" t="n"/>
+      <c r="G127" s="10" t="n"/>
       <c r="H127" s="10" t="n"/>
       <c r="I127" s="10" t="n"/>
       <c r="J127" s="11" t="n"/>
     </row>
-    <row r="128" ht="24" customHeight="1">
-      <c r="A128" s="36" t="n">
-        <v>26</v>
-      </c>
-      <c r="B128" s="36" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="C128" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D128" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E128" s="9" t="inlineStr">
-        <is>
-          <t>Activate enhancement</t>
-        </is>
-      </c>
-      <c r="F128" s="37" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-1;</t>
-        </is>
-      </c>
-      <c r="G128" s="9" t="inlineStr"/>
+    <row r="128" ht="32" customHeight="1">
+      <c r="A128" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t>1526728564</t>
+        </is>
+      </c>
+      <c r="C128" s="33" t="inlineStr">
+        <is>
+          <t>L.Thrp.bits.DL.CAUser</t>
+        </is>
+      </c>
+      <c r="D128" s="12" t="inlineStr">
+        <is>
+          <t>CA UE DL bits</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-5 / 5-8; CA UE rate KPI</t>
+        </is>
+      </c>
+      <c r="F128" s="10" t="n"/>
+      <c r="G128" s="10" t="n"/>
       <c r="H128" s="10" t="n"/>
       <c r="I128" s="10" t="n"/>
       <c r="J128" s="11" t="n"/>
     </row>
-    <row r="129" ht="24" customHeight="1">
-      <c r="A129" s="32" t="n">
-        <v>27</v>
-      </c>
-      <c r="B129" s="32" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="C129" s="12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D129" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E129" s="12" t="inlineStr">
-        <is>
-          <t>Optimize enhancement</t>
-        </is>
-      </c>
-      <c r="F129" s="33" t="inlineStr">
-        <is>
-          <t>MOD CELLWTTXPARACFG: LocalCellId=0, WbbMultiCarrierCoordA2Ofs=2;</t>
-        </is>
-      </c>
-      <c r="G129" s="12" t="inlineStr">
-        <is>
-          <t>Doc: Setting WbbMultiCarrierCoordA2Ofs (repeat 0,1).</t>
-        </is>
-      </c>
+    <row r="129" ht="32" customHeight="1">
+      <c r="A129" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>1526740440</t>
+        </is>
+      </c>
+      <c r="C129" s="37" t="inlineStr">
+        <is>
+          <t>L.Thrp.bits.DL.LastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>CA UE last-TTI DL bits</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-5</t>
+        </is>
+      </c>
+      <c r="F129" s="10" t="n"/>
+      <c r="G129" s="10" t="n"/>
       <c r="H129" s="10" t="n"/>
       <c r="I129" s="10" t="n"/>
       <c r="J129" s="11" t="n"/>
     </row>
-    <row r="130" ht="24" customHeight="1">
-      <c r="A130" s="36" t="n">
-        <v>28</v>
-      </c>
-      <c r="B130" s="36" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="C130" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D130" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E130" s="9" t="inlineStr">
-        <is>
-          <t>Optimize enhancement</t>
-        </is>
-      </c>
-      <c r="F130" s="37" t="inlineStr">
-        <is>
-          <t>MOD CELLWTTXPARACFG: LocalCellId=1, WbbMultiCarrierCoordA2Ofs=2;</t>
-        </is>
-      </c>
-      <c r="G130" s="9" t="inlineStr"/>
+    <row r="130" ht="32" customHeight="1">
+      <c r="A130" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t>1526740441</t>
+        </is>
+      </c>
+      <c r="C130" s="33" t="inlineStr">
+        <is>
+          <t>L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D130" s="12" t="inlineStr">
+        <is>
+          <t>CA UE DL time last-TTI removed</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-5</t>
+        </is>
+      </c>
+      <c r="F130" s="10" t="n"/>
+      <c r="G130" s="10" t="n"/>
       <c r="H130" s="10" t="n"/>
       <c r="I130" s="10" t="n"/>
       <c r="J130" s="11" t="n"/>
     </row>
-    <row r="131" ht="24" customHeight="1">
-      <c r="A131" s="32" t="n">
-        <v>29</v>
-      </c>
-      <c r="B131" s="32" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="C131" s="12" t="inlineStr">
-        <is>
-          <t>Adaptive</t>
-        </is>
-      </c>
-      <c r="D131" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E131" s="12" t="inlineStr">
-        <is>
-          <t>Optimize enhancement</t>
-        </is>
-      </c>
-      <c r="F131" s="33" t="inlineStr">
-        <is>
-          <t>MOD SCCFREQCFG: PccDlEarfcn=123, SccDlEarfcn=456, SccA2RsrpThldExtendedOfs=-10;</t>
-        </is>
-      </c>
-      <c r="G131" s="12" t="inlineStr">
-        <is>
-          <t>Doc: low-frequency PCC EARFCN 123, high-frequency WBB SCC EARFCN 456.</t>
-        </is>
-      </c>
+    <row r="131" ht="32" customHeight="1">
+      <c r="A131" s="36" t="n">
+        <v>14</v>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>1526729045</t>
+        </is>
+      </c>
+      <c r="C131" s="37" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Add.Att</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>DL SCell add attempts</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8; SCell cfg success vs HO</t>
+        </is>
+      </c>
+      <c r="F131" s="10" t="n"/>
+      <c r="G131" s="10" t="n"/>
       <c r="H131" s="10" t="n"/>
       <c r="I131" s="10" t="n"/>
       <c r="J131" s="11" t="n"/>
     </row>
-    <row r="132" ht="24" customHeight="1">
-      <c r="A132" s="36" t="n">
-        <v>30</v>
-      </c>
-      <c r="B132" s="36" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="C132" s="9" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D132" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E132" s="9" t="inlineStr">
-        <is>
-          <t>Deactivate enhancement</t>
-        </is>
-      </c>
-      <c r="F132" s="37" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=0, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-0;</t>
-        </is>
-      </c>
-      <c r="G132" s="9" t="inlineStr">
-        <is>
-          <t>Doc deactivation. Repeat LocalCellId=1.</t>
-        </is>
-      </c>
+    <row r="132" ht="32" customHeight="1">
+      <c r="A132" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t>1526729046</t>
+        </is>
+      </c>
+      <c r="C132" s="33" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Add.Succ</t>
+        </is>
+      </c>
+      <c r="D132" s="12" t="inlineStr">
+        <is>
+          <t>DL SCell add success</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-4 / 5-8</t>
+        </is>
+      </c>
+      <c r="F132" s="10" t="n"/>
+      <c r="G132" s="10" t="n"/>
       <c r="H132" s="10" t="n"/>
       <c r="I132" s="10" t="n"/>
       <c r="J132" s="11" t="n"/>
     </row>
-    <row r="133" ht="24" customHeight="1">
-      <c r="A133" s="32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B133" s="32" t="inlineStr">
-        <is>
-          <t>31</t>
-        </is>
-      </c>
-      <c r="C133" s="12" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="D133" s="12" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="E133" s="12" t="inlineStr">
-        <is>
-          <t>Deactivate enhancement</t>
-        </is>
-      </c>
-      <c r="F133" s="33" t="inlineStr">
-        <is>
-          <t>MOD CAMGTCFG: LocalCellId=1, CellCaAlgoSwitch=WbbCaMultiCarrierCoordSw-0;</t>
-        </is>
-      </c>
-      <c r="G133" s="12" t="inlineStr"/>
+    <row r="133" ht="32" customHeight="1">
+      <c r="A133" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>1526746999–7008</t>
+        </is>
+      </c>
+      <c r="C133" s="37" t="inlineStr">
+        <is>
+          <t>L.Thrp.DL.BitRate.Samp.CaUe.Index0 … Index9</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>CA UE DL bit-rate samples (10 bins)</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Table 4-4 monitoring</t>
+        </is>
+      </c>
+      <c r="F133" s="10" t="n"/>
+      <c r="G133" s="10" t="n"/>
       <c r="H133" s="10" t="n"/>
       <c r="I133" s="10" t="n"/>
       <c r="J133" s="11" t="n"/>
     </row>
-    <row r="134" ht="22" customHeight="1">
-      <c r="A134" s="5" t="inlineStr">
-        <is>
-          <t>G.  Counters  (Tables 4-3, 4-4, 5-4–5-8, 5.4.2)</t>
-        </is>
-      </c>
-      <c r="B134" s="6" t="n"/>
-      <c r="C134" s="6" t="n"/>
-      <c r="D134" s="6" t="n"/>
-      <c r="E134" s="6" t="n"/>
-      <c r="F134" s="6" t="n"/>
-      <c r="G134" s="6" t="n"/>
-      <c r="H134" s="6" t="n"/>
-      <c r="I134" s="6" t="n"/>
-      <c r="J134" s="6" t="n"/>
-    </row>
-    <row r="135" ht="22" customHeight="1">
-      <c r="A135" s="7" t="inlineStr">
-        <is>
-          <t>SN</t>
-        </is>
-      </c>
-      <c r="B135" s="7" t="inlineStr">
-        <is>
-          <t>Counter ID</t>
-        </is>
-      </c>
-      <c r="C135" s="7" t="inlineStr">
-        <is>
-          <t>Counter Name</t>
-        </is>
-      </c>
-      <c r="D135" s="7" t="inlineStr">
-        <is>
-          <t>Function / what it measures</t>
-        </is>
-      </c>
-      <c r="E135" s="7" t="inlineStr">
-        <is>
-          <t>Use</t>
-        </is>
-      </c>
-      <c r="F135" s="7" t="inlineStr"/>
-      <c r="G135" s="7" t="inlineStr"/>
-      <c r="H135" s="7" t="inlineStr"/>
-      <c r="I135" s="7" t="inlineStr"/>
-      <c r="J135" s="7" t="inlineStr"/>
+    <row r="134" ht="32" customHeight="1">
+      <c r="A134" s="32" t="n">
+        <v>17</v>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t>1526728261</t>
+        </is>
+      </c>
+      <c r="C134" s="33" t="inlineStr">
+        <is>
+          <t>L.Thrp.bits.DL</t>
+        </is>
+      </c>
+      <c r="D134" s="12" t="inlineStr">
+        <is>
+          <t>All-UE DL bits</t>
+        </is>
+      </c>
+      <c r="E134" s="12" t="inlineStr">
+        <is>
+          <t>Table 5-4 MBB perceived rate</t>
+        </is>
+      </c>
+      <c r="F134" s="10" t="n"/>
+      <c r="G134" s="10" t="n"/>
+      <c r="H134" s="10" t="n"/>
+      <c r="I134" s="10" t="n"/>
+      <c r="J134" s="11" t="n"/>
+    </row>
+    <row r="135" ht="32" customHeight="1">
+      <c r="A135" s="36" t="n">
+        <v>18</v>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>1526729005</t>
+        </is>
+      </c>
+      <c r="C135" s="37" t="inlineStr">
+        <is>
+          <t>L.Thrp.bits.DL.LastTTI</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>All-UE last-TTI DL bits</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Table 5-4</t>
+        </is>
+      </c>
+      <c r="F135" s="10" t="n"/>
+      <c r="G135" s="10" t="n"/>
+      <c r="H135" s="10" t="n"/>
+      <c r="I135" s="10" t="n"/>
+      <c r="J135" s="11" t="n"/>
     </row>
     <row r="136" ht="32" customHeight="1">
       <c r="A136" s="32" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="B136" s="12" t="inlineStr">
         <is>
-          <t>1526729994</t>
+          <t>1526745879</t>
         </is>
       </c>
       <c r="C136" s="33" t="inlineStr">
         <is>
-          <t>L.HHO.InterFreq.ULquality.PrepAttOut</t>
+          <t>L.Thrp.bits.DL.WBB</t>
         </is>
       </c>
       <c r="D136" s="12" t="inlineStr">
         <is>
-          <t>UL-quality inter-freq HO preparations</t>
+          <t>WBB DL bits</t>
         </is>
       </c>
       <c r="E136" s="12" t="inlineStr">
         <is>
-          <t>Table 4-3 activation: values increase ⇒ SC has taken effect</t>
+          <t>Tables 5-4 / 5-6</t>
         </is>
       </c>
       <c r="F136" s="10" t="n"/>
@@ -26606,26 +26535,26 @@
     </row>
     <row r="137" ht="32" customHeight="1">
       <c r="A137" s="36" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B137" s="9" t="inlineStr">
         <is>
-          <t>1526729996</t>
+          <t>1526745880</t>
         </is>
       </c>
       <c r="C137" s="37" t="inlineStr">
         <is>
-          <t>L.HHO.InterFreq.ULquality.ExecAttOut</t>
+          <t>L.Thrp.bits.DL.LastTTI.WBB</t>
         </is>
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>UL-quality inter-freq HO executions</t>
+          <t>WBB last-TTI DL bits</t>
         </is>
       </c>
       <c r="E137" s="9" t="inlineStr">
         <is>
-          <t>Table 4-3</t>
+          <t>Tables 5-4 / 5-6</t>
         </is>
       </c>
       <c r="F137" s="10" t="n"/>
@@ -26636,26 +26565,26 @@
     </row>
     <row r="138" ht="32" customHeight="1">
       <c r="A138" s="32" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t>1526729998</t>
+          <t>1526729015</t>
         </is>
       </c>
       <c r="C138" s="33" t="inlineStr">
         <is>
-          <t>L.HHO.InterFreq.ULquality.ExecSuccOut</t>
+          <t>L.Thrp.Time.DL.RmvLastTTI</t>
         </is>
       </c>
       <c r="D138" s="12" t="inlineStr">
         <is>
-          <t>UL-quality inter-freq HO success</t>
+          <t>All-UE DL time last-TTI removed</t>
         </is>
       </c>
       <c r="E138" s="12" t="inlineStr">
         <is>
-          <t>Table 4-3; success rate KPI</t>
+          <t>Table 5-4</t>
         </is>
       </c>
       <c r="F138" s="10" t="n"/>
@@ -26666,26 +26595,26 @@
     </row>
     <row r="139" ht="32" customHeight="1">
       <c r="A139" s="36" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B139" s="9" t="inlineStr">
         <is>
-          <t>1526729995</t>
+          <t>1526745881</t>
         </is>
       </c>
       <c r="C139" s="37" t="inlineStr">
         <is>
-          <t>L.HHO.InterFddTdd.ULquality.PrepAttOut</t>
+          <t>L.Thrp.Time.DL.RmvLastTTI.WBB</t>
         </is>
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>UL-quality FDD↔TDD HO preparations</t>
+          <t>WBB DL time last-TTI removed</t>
         </is>
       </c>
       <c r="E139" s="9" t="inlineStr">
         <is>
-          <t>Table 4-3</t>
+          <t>Tables 5-4 / 5-6; Ch.5.2.2 may increase</t>
         </is>
       </c>
       <c r="F139" s="10" t="n"/>
@@ -26696,26 +26625,26 @@
     </row>
     <row r="140" ht="32" customHeight="1">
       <c r="A140" s="32" t="n">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B140" s="12" t="inlineStr">
         <is>
-          <t>1526729997</t>
+          <t>1526735542</t>
         </is>
       </c>
       <c r="C140" s="33" t="inlineStr">
         <is>
-          <t>L.HHO.InterFddTdd.ULquality.ExecAttOut</t>
+          <t>L.Thrp.Relay.bits.DL</t>
         </is>
       </c>
       <c r="D140" s="12" t="inlineStr">
         <is>
-          <t>UL-quality FDD↔TDD HO executions</t>
+          <t>RRN DL bits</t>
         </is>
       </c>
       <c r="E140" s="12" t="inlineStr">
         <is>
-          <t>Table 4-3</t>
+          <t>Table 5-7</t>
         </is>
       </c>
       <c r="F140" s="10" t="n"/>
@@ -26726,26 +26655,26 @@
     </row>
     <row r="141" ht="32" customHeight="1">
       <c r="A141" s="36" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B141" s="9" t="inlineStr">
         <is>
-          <t>1526729999</t>
+          <t>1526735543</t>
         </is>
       </c>
       <c r="C141" s="37" t="inlineStr">
         <is>
-          <t>L.HHO.InterFddTdd.ULquality.ExecSuccOut</t>
+          <t>L.Thrp.Relay.Time.DL</t>
         </is>
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>UL-quality FDD↔TDD HO success</t>
+          <t>RRN DL time</t>
         </is>
       </c>
       <c r="E141" s="9" t="inlineStr">
         <is>
-          <t>Table 4-3</t>
+          <t>Table 5-7; Ch.5.4.2: increase on low-freq cells ⇒ RRN enhancement took effect</t>
         </is>
       </c>
       <c r="F141" s="10" t="n"/>
@@ -26756,26 +26685,26 @@
     </row>
     <row r="142" ht="32" customHeight="1">
       <c r="A142" s="32" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="B142" s="12" t="inlineStr">
         <is>
-          <t>1526728426</t>
+          <t>1526745954</t>
         </is>
       </c>
       <c r="C142" s="33" t="inlineStr">
         <is>
-          <t>L.Traffic.User.PCell.DL.Avg</t>
+          <t>L.ChMeas.PRB.DL.PDSCH.WBBUsed.Avg</t>
         </is>
       </c>
       <c r="D142" s="12" t="inlineStr">
         <is>
-          <t>Avg CA UEs using this cell as PCell</t>
+          <t>Avg PDSCH PRBs used by WBB</t>
         </is>
       </c>
       <c r="E142" s="12" t="inlineStr">
         <is>
-          <t>Table 4-4 / 5-8; Ch.4.2.2 says this moves after PCell swap</t>
+          <t>Ch.5.2.2: decreases on low-freq, increases on high-freq</t>
         </is>
       </c>
       <c r="F142" s="10" t="n"/>
@@ -26786,26 +26715,26 @@
     </row>
     <row r="143" ht="32" customHeight="1">
       <c r="A143" s="36" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="B143" s="9" t="inlineStr">
         <is>
-          <t>1526728427</t>
+          <t>1526740478</t>
         </is>
       </c>
       <c r="C143" s="37" t="inlineStr">
         <is>
-          <t>L.Traffic.User.SCell.DL.Avg</t>
+          <t>L.Traffic.SpecSerUser.Avg</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>Avg CA UEs using this cell as SCell</t>
+          <t>Specified-service (MBB) users</t>
         </is>
       </c>
       <c r="E143" s="9" t="inlineStr">
         <is>
-          <t>Table 4-4 / 5-8</t>
+          <t>Ch.5.4.2: decrease to a non-zero value on low-freq cells ⇒ WBB enhancement took effect</t>
         </is>
       </c>
       <c r="F143" s="10" t="n"/>
@@ -26814,88 +26743,78 @@
       <c r="I143" s="10" t="n"/>
       <c r="J143" s="11" t="n"/>
     </row>
-    <row r="144" ht="32" customHeight="1">
-      <c r="A144" s="32" t="n">
-        <v>9</v>
-      </c>
-      <c r="B144" s="12" t="inlineStr">
-        <is>
-          <t>1526732658</t>
-        </is>
-      </c>
-      <c r="C144" s="33" t="inlineStr">
-        <is>
-          <t>L.CA.Traffic.bits.DL.PCell</t>
-        </is>
-      </c>
-      <c r="D144" s="12" t="inlineStr">
-        <is>
-          <t>DL bits on PCell of CA UEs</t>
-        </is>
-      </c>
-      <c r="E144" s="12" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-8</t>
-        </is>
-      </c>
-      <c r="F144" s="10" t="n"/>
-      <c r="G144" s="10" t="n"/>
-      <c r="H144" s="10" t="n"/>
-      <c r="I144" s="10" t="n"/>
-      <c r="J144" s="11" t="n"/>
-    </row>
-    <row r="145" ht="32" customHeight="1">
-      <c r="A145" s="36" t="n">
-        <v>10</v>
-      </c>
-      <c r="B145" s="9" t="inlineStr">
-        <is>
-          <t>1526729259</t>
-        </is>
-      </c>
-      <c r="C145" s="37" t="inlineStr">
-        <is>
-          <t>L.CA.Traffic.bits.DL.SCell</t>
-        </is>
-      </c>
-      <c r="D145" s="9" t="inlineStr">
-        <is>
-          <t>DL bits on SCell of CA UEs</t>
-        </is>
-      </c>
-      <c r="E145" s="9" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-8</t>
-        </is>
-      </c>
-      <c r="F145" s="10" t="n"/>
-      <c r="G145" s="10" t="n"/>
-      <c r="H145" s="10" t="n"/>
-      <c r="I145" s="10" t="n"/>
-      <c r="J145" s="11" t="n"/>
-    </row>
-    <row r="146" ht="32" customHeight="1">
-      <c r="A146" s="32" t="n">
-        <v>11</v>
-      </c>
-      <c r="B146" s="12" t="inlineStr">
-        <is>
-          <t>1526728564</t>
-        </is>
-      </c>
-      <c r="C146" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL.CAUser</t>
-        </is>
-      </c>
-      <c r="D146" s="12" t="inlineStr">
-        <is>
-          <t>CA UE DL bits</t>
-        </is>
-      </c>
-      <c r="E146" s="12" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-5 / 5-8; CA UE rate KPI</t>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>H.  KPI formulas  (Ch.4.2.1, 4.2.2, 4.4.2, 5.2)</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="n"/>
+      <c r="C144" s="6" t="n"/>
+      <c r="D144" s="6" t="n"/>
+      <c r="E144" s="6" t="n"/>
+      <c r="F144" s="6" t="n"/>
+      <c r="G144" s="6" t="n"/>
+      <c r="H144" s="6" t="n"/>
+      <c r="I144" s="6" t="n"/>
+      <c r="J144" s="6" t="n"/>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t>Formula (from document)</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="F145" s="7" t="inlineStr"/>
+      <c r="G145" s="7" t="inlineStr"/>
+      <c r="H145" s="7" t="inlineStr"/>
+      <c r="I145" s="7" t="inlineStr"/>
+      <c r="J145" s="7" t="inlineStr"/>
+    </row>
+    <row r="146" ht="48" customHeight="1">
+      <c r="A146" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>UL-quality inter-freq HO success</t>
+        </is>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.ExecSuccOut / L.HHO.InterFreq.ULquality.ExecAttOut × 100%</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>From Table 4-3 counters. Rise in Prep/Exec/Succ verifies activation.</t>
         </is>
       </c>
       <c r="F146" s="10" t="n"/>
@@ -26904,28 +26823,30 @@
       <c r="I146" s="10" t="n"/>
       <c r="J146" s="11" t="n"/>
     </row>
-    <row r="147" ht="32" customHeight="1">
-      <c r="A147" s="36" t="n">
-        <v>12</v>
-      </c>
-      <c r="B147" s="9" t="inlineStr">
-        <is>
-          <t>1526740440</t>
-        </is>
-      </c>
-      <c r="C147" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL.LastTTI.CAUser</t>
-        </is>
-      </c>
-      <c r="D147" s="9" t="inlineStr">
-        <is>
-          <t>CA UE last-TTI DL bits</t>
-        </is>
-      </c>
-      <c r="E147" s="9" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-5</t>
+    <row r="147" ht="48" customHeight="1">
+      <c r="A147" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B147" s="12" t="inlineStr">
+        <is>
+          <t>UL-quality FDD↔TDD HO success</t>
+        </is>
+      </c>
+      <c r="C147" s="12" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFddTdd.ULquality.ExecSuccOut / L.HHO.InterFddTdd.ULquality.ExecAttOut × 100%</t>
+        </is>
+      </c>
+      <c r="D147" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E147" s="12" t="inlineStr">
+        <is>
+          <t>Table 4-3</t>
         </is>
       </c>
       <c r="F147" s="10" t="n"/>
@@ -26934,28 +26855,30 @@
       <c r="I147" s="10" t="n"/>
       <c r="J147" s="11" t="n"/>
     </row>
-    <row r="148" ht="32" customHeight="1">
-      <c r="A148" s="32" t="n">
-        <v>13</v>
-      </c>
-      <c r="B148" s="12" t="inlineStr">
-        <is>
-          <t>1526740441</t>
-        </is>
-      </c>
-      <c r="C148" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
-        </is>
-      </c>
-      <c r="D148" s="12" t="inlineStr">
-        <is>
-          <t>CA UE DL time last-TTI removed</t>
-        </is>
-      </c>
-      <c r="E148" s="12" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-5</t>
+    <row r="148" ht="48" customHeight="1">
+      <c r="A148" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>Average downlink throughput of CA UEs</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>(L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
+        <is>
+          <t>Ch.4.2.1 Scenario 1. If CA UE proportion rises after SC, this KPI may even drop.</t>
         </is>
       </c>
       <c r="F148" s="10" t="n"/>
@@ -26964,28 +26887,30 @@
       <c r="I148" s="10" t="n"/>
       <c r="J148" s="11" t="n"/>
     </row>
-    <row r="149" ht="32" customHeight="1">
-      <c r="A149" s="36" t="n">
-        <v>14</v>
-      </c>
-      <c r="B149" s="9" t="inlineStr">
-        <is>
-          <t>1526729045</t>
-        </is>
-      </c>
-      <c r="C149" s="37" t="inlineStr">
-        <is>
-          <t>L.CA.DLSCell.Add.Att</t>
-        </is>
-      </c>
-      <c r="D149" s="9" t="inlineStr">
-        <is>
-          <t>DL SCell add attempts</t>
-        </is>
-      </c>
-      <c r="E149" s="9" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-8; SCell cfg success vs HO</t>
+    <row r="149" ht="48" customHeight="1">
+      <c r="A149" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t>SCell configuration success rate</t>
+        </is>
+      </c>
+      <c r="C149" s="12" t="inlineStr">
+        <is>
+          <t>L.CA.DLSCell.Add.Succ / L.CA.DLSCell.Add.Att × 100%</t>
+        </is>
+      </c>
+      <c r="D149" s="12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E149" s="12" t="inlineStr">
+        <is>
+          <t>Ch.4.2.2 / 5.2.2: affected by HO success once HoWithSccCfgSwitch is on.</t>
         </is>
       </c>
       <c r="F149" s="10" t="n"/>
@@ -26994,28 +26919,30 @@
       <c r="I149" s="10" t="n"/>
       <c r="J149" s="11" t="n"/>
     </row>
-    <row r="150" ht="32" customHeight="1">
-      <c r="A150" s="32" t="n">
-        <v>15</v>
-      </c>
-      <c r="B150" s="12" t="inlineStr">
-        <is>
-          <t>1526729046</t>
-        </is>
-      </c>
-      <c r="C150" s="33" t="inlineStr">
-        <is>
-          <t>L.CA.DLSCell.Add.Succ</t>
-        </is>
-      </c>
-      <c r="D150" s="12" t="inlineStr">
-        <is>
-          <t>DL SCell add success</t>
-        </is>
-      </c>
-      <c r="E150" s="12" t="inlineStr">
-        <is>
-          <t>Table 4-4 / 5-8</t>
+    <row r="150" ht="48" customHeight="1">
+      <c r="A150" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>Perceived data rate of MBB UEs (enhancement)</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>[(L.Thrp.bits.DL − L.Thrp.bits.DL.LastTTI) − (L.Thrp.bits.DL.WBB − L.Thrp.bits.DL.LastTTI.WBB)] / (L.Thrp.Time.DL.RmvLastTTI − L.Thrp.Time.DL.RmvLastTTI.WBB)</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E150" s="9" t="inlineStr">
+        <is>
+          <t>Ch.5.2.1 Table 5-4. Expected to increase when enhancement is activated (low-freq were normal cells).</t>
         </is>
       </c>
       <c r="F150" s="10" t="n"/>
@@ -27024,28 +26951,30 @@
       <c r="I150" s="10" t="n"/>
       <c r="J150" s="11" t="n"/>
     </row>
-    <row r="151" ht="32" customHeight="1">
-      <c r="A151" s="36" t="n">
-        <v>16</v>
-      </c>
-      <c r="B151" s="9" t="inlineStr">
-        <is>
-          <t>1526746999–7008</t>
-        </is>
-      </c>
-      <c r="C151" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.DL.BitRate.Samp.CaUe.Index0 … Index9</t>
-        </is>
-      </c>
-      <c r="D151" s="9" t="inlineStr">
-        <is>
-          <t>CA UE DL bit-rate samples (10 bins)</t>
-        </is>
-      </c>
-      <c r="E151" s="9" t="inlineStr">
-        <is>
-          <t>Table 4-4 monitoring</t>
+    <row r="151" ht="48" customHeight="1">
+      <c r="A151" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B151" s="12" t="inlineStr">
+        <is>
+          <t>Perceived data rate of CA UEs (enhancement impact)</t>
+        </is>
+      </c>
+      <c r="C151" s="12" t="inlineStr">
+        <is>
+          <t>(L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="D151" s="12" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E151" s="12" t="inlineStr">
+        <is>
+          <t>Ch.5.2.2: overall average perceived CA UE rate decreases after enhancement.</t>
         </is>
       </c>
       <c r="F151" s="10" t="n"/>
@@ -27054,28 +26983,30 @@
       <c r="I151" s="10" t="n"/>
       <c r="J151" s="11" t="n"/>
     </row>
-    <row r="152" ht="32" customHeight="1">
-      <c r="A152" s="32" t="n">
-        <v>17</v>
-      </c>
-      <c r="B152" s="12" t="inlineStr">
-        <is>
-          <t>1526728261</t>
-        </is>
-      </c>
-      <c r="C152" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL</t>
-        </is>
-      </c>
-      <c r="D152" s="12" t="inlineStr">
-        <is>
-          <t>All-UE DL bits</t>
-        </is>
-      </c>
-      <c r="E152" s="12" t="inlineStr">
-        <is>
-          <t>Table 5-4 MBB perceived rate</t>
+    <row r="152" ht="48" customHeight="1">
+      <c r="A152" s="9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>Perceived data rate of WBB UEs</t>
+        </is>
+      </c>
+      <c r="C152" s="9" t="inlineStr">
+        <is>
+          <t>(L.Thrp.bits.DL.WBB − L.Thrp.bits.DL.LastTTI.WBB) / L.Thrp.Time.DL.RmvLastTTI.WBB</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E152" s="9" t="inlineStr">
+        <is>
+          <t>Ch.5.2.2 Table 5-6: decreases. CA takes effect for a smaller proportion of WBB UEs.</t>
         </is>
       </c>
       <c r="F152" s="10" t="n"/>
@@ -27084,28 +27015,30 @@
       <c r="I152" s="10" t="n"/>
       <c r="J152" s="11" t="n"/>
     </row>
-    <row r="153" ht="32" customHeight="1">
-      <c r="A153" s="36" t="n">
-        <v>18</v>
-      </c>
-      <c r="B153" s="9" t="inlineStr">
-        <is>
-          <t>1526729005</t>
-        </is>
-      </c>
-      <c r="C153" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL.LastTTI</t>
-        </is>
-      </c>
-      <c r="D153" s="9" t="inlineStr">
-        <is>
-          <t>All-UE last-TTI DL bits</t>
-        </is>
-      </c>
-      <c r="E153" s="9" t="inlineStr">
-        <is>
-          <t>Table 5-4</t>
+    <row r="153" ht="48" customHeight="1">
+      <c r="A153" s="12" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B153" s="12" t="inlineStr">
+        <is>
+          <t>Perceived data rate of RRNs</t>
+        </is>
+      </c>
+      <c r="C153" s="12" t="inlineStr">
+        <is>
+          <t>L.Thrp.Relay.bits.DL / L.Thrp.Relay.Time.DL</t>
+        </is>
+      </c>
+      <c r="D153" s="12" t="inlineStr">
+        <is>
+          <t>bit/s</t>
+        </is>
+      </c>
+      <c r="E153" s="12" t="inlineStr">
+        <is>
+          <t>Ch.5.2.2 Table 5-7: decreases.</t>
         </is>
       </c>
       <c r="F153" s="10" t="n"/>
@@ -27114,242 +27047,233 @@
       <c r="I153" s="10" t="n"/>
       <c r="J153" s="11" t="n"/>
     </row>
-    <row r="154" ht="32" customHeight="1">
-      <c r="A154" s="32" t="n">
-        <v>19</v>
-      </c>
-      <c r="B154" s="12" t="inlineStr">
-        <is>
-          <t>1526745879</t>
-        </is>
-      </c>
-      <c r="C154" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL.WBB</t>
-        </is>
-      </c>
-      <c r="D154" s="12" t="inlineStr">
-        <is>
-          <t>WBB DL bits</t>
-        </is>
-      </c>
-      <c r="E154" s="12" t="inlineStr">
-        <is>
-          <t>Tables 5-4 / 5-6</t>
-        </is>
-      </c>
-      <c r="F154" s="10" t="n"/>
-      <c r="G154" s="10" t="n"/>
-      <c r="H154" s="10" t="n"/>
-      <c r="I154" s="10" t="n"/>
-      <c r="J154" s="11" t="n"/>
-    </row>
-    <row r="155" ht="32" customHeight="1">
-      <c r="A155" s="36" t="n">
-        <v>20</v>
-      </c>
-      <c r="B155" s="9" t="inlineStr">
-        <is>
-          <t>1526745880</t>
-        </is>
-      </c>
-      <c r="C155" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.bits.DL.LastTTI.WBB</t>
-        </is>
-      </c>
-      <c r="D155" s="9" t="inlineStr">
-        <is>
-          <t>WBB last-TTI DL bits</t>
-        </is>
-      </c>
-      <c r="E155" s="9" t="inlineStr">
-        <is>
-          <t>Tables 5-4 / 5-6</t>
-        </is>
-      </c>
-      <c r="F155" s="10" t="n"/>
-      <c r="G155" s="10" t="n"/>
-      <c r="H155" s="10" t="n"/>
-      <c r="I155" s="10" t="n"/>
-      <c r="J155" s="11" t="n"/>
-    </row>
-    <row r="156" ht="32" customHeight="1">
-      <c r="A156" s="32" t="n">
-        <v>21</v>
-      </c>
-      <c r="B156" s="12" t="inlineStr">
-        <is>
-          <t>1526729015</t>
-        </is>
-      </c>
-      <c r="C156" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.Time.DL.RmvLastTTI</t>
-        </is>
-      </c>
-      <c r="D156" s="12" t="inlineStr">
-        <is>
-          <t>All-UE DL time last-TTI removed</t>
-        </is>
-      </c>
-      <c r="E156" s="12" t="inlineStr">
-        <is>
-          <t>Table 5-4</t>
-        </is>
-      </c>
-      <c r="F156" s="10" t="n"/>
-      <c r="G156" s="10" t="n"/>
-      <c r="H156" s="10" t="n"/>
-      <c r="I156" s="10" t="n"/>
-      <c r="J156" s="11" t="n"/>
-    </row>
-    <row r="157" ht="32" customHeight="1">
-      <c r="A157" s="36" t="n">
-        <v>22</v>
-      </c>
-      <c r="B157" s="9" t="inlineStr">
-        <is>
-          <t>1526745881</t>
-        </is>
-      </c>
-      <c r="C157" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.Time.DL.RmvLastTTI.WBB</t>
-        </is>
-      </c>
-      <c r="D157" s="9" t="inlineStr">
-        <is>
-          <t>WBB DL time last-TTI removed</t>
-        </is>
-      </c>
-      <c r="E157" s="9" t="inlineStr">
-        <is>
-          <t>Tables 5-4 / 5-6; Ch.5.2.2 may increase</t>
-        </is>
-      </c>
-      <c r="F157" s="10" t="n"/>
-      <c r="G157" s="10" t="n"/>
-      <c r="H157" s="10" t="n"/>
-      <c r="I157" s="10" t="n"/>
-      <c r="J157" s="11" t="n"/>
-    </row>
-    <row r="158" ht="32" customHeight="1">
-      <c r="A158" s="32" t="n">
-        <v>23</v>
-      </c>
-      <c r="B158" s="12" t="inlineStr">
-        <is>
-          <t>1526735542</t>
-        </is>
-      </c>
-      <c r="C158" s="33" t="inlineStr">
-        <is>
-          <t>L.Thrp.Relay.bits.DL</t>
-        </is>
-      </c>
-      <c r="D158" s="12" t="inlineStr">
-        <is>
-          <t>RRN DL bits</t>
-        </is>
-      </c>
-      <c r="E158" s="12" t="inlineStr">
-        <is>
-          <t>Table 5-7</t>
-        </is>
-      </c>
-      <c r="F158" s="10" t="n"/>
-      <c r="G158" s="10" t="n"/>
-      <c r="H158" s="10" t="n"/>
-      <c r="I158" s="10" t="n"/>
-      <c r="J158" s="11" t="n"/>
-    </row>
-    <row r="159" ht="32" customHeight="1">
-      <c r="A159" s="36" t="n">
-        <v>24</v>
+    <row r="154" ht="20" customHeight="1">
+      <c r="A154" s="26" t="inlineStr">
+        <is>
+          <t>H worked example  —  CA UE average DL throughput  (Ch.4.2.1 formula + sample counts)</t>
+        </is>
+      </c>
+      <c r="B154" s="6" t="n"/>
+      <c r="C154" s="6" t="n"/>
+      <c r="D154" s="6" t="n"/>
+      <c r="E154" s="6" t="n"/>
+      <c r="F154" s="6" t="n"/>
+      <c r="G154" s="6" t="n"/>
+      <c r="H154" s="6" t="n"/>
+      <c r="I154" s="6" t="n"/>
+      <c r="J154" s="6" t="n"/>
+    </row>
+    <row r="155" ht="42" customHeight="1">
+      <c r="A155" s="27" t="inlineStr">
+        <is>
+          <t>3GPP / Huawei condition:
+R = (L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
+        </is>
+      </c>
+      <c r="B155" s="28" t="n"/>
+      <c r="C155" s="28" t="n"/>
+      <c r="D155" s="28" t="n"/>
+      <c r="E155" s="28" t="n"/>
+      <c r="F155" s="28" t="n"/>
+      <c r="G155" s="28" t="n"/>
+      <c r="H155" s="28" t="n"/>
+      <c r="I155" s="28" t="n"/>
+      <c r="J155" s="28" t="n"/>
+    </row>
+    <row r="156" ht="90" customHeight="1">
+      <c r="A156" s="13" t="inlineStr">
+        <is>
+          <t>Worked example (sample values from the document or typical live-network settings):
+Suppose a 15-minute bin on the high/low pair after SC:
+  L.Thrp.bits.DL.CAUser = 7.20×10^12 bit
+  L.Thrp.bits.DL.LastTTI.CAUser = 0.45×10^12 bit
+  L.Thrp.Time.DL.RmvLastTTI.CAUser = 1.50×10^8 ms
+  R = (7.20 − 0.45)×10^12 / 1.50×10^8 = 6.75×10^12 / 1.50×10^8 = 4.50×10^4 bit/ms = 45.0 Mbit/s.
+Result: Compare the same formula on cell-edge bins (PUSCH MCS 0–3 share, Ch.4.2.1 Scenario 1) before vs after SC. If CA UE proportion also rose, Ch.4.2.1 warns this average can fall even when network User DL Average Throughput rose.</t>
+        </is>
+      </c>
+      <c r="B156" s="14" t="n"/>
+      <c r="C156" s="14" t="n"/>
+      <c r="D156" s="14" t="n"/>
+      <c r="E156" s="14" t="n"/>
+      <c r="F156" s="14" t="n"/>
+      <c r="G156" s="14" t="n"/>
+      <c r="H156" s="14" t="n"/>
+      <c r="I156" s="14" t="n"/>
+      <c r="J156" s="14" t="n"/>
+    </row>
+    <row r="157" ht="22" customHeight="1">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>I.  Licenses — FDD and TDD  (Ch.4.3.1 / 5.3.1  —  same license covers enhancement)</t>
+        </is>
+      </c>
+      <c r="B157" s="6" t="n"/>
+      <c r="C157" s="6" t="n"/>
+      <c r="D157" s="6" t="n"/>
+      <c r="E157" s="6" t="n"/>
+      <c r="F157" s="6" t="n"/>
+      <c r="G157" s="6" t="n"/>
+      <c r="H157" s="6" t="n"/>
+      <c r="I157" s="6" t="n"/>
+      <c r="J157" s="6" t="n"/>
+    </row>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t>RAT</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>Feature ID</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="inlineStr">
+        <is>
+          <t>Feature name</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="F158" s="7" t="inlineStr">
+        <is>
+          <t>Sales unit</t>
+        </is>
+      </c>
+      <c r="G158" s="7" t="inlineStr">
+        <is>
+          <t>When consumed</t>
+        </is>
+      </c>
+      <c r="H158" s="7" t="inlineStr"/>
+      <c r="I158" s="7" t="inlineStr"/>
+      <c r="J158" s="7" t="inlineStr"/>
+    </row>
+    <row r="159" ht="48" customHeight="1">
+      <c r="A159" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="B159" s="9" t="inlineStr">
         <is>
-          <t>1526735543</t>
-        </is>
-      </c>
-      <c r="C159" s="37" t="inlineStr">
-        <is>
-          <t>L.Thrp.Relay.Time.DL</t>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="inlineStr">
+        <is>
+          <t>LCOFD-131312</t>
         </is>
       </c>
       <c r="D159" s="9" t="inlineStr">
         <is>
-          <t>RRN DL time</t>
+          <t>LTE Spectrum Coordination (LTE FDD)</t>
         </is>
       </c>
       <c r="E159" s="9" t="inlineStr">
         <is>
-          <t>Table 5-7; Ch.5.4.2: increase on low-freq cells ⇒ RRN enhancement took effect</t>
-        </is>
-      </c>
-      <c r="F159" s="10" t="n"/>
-      <c r="G159" s="10" t="n"/>
+          <t>LT1SUNPLTE00</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>per cell</t>
+        </is>
+      </c>
+      <c r="G159" s="9" t="inlineStr">
+        <is>
+          <t>Ch.4.3.1 and Ch.5.3.1. Enhancement uses the same license. Insufficiency of certain items affects CELL ACTIVATION — see License Control Item Lists.</t>
+        </is>
+      </c>
       <c r="H159" s="10" t="n"/>
       <c r="I159" s="10" t="n"/>
       <c r="J159" s="11" t="n"/>
     </row>
-    <row r="160" ht="32" customHeight="1">
-      <c r="A160" s="32" t="n">
-        <v>25</v>
+    <row r="160" ht="48" customHeight="1">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="B160" s="12" t="inlineStr">
         <is>
-          <t>1526745954</t>
-        </is>
-      </c>
-      <c r="C160" s="33" t="inlineStr">
-        <is>
-          <t>L.ChMeas.PRB.DL.PDSCH.WBBUsed.Avg</t>
+          <t>TDD</t>
+        </is>
+      </c>
+      <c r="C160" s="12" t="inlineStr">
+        <is>
+          <t>TDLCOFD-131312</t>
         </is>
       </c>
       <c r="D160" s="12" t="inlineStr">
         <is>
-          <t>Avg PDSCH PRBs used by WBB</t>
+          <t>LTE Spectrum Coordination (LTE TDD)</t>
         </is>
       </c>
       <c r="E160" s="12" t="inlineStr">
         <is>
-          <t>Ch.5.2.2: decreases on low-freq, increases on high-freq</t>
-        </is>
-      </c>
-      <c r="F160" s="10" t="n"/>
-      <c r="G160" s="10" t="n"/>
+          <t>LT1SLTESPC00</t>
+        </is>
+      </c>
+      <c r="F160" s="12" t="inlineStr">
+        <is>
+          <t>per cell</t>
+        </is>
+      </c>
+      <c r="G160" s="12" t="inlineStr">
+        <is>
+          <t>Ch.4.3.1 and Ch.5.3.1. Same note on cell activation. No FDD/TDD feature-difference in switches or principles (§2.4).</t>
+        </is>
+      </c>
       <c r="H160" s="10" t="n"/>
       <c r="I160" s="10" t="n"/>
       <c r="J160" s="11" t="n"/>
     </row>
-    <row r="161" ht="32" customHeight="1">
-      <c r="A161" s="36" t="n">
-        <v>26</v>
+    <row r="161" ht="48" customHeight="1">
+      <c r="A161" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="B161" s="9" t="inlineStr">
         <is>
-          <t>1526740478</t>
-        </is>
-      </c>
-      <c r="C161" s="37" t="inlineStr">
-        <is>
-          <t>L.Traffic.SpecSerUser.Avg</t>
+          <t>FDD/TDD</t>
+        </is>
+      </c>
+      <c r="C161" s="9" t="inlineStr">
+        <is>
+          <t>(this workbook Steps 1–4)</t>
         </is>
       </c>
       <c r="D161" s="9" t="inlineStr">
         <is>
-          <t>Specified-service (MBB) users</t>
+          <t>Carrier aggregation (prerequisite)</t>
         </is>
       </c>
       <c r="E161" s="9" t="inlineStr">
         <is>
-          <t>Ch.5.4.2: decrease to a non-zero value on low-freq cells ⇒ WBB enhancement took effect</t>
-        </is>
-      </c>
-      <c r="F161" s="10" t="n"/>
-      <c r="G161" s="10" t="n"/>
+          <t>LAOFD / TDLAOFD / LEOFD as deployed</t>
+        </is>
+      </c>
+      <c r="F161" s="9" t="inlineStr">
+        <is>
+          <t>per cell</t>
+        </is>
+      </c>
+      <c r="G161" s="9" t="inlineStr">
+        <is>
+          <t>CA must already be licensed and active. SC does not replace CA licenses.</t>
+        </is>
+      </c>
       <c r="H161" s="10" t="n"/>
       <c r="I161" s="10" t="n"/>
       <c r="J161" s="11" t="n"/>
@@ -27357,7 +27281,7 @@
     <row r="162" ht="22" customHeight="1">
       <c r="A162" s="5" t="inlineStr">
         <is>
-          <t>H.  KPI formulas  (Ch.4.2.1, 4.2.2, 4.4.2, 5.2)</t>
+          <t>J.  LTE Spectrum Coordination Enhancement  (Ch.5)  —  WBB UEs and RRNs</t>
         </is>
       </c>
       <c r="B162" s="6" t="n"/>
@@ -27370,559 +27294,24 @@
       <c r="I162" s="6" t="n"/>
       <c r="J162" s="6" t="n"/>
     </row>
-    <row r="163" ht="22" customHeight="1">
-      <c r="A163" s="7" t="inlineStr">
-        <is>
-          <t>SN</t>
-        </is>
-      </c>
-      <c r="B163" s="7" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-      <c r="C163" s="7" t="inlineStr">
-        <is>
-          <t>Formula (from document)</t>
-        </is>
-      </c>
-      <c r="D163" s="7" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E163" s="7" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="F163" s="7" t="inlineStr"/>
-      <c r="G163" s="7" t="inlineStr"/>
-      <c r="H163" s="7" t="inlineStr"/>
-      <c r="I163" s="7" t="inlineStr"/>
-      <c r="J163" s="7" t="inlineStr"/>
-    </row>
-    <row r="164" ht="48" customHeight="1">
-      <c r="A164" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B164" s="9" t="inlineStr">
-        <is>
-          <t>UL-quality inter-freq HO success</t>
-        </is>
-      </c>
-      <c r="C164" s="9" t="inlineStr">
-        <is>
-          <t>L.HHO.InterFreq.ULquality.ExecSuccOut / L.HHO.InterFreq.ULquality.ExecAttOut × 100%</t>
-        </is>
-      </c>
-      <c r="D164" s="9" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E164" s="9" t="inlineStr">
-        <is>
-          <t>From Table 4-3 counters. Rise in Prep/Exec/Succ verifies activation.</t>
-        </is>
-      </c>
-      <c r="F164" s="10" t="n"/>
-      <c r="G164" s="10" t="n"/>
-      <c r="H164" s="10" t="n"/>
-      <c r="I164" s="10" t="n"/>
-      <c r="J164" s="11" t="n"/>
-    </row>
-    <row r="165" ht="48" customHeight="1">
-      <c r="A165" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B165" s="12" t="inlineStr">
-        <is>
-          <t>UL-quality FDD↔TDD HO success</t>
-        </is>
-      </c>
-      <c r="C165" s="12" t="inlineStr">
-        <is>
-          <t>L.HHO.InterFddTdd.ULquality.ExecSuccOut / L.HHO.InterFddTdd.ULquality.ExecAttOut × 100%</t>
-        </is>
-      </c>
-      <c r="D165" s="12" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E165" s="12" t="inlineStr">
-        <is>
-          <t>Table 4-3</t>
-        </is>
-      </c>
-      <c r="F165" s="10" t="n"/>
-      <c r="G165" s="10" t="n"/>
-      <c r="H165" s="10" t="n"/>
-      <c r="I165" s="10" t="n"/>
-      <c r="J165" s="11" t="n"/>
-    </row>
-    <row r="166" ht="48" customHeight="1">
-      <c r="A166" s="9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B166" s="9" t="inlineStr">
-        <is>
-          <t>Average downlink throughput of CA UEs</t>
-        </is>
-      </c>
-      <c r="C166" s="9" t="inlineStr">
-        <is>
-          <t>(L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
-        </is>
-      </c>
-      <c r="D166" s="9" t="inlineStr">
-        <is>
-          <t>bit/s</t>
-        </is>
-      </c>
-      <c r="E166" s="9" t="inlineStr">
-        <is>
-          <t>Ch.4.2.1 Scenario 1. If CA UE proportion rises after SC, this KPI may even drop.</t>
-        </is>
-      </c>
-      <c r="F166" s="10" t="n"/>
-      <c r="G166" s="10" t="n"/>
-      <c r="H166" s="10" t="n"/>
-      <c r="I166" s="10" t="n"/>
-      <c r="J166" s="11" t="n"/>
-    </row>
-    <row r="167" ht="48" customHeight="1">
-      <c r="A167" s="12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B167" s="12" t="inlineStr">
-        <is>
-          <t>SCell configuration success rate</t>
-        </is>
-      </c>
-      <c r="C167" s="12" t="inlineStr">
-        <is>
-          <t>L.CA.DLSCell.Add.Succ / L.CA.DLSCell.Add.Att × 100%</t>
-        </is>
-      </c>
-      <c r="D167" s="12" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E167" s="12" t="inlineStr">
-        <is>
-          <t>Ch.4.2.2 / 5.2.2: affected by HO success once HoWithSccCfgSwitch is on.</t>
-        </is>
-      </c>
-      <c r="F167" s="10" t="n"/>
-      <c r="G167" s="10" t="n"/>
-      <c r="H167" s="10" t="n"/>
-      <c r="I167" s="10" t="n"/>
-      <c r="J167" s="11" t="n"/>
-    </row>
-    <row r="168" ht="48" customHeight="1">
-      <c r="A168" s="9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B168" s="9" t="inlineStr">
-        <is>
-          <t>Perceived data rate of MBB UEs (enhancement)</t>
-        </is>
-      </c>
-      <c r="C168" s="9" t="inlineStr">
-        <is>
-          <t>[(L.Thrp.bits.DL − L.Thrp.bits.DL.LastTTI) − (L.Thrp.bits.DL.WBB − L.Thrp.bits.DL.LastTTI.WBB)] / (L.Thrp.Time.DL.RmvLastTTI − L.Thrp.Time.DL.RmvLastTTI.WBB)</t>
-        </is>
-      </c>
-      <c r="D168" s="9" t="inlineStr">
-        <is>
-          <t>bit/s</t>
-        </is>
-      </c>
-      <c r="E168" s="9" t="inlineStr">
-        <is>
-          <t>Ch.5.2.1 Table 5-4. Expected to increase when enhancement is activated (low-freq were normal cells).</t>
-        </is>
-      </c>
-      <c r="F168" s="10" t="n"/>
-      <c r="G168" s="10" t="n"/>
-      <c r="H168" s="10" t="n"/>
-      <c r="I168" s="10" t="n"/>
-      <c r="J168" s="11" t="n"/>
-    </row>
-    <row r="169" ht="48" customHeight="1">
-      <c r="A169" s="12" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B169" s="12" t="inlineStr">
-        <is>
-          <t>Perceived data rate of CA UEs (enhancement impact)</t>
-        </is>
-      </c>
-      <c r="C169" s="12" t="inlineStr">
-        <is>
-          <t>(L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
-        </is>
-      </c>
-      <c r="D169" s="12" t="inlineStr">
-        <is>
-          <t>bit/s</t>
-        </is>
-      </c>
-      <c r="E169" s="12" t="inlineStr">
-        <is>
-          <t>Ch.5.2.2: overall average perceived CA UE rate decreases after enhancement.</t>
-        </is>
-      </c>
-      <c r="F169" s="10" t="n"/>
-      <c r="G169" s="10" t="n"/>
-      <c r="H169" s="10" t="n"/>
-      <c r="I169" s="10" t="n"/>
-      <c r="J169" s="11" t="n"/>
-    </row>
-    <row r="170" ht="48" customHeight="1">
-      <c r="A170" s="9" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B170" s="9" t="inlineStr">
-        <is>
-          <t>Perceived data rate of WBB UEs</t>
-        </is>
-      </c>
-      <c r="C170" s="9" t="inlineStr">
-        <is>
-          <t>(L.Thrp.bits.DL.WBB − L.Thrp.bits.DL.LastTTI.WBB) / L.Thrp.Time.DL.RmvLastTTI.WBB</t>
-        </is>
-      </c>
-      <c r="D170" s="9" t="inlineStr">
-        <is>
-          <t>bit/s</t>
-        </is>
-      </c>
-      <c r="E170" s="9" t="inlineStr">
-        <is>
-          <t>Ch.5.2.2 Table 5-6: decreases. CA takes effect for a smaller proportion of WBB UEs.</t>
-        </is>
-      </c>
-      <c r="F170" s="10" t="n"/>
-      <c r="G170" s="10" t="n"/>
-      <c r="H170" s="10" t="n"/>
-      <c r="I170" s="10" t="n"/>
-      <c r="J170" s="11" t="n"/>
-    </row>
-    <row r="171" ht="48" customHeight="1">
-      <c r="A171" s="12" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B171" s="12" t="inlineStr">
-        <is>
-          <t>Perceived data rate of RRNs</t>
-        </is>
-      </c>
-      <c r="C171" s="12" t="inlineStr">
-        <is>
-          <t>L.Thrp.Relay.bits.DL / L.Thrp.Relay.Time.DL</t>
-        </is>
-      </c>
-      <c r="D171" s="12" t="inlineStr">
-        <is>
-          <t>bit/s</t>
-        </is>
-      </c>
-      <c r="E171" s="12" t="inlineStr">
-        <is>
-          <t>Ch.5.2.2 Table 5-7: decreases.</t>
-        </is>
-      </c>
-      <c r="F171" s="10" t="n"/>
-      <c r="G171" s="10" t="n"/>
-      <c r="H171" s="10" t="n"/>
-      <c r="I171" s="10" t="n"/>
-      <c r="J171" s="11" t="n"/>
-    </row>
-    <row r="172" ht="20" customHeight="1">
-      <c r="A172" s="26" t="inlineStr">
-        <is>
-          <t>H worked example  —  CA UE average DL throughput  (Ch.4.2.1 formula + sample counts)</t>
-        </is>
-      </c>
-      <c r="B172" s="6" t="n"/>
-      <c r="C172" s="6" t="n"/>
-      <c r="D172" s="6" t="n"/>
-      <c r="E172" s="6" t="n"/>
-      <c r="F172" s="6" t="n"/>
-      <c r="G172" s="6" t="n"/>
-      <c r="H172" s="6" t="n"/>
-      <c r="I172" s="6" t="n"/>
-      <c r="J172" s="6" t="n"/>
-    </row>
-    <row r="173" ht="42" customHeight="1">
-      <c r="A173" s="27" t="inlineStr">
-        <is>
-          <t>3GPP / Huawei condition:
-R = (L.Thrp.bits.DL.CAUser − L.Thrp.bits.DL.LastTTI.CAUser) / L.Thrp.Time.DL.RmvLastTTI.CAUser</t>
-        </is>
-      </c>
-      <c r="B173" s="28" t="n"/>
-      <c r="C173" s="28" t="n"/>
-      <c r="D173" s="28" t="n"/>
-      <c r="E173" s="28" t="n"/>
-      <c r="F173" s="28" t="n"/>
-      <c r="G173" s="28" t="n"/>
-      <c r="H173" s="28" t="n"/>
-      <c r="I173" s="28" t="n"/>
-      <c r="J173" s="28" t="n"/>
-    </row>
-    <row r="174" ht="90" customHeight="1">
-      <c r="A174" s="13" t="inlineStr">
-        <is>
-          <t>Worked example (sample values from the document or typical live-network settings):
-Suppose a 15-minute bin on the high/low pair after SC:
-  L.Thrp.bits.DL.CAUser = 7.20×10^12 bit
-  L.Thrp.bits.DL.LastTTI.CAUser = 0.45×10^12 bit
-  L.Thrp.Time.DL.RmvLastTTI.CAUser = 1.50×10^8 ms
-  R = (7.20 − 0.45)×10^12 / 1.50×10^8 = 6.75×10^12 / 1.50×10^8 = 4.50×10^4 bit/ms = 45.0 Mbit/s.
-Result: Compare the same formula on cell-edge bins (PUSCH MCS 0–3 share, Ch.4.2.1 Scenario 1) before vs after SC. If CA UE proportion also rose, Ch.4.2.1 warns this average can fall even when network User DL Average Throughput rose.</t>
-        </is>
-      </c>
-      <c r="B174" s="14" t="n"/>
-      <c r="C174" s="14" t="n"/>
-      <c r="D174" s="14" t="n"/>
-      <c r="E174" s="14" t="n"/>
-      <c r="F174" s="14" t="n"/>
-      <c r="G174" s="14" t="n"/>
-      <c r="H174" s="14" t="n"/>
-      <c r="I174" s="14" t="n"/>
-      <c r="J174" s="14" t="n"/>
-    </row>
-    <row r="175" ht="22" customHeight="1">
-      <c r="A175" s="5" t="inlineStr">
-        <is>
-          <t>I.  Licenses — FDD and TDD  (Ch.4.3.1 / 5.3.1  —  same license covers enhancement)</t>
-        </is>
-      </c>
-      <c r="B175" s="6" t="n"/>
-      <c r="C175" s="6" t="n"/>
-      <c r="D175" s="6" t="n"/>
-      <c r="E175" s="6" t="n"/>
-      <c r="F175" s="6" t="n"/>
-      <c r="G175" s="6" t="n"/>
-      <c r="H175" s="6" t="n"/>
-      <c r="I175" s="6" t="n"/>
-      <c r="J175" s="6" t="n"/>
-    </row>
-    <row r="176" ht="22" customHeight="1">
-      <c r="A176" s="7" t="inlineStr">
-        <is>
-          <t>SN</t>
-        </is>
-      </c>
-      <c r="B176" s="7" t="inlineStr">
-        <is>
-          <t>RAT</t>
-        </is>
-      </c>
-      <c r="C176" s="7" t="inlineStr">
-        <is>
-          <t>Feature ID</t>
-        </is>
-      </c>
-      <c r="D176" s="7" t="inlineStr">
-        <is>
-          <t>Feature name</t>
-        </is>
-      </c>
-      <c r="E176" s="7" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="F176" s="7" t="inlineStr">
-        <is>
-          <t>Sales unit</t>
-        </is>
-      </c>
-      <c r="G176" s="7" t="inlineStr">
-        <is>
-          <t>When consumed</t>
-        </is>
-      </c>
-      <c r="H176" s="7" t="inlineStr"/>
-      <c r="I176" s="7" t="inlineStr"/>
-      <c r="J176" s="7" t="inlineStr"/>
-    </row>
-    <row r="177" ht="48" customHeight="1">
-      <c r="A177" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B177" s="9" t="inlineStr">
-        <is>
-          <t>FDD</t>
-        </is>
-      </c>
-      <c r="C177" s="9" t="inlineStr">
-        <is>
-          <t>LCOFD-131312</t>
-        </is>
-      </c>
-      <c r="D177" s="9" t="inlineStr">
-        <is>
-          <t>LTE Spectrum Coordination (LTE FDD)</t>
-        </is>
-      </c>
-      <c r="E177" s="9" t="inlineStr">
-        <is>
-          <t>LT1SUNPLTE00</t>
-        </is>
-      </c>
-      <c r="F177" s="9" t="inlineStr">
-        <is>
-          <t>per cell</t>
-        </is>
-      </c>
-      <c r="G177" s="9" t="inlineStr">
-        <is>
-          <t>Ch.4.3.1 and Ch.5.3.1. Enhancement uses the same license. Insufficiency of certain items affects CELL ACTIVATION — see License Control Item Lists.</t>
-        </is>
-      </c>
-      <c r="H177" s="10" t="n"/>
-      <c r="I177" s="10" t="n"/>
-      <c r="J177" s="11" t="n"/>
-    </row>
-    <row r="178" ht="48" customHeight="1">
-      <c r="A178" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B178" s="12" t="inlineStr">
-        <is>
-          <t>TDD</t>
-        </is>
-      </c>
-      <c r="C178" s="12" t="inlineStr">
-        <is>
-          <t>TDLCOFD-131312</t>
-        </is>
-      </c>
-      <c r="D178" s="12" t="inlineStr">
-        <is>
-          <t>LTE Spectrum Coordination (LTE TDD)</t>
-        </is>
-      </c>
-      <c r="E178" s="12" t="inlineStr">
-        <is>
-          <t>LT1SLTESPC00</t>
-        </is>
-      </c>
-      <c r="F178" s="12" t="inlineStr">
-        <is>
-          <t>per cell</t>
-        </is>
-      </c>
-      <c r="G178" s="12" t="inlineStr">
-        <is>
-          <t>Ch.4.3.1 and Ch.5.3.1. Same note on cell activation. No FDD/TDD feature-difference in switches or principles (§2.4).</t>
-        </is>
-      </c>
-      <c r="H178" s="10" t="n"/>
-      <c r="I178" s="10" t="n"/>
-      <c r="J178" s="11" t="n"/>
-    </row>
-    <row r="179" ht="48" customHeight="1">
-      <c r="A179" s="9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B179" s="9" t="inlineStr">
-        <is>
-          <t>FDD/TDD</t>
-        </is>
-      </c>
-      <c r="C179" s="9" t="inlineStr">
-        <is>
-          <t>(this workbook Steps 1–4)</t>
-        </is>
-      </c>
-      <c r="D179" s="9" t="inlineStr">
-        <is>
-          <t>Carrier aggregation (prerequisite)</t>
-        </is>
-      </c>
-      <c r="E179" s="9" t="inlineStr">
-        <is>
-          <t>LAOFD / TDLAOFD / LEOFD as deployed</t>
-        </is>
-      </c>
-      <c r="F179" s="9" t="inlineStr">
-        <is>
-          <t>per cell</t>
-        </is>
-      </c>
-      <c r="G179" s="9" t="inlineStr">
-        <is>
-          <t>CA must already be licensed and active. SC does not replace CA licenses.</t>
-        </is>
-      </c>
-      <c r="H179" s="10" t="n"/>
-      <c r="I179" s="10" t="n"/>
-      <c r="J179" s="11" t="n"/>
-    </row>
-    <row r="180" ht="22" customHeight="1">
-      <c r="A180" s="5" t="inlineStr">
-        <is>
-          <t>J.  LTE Spectrum Coordination Enhancement  (Ch.5)  —  WBB UEs and RRNs</t>
-        </is>
-      </c>
-      <c r="B180" s="6" t="n"/>
-      <c r="C180" s="6" t="n"/>
-      <c r="D180" s="6" t="n"/>
-      <c r="E180" s="6" t="n"/>
-      <c r="F180" s="6" t="n"/>
-      <c r="G180" s="6" t="n"/>
-      <c r="H180" s="6" t="n"/>
-      <c r="I180" s="6" t="n"/>
-      <c r="J180" s="6" t="n"/>
-    </row>
-    <row r="181" ht="20" customHeight="1">
-      <c r="A181" s="21" t="inlineStr">
+    <row r="163" ht="20" customHeight="1">
+      <c r="A163" s="21" t="inlineStr">
         <is>
           <t>J1.  WBB UEs  (Ch.5.1.1)  —  trigger is downlink RSRP, not UL SINR</t>
         </is>
       </c>
-      <c r="B181" s="22" t="n"/>
-      <c r="C181" s="22" t="n"/>
-      <c r="D181" s="22" t="n"/>
-      <c r="E181" s="22" t="n"/>
-      <c r="F181" s="22" t="n"/>
-      <c r="G181" s="22" t="n"/>
-      <c r="H181" s="22" t="n"/>
-      <c r="I181" s="22" t="n"/>
-      <c r="J181" s="22" t="n"/>
-    </row>
-    <row r="182" ht="130" customHeight="1">
-      <c r="A182" s="18" t="inlineStr">
+      <c r="B163" s="22" t="n"/>
+      <c r="C163" s="22" t="n"/>
+      <c r="D163" s="22" t="n"/>
+      <c r="E163" s="22" t="n"/>
+      <c r="F163" s="22" t="n"/>
+      <c r="G163" s="22" t="n"/>
+      <c r="H163" s="22" t="n"/>
+      <c r="I163" s="22" t="n"/>
+      <c r="J163" s="22" t="n"/>
+    </row>
+    <row r="164" ht="130" customHeight="1">
+      <c r="A164" s="18" t="inlineStr">
         <is>
           <t>In addition to Ch.4, enhancement applies to CA-capable WBB UEs. When the UE is at the coverage edge of its high-frequency serving cell and has low downlink RSRP there, the eNodeB evaluates whether a low-frequency cell can provide better performance; if yes, HO PCell to that low-frequency cell and configure the original PCell as SCell.
 WBB UEs are identified by SPID or by QCI (see WBB FPD).
@@ -27931,34 +27320,34 @@
 After HO to an MBB service cell: original PCell becomes SCell; WBB-dedicated cells can be SCells; MBB service cells cannot be SCells; eNodeB will not remove SCells based on A2; DL data is scheduled only in SCells whenever possible (if all SCell config fails, UE may use the MBB PCell).</t>
         </is>
       </c>
-      <c r="B182" s="19" t="n"/>
-      <c r="C182" s="19" t="n"/>
-      <c r="D182" s="19" t="n"/>
-      <c r="E182" s="19" t="n"/>
-      <c r="F182" s="19" t="n"/>
-      <c r="G182" s="19" t="n"/>
-      <c r="H182" s="19" t="n"/>
-      <c r="I182" s="19" t="n"/>
-      <c r="J182" s="19" t="n"/>
-    </row>
-    <row r="183" ht="20" customHeight="1">
-      <c r="A183" s="26" t="inlineStr">
+      <c r="B164" s="19" t="n"/>
+      <c r="C164" s="19" t="n"/>
+      <c r="D164" s="19" t="n"/>
+      <c r="E164" s="19" t="n"/>
+      <c r="F164" s="19" t="n"/>
+      <c r="G164" s="19" t="n"/>
+      <c r="H164" s="19" t="n"/>
+      <c r="I164" s="19" t="n"/>
+      <c r="J164" s="19" t="n"/>
+    </row>
+    <row r="165" ht="20" customHeight="1">
+      <c r="A165" s="26" t="inlineStr">
         <is>
           <t>J2.  WBB A2 threshold  (Table 5-1)  +  A5 Thresh1/Thresh2  (Tables 5-2 / 5-3)</t>
         </is>
       </c>
-      <c r="B183" s="6" t="n"/>
-      <c r="C183" s="6" t="n"/>
-      <c r="D183" s="6" t="n"/>
-      <c r="E183" s="6" t="n"/>
-      <c r="F183" s="6" t="n"/>
-      <c r="G183" s="6" t="n"/>
-      <c r="H183" s="6" t="n"/>
-      <c r="I183" s="6" t="n"/>
-      <c r="J183" s="6" t="n"/>
-    </row>
-    <row r="184" ht="90" customHeight="1">
-      <c r="A184" s="27" t="inlineStr">
+      <c r="B165" s="6" t="n"/>
+      <c r="C165" s="6" t="n"/>
+      <c r="D165" s="6" t="n"/>
+      <c r="E165" s="6" t="n"/>
+      <c r="F165" s="6" t="n"/>
+      <c r="G165" s="6" t="n"/>
+      <c r="H165" s="6" t="n"/>
+      <c r="I165" s="6" t="n"/>
+      <c r="J165" s="6" t="n"/>
+    </row>
+    <row r="166" ht="90" customHeight="1">
+      <c r="A166" s="27" t="inlineStr">
         <is>
           <t>3GPP / Huawei condition:
 A2 (SPID WBB) = InterFreqHoA2ThdRsrp + SpidCfg.InterFreqHoA2RsrpThdFactor + WbbMultiCarrierCoordA2Ofs
@@ -27969,18 +27358,18 @@
     Max{ PccFreqCfg.PccA4RsrpThd ,  InterFreqHoA2ThdRsrp + WbbMultiCarrierCoordA2Ofs + 2 }</t>
         </is>
       </c>
-      <c r="B184" s="28" t="n"/>
-      <c r="C184" s="28" t="n"/>
-      <c r="D184" s="28" t="n"/>
-      <c r="E184" s="28" t="n"/>
-      <c r="F184" s="28" t="n"/>
-      <c r="G184" s="28" t="n"/>
-      <c r="H184" s="28" t="n"/>
-      <c r="I184" s="28" t="n"/>
-      <c r="J184" s="28" t="n"/>
-    </row>
-    <row r="185" ht="90" customHeight="1">
-      <c r="A185" s="13" t="inlineStr">
+      <c r="B166" s="28" t="n"/>
+      <c r="C166" s="28" t="n"/>
+      <c r="D166" s="28" t="n"/>
+      <c r="E166" s="28" t="n"/>
+      <c r="F166" s="28" t="n"/>
+      <c r="G166" s="28" t="n"/>
+      <c r="H166" s="28" t="n"/>
+      <c r="I166" s="28" t="n"/>
+      <c r="J166" s="28" t="n"/>
+    </row>
+    <row r="167" ht="90" customHeight="1">
+      <c r="A167" s="13" t="inlineStr">
         <is>
           <t>Worked example (sample values from the document or typical live-network settings):
 Doc MML: WbbMultiCarrierCoordA2Ofs = 2. Assume InterFreqHoA2ThdRsrp = −105 dBm, PccA4RsrpThd = −105 dBm, QCI-identified WBB UE, adaptive, RSRP.
@@ -27989,68 +27378,68 @@
 Result: PCell RSRP must stay below A2 (−103) throughout TTT; neighbor must exceed A5 Thresh2 (−101) with Thresh1 always true at realistic RSRP. If the A5 target is an MBB service cell that cannot aggregate with any current serving cell, eNodeB does not HO.</t>
         </is>
       </c>
-      <c r="B185" s="14" t="n"/>
-      <c r="C185" s="14" t="n"/>
-      <c r="D185" s="14" t="n"/>
-      <c r="E185" s="14" t="n"/>
-      <c r="F185" s="14" t="n"/>
-      <c r="G185" s="14" t="n"/>
-      <c r="H185" s="14" t="n"/>
-      <c r="I185" s="14" t="n"/>
-      <c r="J185" s="14" t="n"/>
-    </row>
-    <row r="186" ht="20" customHeight="1">
-      <c r="A186" s="21" t="inlineStr">
+      <c r="B167" s="14" t="n"/>
+      <c r="C167" s="14" t="n"/>
+      <c r="D167" s="14" t="n"/>
+      <c r="E167" s="14" t="n"/>
+      <c r="F167" s="14" t="n"/>
+      <c r="G167" s="14" t="n"/>
+      <c r="H167" s="14" t="n"/>
+      <c r="I167" s="14" t="n"/>
+      <c r="J167" s="14" t="n"/>
+    </row>
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="21" t="inlineStr">
         <is>
           <t>J3.  RRNs  (Ch.5.1.2)</t>
         </is>
       </c>
-      <c r="B186" s="22" t="n"/>
-      <c r="C186" s="22" t="n"/>
-      <c r="D186" s="22" t="n"/>
-      <c r="E186" s="22" t="n"/>
-      <c r="F186" s="22" t="n"/>
-      <c r="G186" s="22" t="n"/>
-      <c r="H186" s="22" t="n"/>
-      <c r="I186" s="22" t="n"/>
-      <c r="J186" s="22" t="n"/>
-    </row>
-    <row r="187" ht="64" customHeight="1">
-      <c r="A187" s="18" t="inlineStr">
+      <c r="B168" s="22" t="n"/>
+      <c r="C168" s="22" t="n"/>
+      <c r="D168" s="22" t="n"/>
+      <c r="E168" s="22" t="n"/>
+      <c r="F168" s="22" t="n"/>
+      <c r="G168" s="22" t="n"/>
+      <c r="H168" s="22" t="n"/>
+      <c r="I168" s="22" t="n"/>
+      <c r="J168" s="22" t="n"/>
+    </row>
+    <row r="169" ht="64" customHeight="1">
+      <c r="A169" s="18" t="inlineStr">
         <is>
           <t>•  Out-of-band relay CA: if RRN PCell is not an MBB service cell, MBB cells cannot be SCells. If PCell is MBB, non-MBB cells can be SCells; DL scheduled only in SCells when possible; if all SCell config fails, RRN may use the MBB cell.
 •  Enabled when MBBSERCELL is set on the low-frequency no-WBB-access cells AND WbbCaMultiCarrierCoordSw is selected.
 •  Verification (Ch.5.4.2): L.Thrp.Relay.Time.DL (1526735543) increases on low-frequency cells.</t>
         </is>
       </c>
-      <c r="B187" s="19" t="n"/>
-      <c r="C187" s="19" t="n"/>
-      <c r="D187" s="19" t="n"/>
-      <c r="E187" s="19" t="n"/>
-      <c r="F187" s="19" t="n"/>
-      <c r="G187" s="19" t="n"/>
-      <c r="H187" s="19" t="n"/>
-      <c r="I187" s="19" t="n"/>
-      <c r="J187" s="19" t="n"/>
-    </row>
-    <row r="188" ht="22" customHeight="1">
-      <c r="A188" s="5" t="inlineStr">
+      <c r="B169" s="19" t="n"/>
+      <c r="C169" s="19" t="n"/>
+      <c r="D169" s="19" t="n"/>
+      <c r="E169" s="19" t="n"/>
+      <c r="F169" s="19" t="n"/>
+      <c r="G169" s="19" t="n"/>
+      <c r="H169" s="19" t="n"/>
+      <c r="I169" s="19" t="n"/>
+      <c r="J169" s="19" t="n"/>
+    </row>
+    <row r="170" ht="22" customHeight="1">
+      <c r="A170" s="5" t="inlineStr">
         <is>
           <t>K.  Hardware, UE, MAE, verification  (Ch.4.3.3–4.4.3, 5.3.3–5.4.3)</t>
         </is>
       </c>
-      <c r="B188" s="6" t="n"/>
-      <c r="C188" s="6" t="n"/>
-      <c r="D188" s="6" t="n"/>
-      <c r="E188" s="6" t="n"/>
-      <c r="F188" s="6" t="n"/>
-      <c r="G188" s="6" t="n"/>
-      <c r="H188" s="6" t="n"/>
-      <c r="I188" s="6" t="n"/>
-      <c r="J188" s="6" t="n"/>
-    </row>
-    <row r="189" ht="110" customHeight="1">
-      <c r="A189" s="18" t="inlineStr">
+      <c r="B170" s="6" t="n"/>
+      <c r="C170" s="6" t="n"/>
+      <c r="D170" s="6" t="n"/>
+      <c r="E170" s="6" t="n"/>
+      <c r="F170" s="6" t="n"/>
+      <c r="G170" s="6" t="n"/>
+      <c r="H170" s="6" t="n"/>
+      <c r="I170" s="6" t="n"/>
+      <c r="J170" s="6" t="n"/>
+    </row>
+    <row r="171" ht="110" customHeight="1">
+      <c r="A171" s="18" t="inlineStr">
         <is>
           <t>•  SC (Ch.4): FDD 3900/5900 macro; TDD 3900/5900 macro + DBS3900/DBS5900 LampSite. LBBPc boards cannot be used. RF: no requirements.
 •  Enhancement (Ch.5): 3900/5900 macro + LampSite. TDD: cells on LBBPc cannot be used. FDD boards: no requirements. RF: no requirements.
@@ -28060,185 +27449,473 @@
 •  Huawei note (Ch.2.1): this FPD is activation guidance. Gains depend on the live scenario; contact Huawei professional service for optimal gains.</t>
         </is>
       </c>
-      <c r="B189" s="19" t="n"/>
-      <c r="C189" s="19" t="n"/>
-      <c r="D189" s="19" t="n"/>
-      <c r="E189" s="19" t="n"/>
-      <c r="F189" s="19" t="n"/>
-      <c r="G189" s="19" t="n"/>
-      <c r="H189" s="19" t="n"/>
-      <c r="I189" s="19" t="n"/>
-      <c r="J189" s="19" t="n"/>
+      <c r="B171" s="19" t="n"/>
+      <c r="C171" s="19" t="n"/>
+      <c r="D171" s="19" t="n"/>
+      <c r="E171" s="19" t="n"/>
+      <c r="F171" s="19" t="n"/>
+      <c r="G171" s="19" t="n"/>
+      <c r="H171" s="19" t="n"/>
+      <c r="I171" s="19" t="n"/>
+      <c r="J171" s="19" t="n"/>
+    </row>
+    <row r="172" ht="22" customHeight="1">
+      <c r="A172" s="42" t="inlineStr">
+        <is>
+          <t>L.  Final summary  —  meeting quick notes  (1-minute brief)</t>
+        </is>
+      </c>
+      <c r="B172" s="43" t="n"/>
+      <c r="C172" s="43" t="n"/>
+      <c r="D172" s="43" t="n"/>
+      <c r="E172" s="43" t="n"/>
+      <c r="F172" s="43" t="n"/>
+      <c r="G172" s="43" t="n"/>
+      <c r="H172" s="43" t="n"/>
+      <c r="I172" s="43" t="n"/>
+      <c r="J172" s="43" t="n"/>
+    </row>
+    <row r="173" ht="28" customHeight="1">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>Use this block in a meeting. All points are from the LTE Spectrum Coordination FPD (eRAN21.1 Issue 01).</t>
+        </is>
+      </c>
+      <c r="B173" s="17" t="n"/>
+      <c r="C173" s="17" t="n"/>
+      <c r="D173" s="17" t="n"/>
+      <c r="E173" s="17" t="n"/>
+      <c r="F173" s="17" t="n"/>
+      <c r="G173" s="17" t="n"/>
+      <c r="H173" s="17" t="n"/>
+      <c r="I173" s="17" t="n"/>
+      <c r="J173" s="17" t="n"/>
+    </row>
+    <row r="174" ht="22" customHeight="1">
+      <c r="A174" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>What to say</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr"/>
+      <c r="D174" s="7" t="inlineStr"/>
+      <c r="E174" s="7" t="inlineStr"/>
+      <c r="F174" s="7" t="inlineStr"/>
+      <c r="G174" s="7" t="inlineStr"/>
+      <c r="H174" s="7" t="inlineStr"/>
+      <c r="I174" s="7" t="inlineStr"/>
+      <c r="J174" s="7" t="inlineStr"/>
+    </row>
+    <row r="175" ht="40" customHeight="1">
+      <c r="A175" s="35" t="inlineStr">
+        <is>
+          <t>What it is (10 s)</t>
+        </is>
+      </c>
+      <c r="B175" s="29" t="inlineStr">
+        <is>
+          <t>LTE Spectrum Coordination is a CA companion: when a CA UE sits at the high-band UL edge, the eNodeB HOs the PCell to a better low-band SCell and keeps the old PCell as SCell, so DL still uses both bands while UL rides the coverage layer. Feature IDs: LCOFD-131312 (FDD) / TDLCOFD-131312 (TDD). Same for FDD and TDD.</t>
+        </is>
+      </c>
+      <c r="C175" s="10" t="n"/>
+      <c r="D175" s="10" t="n"/>
+      <c r="E175" s="10" t="n"/>
+      <c r="F175" s="10" t="n"/>
+      <c r="G175" s="10" t="n"/>
+      <c r="H175" s="10" t="n"/>
+      <c r="I175" s="10" t="n"/>
+      <c r="J175" s="11" t="n"/>
+    </row>
+    <row r="176" ht="41" customHeight="1">
+      <c r="A176" s="35" t="inlineStr">
+        <is>
+          <t>Benefit (1–2 lines)</t>
+        </is>
+      </c>
+      <c r="B176" s="9" t="inlineStr">
+        <is>
+          <t>It lifts DL usage of CA UEs at the high-frequency UL coverage edge. Best when high/low gap is large. Scenario 1 (both bands already on): PUSCH MCS 0–3 &gt;10% on high band, low-minus-high UL interference &lt;5 dB, CA UE penetration &gt;25% → network User DL Average Throughput up. Scenario 2 (adding a new low band under an existing high band) → both User DL and User UL Average Throughput up.</t>
+        </is>
+      </c>
+      <c r="C176" s="10" t="n"/>
+      <c r="D176" s="10" t="n"/>
+      <c r="E176" s="10" t="n"/>
+      <c r="F176" s="10" t="n"/>
+      <c r="G176" s="10" t="n"/>
+      <c r="H176" s="10" t="n"/>
+      <c r="I176" s="10" t="n"/>
+      <c r="J176" s="11" t="n"/>
+    </row>
+    <row r="177" ht="40" customHeight="1">
+      <c r="A177" s="35" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="B177" s="29" t="inlineStr">
+        <is>
+          <t>CA UE already aggregating. UL SINR used in scheduling (initial MCS) &lt; SpectrumCoordSinrThld (doc MML −2 dB). Then a DL SCell must pass A4 AND be stronger than all its intra-freq neighbours, and must be allowed as PCell. Target pick: PCell/PCC priority → largest BW → lowest EARFCN (or DL air-interface capability first if intelligent selection is ON).</t>
+        </is>
+      </c>
+      <c r="C177" s="10" t="n"/>
+      <c r="D177" s="10" t="n"/>
+      <c r="E177" s="10" t="n"/>
+      <c r="F177" s="10" t="n"/>
+      <c r="G177" s="10" t="n"/>
+      <c r="H177" s="10" t="n"/>
+      <c r="I177" s="10" t="n"/>
+      <c r="J177" s="11" t="n"/>
+    </row>
+    <row r="178" ht="39" customHeight="1">
+      <c r="A178" s="35" t="inlineStr">
+        <is>
+          <t>Leave / after HO</t>
+        </is>
+      </c>
+      <c r="B178" s="9" t="inlineStr">
+        <is>
+          <t>After HO, original SCell = new PCell and original PCell = SCell. In adaptive CA, SCell A2 then manages the old high band (SccA2RsrpThldExtendedOfs; doc −10). Operator off: SpectrumCoordinationSwitch-0. Not a coverage HO; extra HOs raise count, can cut DRX UEs and may drop VoLTE MOS.</t>
+        </is>
+      </c>
+      <c r="C178" s="10" t="n"/>
+      <c r="D178" s="10" t="n"/>
+      <c r="E178" s="10" t="n"/>
+      <c r="F178" s="10" t="n"/>
+      <c r="G178" s="10" t="n"/>
+      <c r="H178" s="10" t="n"/>
+      <c r="I178" s="10" t="n"/>
+      <c r="J178" s="11" t="n"/>
+    </row>
+    <row r="179" ht="37" customHeight="1">
+      <c r="A179" s="35" t="inlineStr">
+        <is>
+          <t>Must-on conditions</t>
+        </is>
+      </c>
+      <c r="B179" s="29" t="inlineStr">
+        <is>
+          <t>HoAdmitSwitch OFF; HoWithSccCfgSwitch ON; SpectrumCoordinationSwitch ON. After enable also ON: CaEnhancedPreAllocSwitch, Dl2CCAckResShareSw, SccA2RmvSwitch. UE must support CA. CA already live (DL 2–8 CC).</t>
+        </is>
+      </c>
+      <c r="C179" s="10" t="n"/>
+      <c r="D179" s="10" t="n"/>
+      <c r="E179" s="10" t="n"/>
+      <c r="F179" s="10" t="n"/>
+      <c r="G179" s="10" t="n"/>
+      <c r="H179" s="10" t="n"/>
+      <c r="I179" s="10" t="n"/>
+      <c r="J179" s="11" t="n"/>
+    </row>
+    <row r="180" ht="37" customHeight="1">
+      <c r="A180" s="35" t="inlineStr">
+        <is>
+          <t>Applicable case</t>
+        </is>
+      </c>
+      <c r="B180" s="9" t="inlineStr">
+        <is>
+          <t>Multi-band CA cluster with overlapping high + low (FPD example 2600 + 850 MHz). Intra-eNodeB. Macro 3900/5900; TDD also LampSite. Not LBBPc.</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="n"/>
+      <c r="D180" s="10" t="n"/>
+      <c r="E180" s="10" t="n"/>
+      <c r="F180" s="10" t="n"/>
+      <c r="G180" s="10" t="n"/>
+      <c r="H180" s="10" t="n"/>
+      <c r="I180" s="10" t="n"/>
+      <c r="J180" s="11" t="n"/>
+    </row>
+    <row r="181" ht="40" customHeight="1">
+      <c r="A181" s="35" t="inlineStr">
+        <is>
+          <t>UL / DL CA limitation</t>
+        </is>
+      </c>
+      <c r="B181" s="29" t="inlineStr">
+        <is>
+          <t>Compatible with DL 2CC–8CC. Does NOT take effect if the UE has 2 CC in UL and 2 CC in DL (UL SCells are never SC targets). If UL is 2 CC and DL is 3–8 CC, it does take effect. This is not UL CA; it only moves which cell is PCell so UL uses the low band.</t>
+        </is>
+      </c>
+      <c r="C181" s="10" t="n"/>
+      <c r="D181" s="10" t="n"/>
+      <c r="E181" s="10" t="n"/>
+      <c r="F181" s="10" t="n"/>
+      <c r="G181" s="10" t="n"/>
+      <c r="H181" s="10" t="n"/>
+      <c r="I181" s="10" t="n"/>
+      <c r="J181" s="11" t="n"/>
+    </row>
+    <row r="182" ht="39" customHeight="1">
+      <c r="A182" s="35" t="inlineStr">
+        <is>
+          <t>GPS required?</t>
+        </is>
+      </c>
+      <c r="B182" s="9" t="inlineStr">
+        <is>
+          <t>No extra GPS requirement in this FPD. SC is an intra-eNodeB PCell change + CA SCell keep. Site sync stays whatever LTE already needs (TDD still needs the site’s existing GPS/1588/sync; SC does not add a GPS license or a new sync feature).</t>
+        </is>
+      </c>
+      <c r="C182" s="10" t="n"/>
+      <c r="D182" s="10" t="n"/>
+      <c r="E182" s="10" t="n"/>
+      <c r="F182" s="10" t="n"/>
+      <c r="G182" s="10" t="n"/>
+      <c r="H182" s="10" t="n"/>
+      <c r="I182" s="10" t="n"/>
+      <c r="J182" s="11" t="n"/>
+    </row>
+    <row r="183" ht="38" customHeight="1">
+      <c r="A183" s="35" t="inlineStr">
+        <is>
+          <t>License (if asked)</t>
+        </is>
+      </c>
+      <c r="B183" s="29" t="inlineStr">
+        <is>
+          <t>FDD LCOFD-131312 model LT1SUNPLTE00 per cell; TDD TDLCOFD-131312 model LT1SLTESPC00 per cell. Enhancement uses the same license. CA licenses still required. License shortage can block ACT CELL.</t>
+        </is>
+      </c>
+      <c r="C183" s="10" t="n"/>
+      <c r="D183" s="10" t="n"/>
+      <c r="E183" s="10" t="n"/>
+      <c r="F183" s="10" t="n"/>
+      <c r="G183" s="10" t="n"/>
+      <c r="H183" s="10" t="n"/>
+      <c r="I183" s="10" t="n"/>
+      <c r="J183" s="11" t="n"/>
+    </row>
+    <row r="184" ht="38" customHeight="1">
+      <c r="A184" s="35" t="inlineStr">
+        <is>
+          <t>How we know it is working</t>
+        </is>
+      </c>
+      <c r="B184" s="9" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.Prep/Exec/Succ (1526729994 / 9996 / 9998) increase. Also watch CA PCell/SCell users and bits, CA UE DL rate, SCell add success (tied to HO success).</t>
+        </is>
+      </c>
+      <c r="C184" s="10" t="n"/>
+      <c r="D184" s="10" t="n"/>
+      <c r="E184" s="10" t="n"/>
+      <c r="F184" s="10" t="n"/>
+      <c r="G184" s="10" t="n"/>
+      <c r="H184" s="10" t="n"/>
+      <c r="I184" s="10" t="n"/>
+      <c r="J184" s="11" t="n"/>
+    </row>
+    <row r="185" ht="41" customHeight="1">
+      <c r="A185" s="35" t="inlineStr">
+        <is>
+          <t>Do not mix / watch-outs</t>
+        </is>
+      </c>
+      <c r="B185" s="29" t="inlineStr">
+        <is>
+          <t>Not DSS, not GSM/UMTS spectrum sharing, not NR UL/DL decoupling. DSS / SUL DSS cut LTE UL RBs → fewer UEs get SC. NSA: may HO PCC off an NSA anchor — deselect SPCT_COORD_INTER_FREQ_HO_SW to exempt NSA UEs. Enhancement (WBB/RRN) is a different bit (WbbCaMultiCarrierCoordSw); NSA PCC anchoring wins over it. SCC coverage-threshold adaptation kills SC carrier management. More HOs; CQI/KPI move with the new PCell quality.</t>
+        </is>
+      </c>
+      <c r="C185" s="10" t="n"/>
+      <c r="D185" s="10" t="n"/>
+      <c r="E185" s="10" t="n"/>
+      <c r="F185" s="10" t="n"/>
+      <c r="G185" s="10" t="n"/>
+      <c r="H185" s="10" t="n"/>
+      <c r="I185" s="10" t="n"/>
+      <c r="J185" s="11" t="n"/>
+    </row>
+    <row r="186" ht="38" customHeight="1">
+      <c r="A186" s="35" t="inlineStr">
+        <is>
+          <t>One-line close</t>
+        </is>
+      </c>
+      <c r="B186" s="9" t="inlineStr">
+        <is>
+          <t>Turn it on only after CA is green on a high/low pair; it does not create CA, it only swaps PCell on poor UL SINR so cell-edge CA UEs keep high-band DL.</t>
+        </is>
+      </c>
+      <c r="C186" s="10" t="n"/>
+      <c r="D186" s="10" t="n"/>
+      <c r="E186" s="10" t="n"/>
+      <c r="F186" s="10" t="n"/>
+      <c r="G186" s="10" t="n"/>
+      <c r="H186" s="10" t="n"/>
+      <c r="I186" s="10" t="n"/>
+      <c r="J186" s="11" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="167">
+  <mergeCells count="163">
     <mergeCell ref="E138:J138"/>
     <mergeCell ref="E143:J143"/>
-    <mergeCell ref="A181:J181"/>
-    <mergeCell ref="A184:J184"/>
     <mergeCell ref="G109:J109"/>
-    <mergeCell ref="E167:J167"/>
+    <mergeCell ref="A156:J156"/>
+    <mergeCell ref="A171:J171"/>
     <mergeCell ref="E149:J149"/>
     <mergeCell ref="A52:J52"/>
-    <mergeCell ref="G119:J119"/>
+    <mergeCell ref="A165:J165"/>
+    <mergeCell ref="B182:J182"/>
     <mergeCell ref="A63:J63"/>
+    <mergeCell ref="G159:J159"/>
+    <mergeCell ref="A155:J155"/>
+    <mergeCell ref="E133:J133"/>
     <mergeCell ref="G111:J111"/>
+    <mergeCell ref="B178:J178"/>
     <mergeCell ref="G72:J72"/>
-    <mergeCell ref="E169:J169"/>
     <mergeCell ref="A173:J173"/>
     <mergeCell ref="G81:J81"/>
     <mergeCell ref="G96:J96"/>
     <mergeCell ref="A34:J34"/>
+    <mergeCell ref="G161:J161"/>
+    <mergeCell ref="A157:J157"/>
     <mergeCell ref="G71:J71"/>
+    <mergeCell ref="B183:J183"/>
     <mergeCell ref="A49:J49"/>
+    <mergeCell ref="B177:J177"/>
     <mergeCell ref="A36:J36"/>
-    <mergeCell ref="E159:J159"/>
+    <mergeCell ref="E125:J125"/>
     <mergeCell ref="C46:J46"/>
-    <mergeCell ref="E164:J164"/>
-    <mergeCell ref="A174:J174"/>
-    <mergeCell ref="E145:J145"/>
+    <mergeCell ref="G160:J160"/>
     <mergeCell ref="E139:J139"/>
-    <mergeCell ref="A183:J183"/>
-    <mergeCell ref="G128:J128"/>
     <mergeCell ref="G66:J66"/>
+    <mergeCell ref="E129:J129"/>
     <mergeCell ref="E142:J142"/>
     <mergeCell ref="E24:J24"/>
-    <mergeCell ref="G121:J121"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="G74:J74"/>
     <mergeCell ref="A55:J55"/>
     <mergeCell ref="G68:J68"/>
+    <mergeCell ref="B180:J180"/>
     <mergeCell ref="G108:J108"/>
+    <mergeCell ref="E131:J131"/>
     <mergeCell ref="E140:J140"/>
-    <mergeCell ref="E171:J171"/>
     <mergeCell ref="G114:J114"/>
     <mergeCell ref="E153:J153"/>
-    <mergeCell ref="A175:J175"/>
-    <mergeCell ref="G123:J123"/>
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="G110:J110"/>
-    <mergeCell ref="E155:J155"/>
     <mergeCell ref="E137:J137"/>
     <mergeCell ref="G113:J113"/>
     <mergeCell ref="G91:J91"/>
+    <mergeCell ref="B179:J179"/>
     <mergeCell ref="A29:J29"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="G85:J85"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="G94:J94"/>
-    <mergeCell ref="E157:J157"/>
-    <mergeCell ref="E166:J166"/>
+    <mergeCell ref="A170:J170"/>
     <mergeCell ref="G75:J75"/>
     <mergeCell ref="G84:J84"/>
     <mergeCell ref="A31:J31"/>
     <mergeCell ref="A58:J58"/>
+    <mergeCell ref="B186:J186"/>
     <mergeCell ref="A40:J40"/>
     <mergeCell ref="G77:J77"/>
-    <mergeCell ref="A186:J186"/>
-    <mergeCell ref="E168:J168"/>
     <mergeCell ref="G86:J86"/>
     <mergeCell ref="A82:J82"/>
-    <mergeCell ref="G178:J178"/>
     <mergeCell ref="A60:J60"/>
     <mergeCell ref="G67:J67"/>
     <mergeCell ref="E136:J136"/>
     <mergeCell ref="G70:J70"/>
     <mergeCell ref="G97:J97"/>
-    <mergeCell ref="G125:J125"/>
     <mergeCell ref="A172:J172"/>
-    <mergeCell ref="A187:J187"/>
     <mergeCell ref="G112:J112"/>
-    <mergeCell ref="G127:J127"/>
-    <mergeCell ref="A189:J189"/>
+    <mergeCell ref="E122:J122"/>
+    <mergeCell ref="B185:J185"/>
+    <mergeCell ref="E127:J127"/>
     <mergeCell ref="E23:J23"/>
     <mergeCell ref="A50:J50"/>
-    <mergeCell ref="G177:J177"/>
+    <mergeCell ref="B184:J184"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B176:J176"/>
     <mergeCell ref="G104:J104"/>
     <mergeCell ref="A42:J42"/>
     <mergeCell ref="E147:J147"/>
     <mergeCell ref="A47:J47"/>
-    <mergeCell ref="E156:J156"/>
-    <mergeCell ref="E170:J170"/>
     <mergeCell ref="G88:J88"/>
+    <mergeCell ref="E128:J128"/>
     <mergeCell ref="A62:J62"/>
-    <mergeCell ref="G129:J129"/>
+    <mergeCell ref="A144:J144"/>
     <mergeCell ref="A20:J20"/>
     <mergeCell ref="G76:J76"/>
     <mergeCell ref="G90:J90"/>
-    <mergeCell ref="A134:J134"/>
     <mergeCell ref="A28:J28"/>
     <mergeCell ref="G99:J99"/>
     <mergeCell ref="E148:J148"/>
-    <mergeCell ref="G131:J131"/>
+    <mergeCell ref="A167:J167"/>
     <mergeCell ref="A30:J30"/>
-    <mergeCell ref="E154:J154"/>
     <mergeCell ref="A59:J59"/>
     <mergeCell ref="G115:J115"/>
-    <mergeCell ref="G130:J130"/>
-    <mergeCell ref="A182:J182"/>
+    <mergeCell ref="E119:J119"/>
     <mergeCell ref="A64:J64"/>
-    <mergeCell ref="G117:J117"/>
+    <mergeCell ref="A169:J169"/>
     <mergeCell ref="A51:J51"/>
     <mergeCell ref="E25:J25"/>
-    <mergeCell ref="G179:J179"/>
     <mergeCell ref="A61:J61"/>
-    <mergeCell ref="G126:J126"/>
-    <mergeCell ref="G132:J132"/>
-    <mergeCell ref="G122:J122"/>
     <mergeCell ref="A162:J162"/>
     <mergeCell ref="E146:J146"/>
-    <mergeCell ref="G116:J116"/>
     <mergeCell ref="A54:J54"/>
+    <mergeCell ref="E121:J121"/>
     <mergeCell ref="G103:J103"/>
     <mergeCell ref="A41:J41"/>
+    <mergeCell ref="E130:J130"/>
     <mergeCell ref="E151:J151"/>
-    <mergeCell ref="E160:J160"/>
+    <mergeCell ref="A164:J164"/>
     <mergeCell ref="G78:J78"/>
-    <mergeCell ref="G118:J118"/>
     <mergeCell ref="A56:J56"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="G87:J87"/>
+    <mergeCell ref="E123:J123"/>
     <mergeCell ref="E150:J150"/>
+    <mergeCell ref="A154:J154"/>
+    <mergeCell ref="E132:J132"/>
+    <mergeCell ref="A163:J163"/>
     <mergeCell ref="A101:J101"/>
     <mergeCell ref="G80:J80"/>
     <mergeCell ref="G95:J95"/>
     <mergeCell ref="A33:J33"/>
     <mergeCell ref="G89:J89"/>
+    <mergeCell ref="A116:J116"/>
     <mergeCell ref="E152:J152"/>
-    <mergeCell ref="E161:J161"/>
     <mergeCell ref="G79:J79"/>
-    <mergeCell ref="A188:J188"/>
     <mergeCell ref="G73:J73"/>
     <mergeCell ref="A100:J100"/>
     <mergeCell ref="A53:J53"/>
+    <mergeCell ref="E118:J118"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A180:J180"/>
-    <mergeCell ref="E158:J158"/>
+    <mergeCell ref="B181:J181"/>
+    <mergeCell ref="B175:J175"/>
     <mergeCell ref="C45:J45"/>
     <mergeCell ref="G106:J106"/>
     <mergeCell ref="G105:J105"/>
     <mergeCell ref="A39:J39"/>
+    <mergeCell ref="A166:J166"/>
     <mergeCell ref="C44:J44"/>
     <mergeCell ref="A48:J48"/>
-    <mergeCell ref="E144:J144"/>
-    <mergeCell ref="G120:J120"/>
+    <mergeCell ref="E124:J124"/>
     <mergeCell ref="G98:J98"/>
+    <mergeCell ref="E120:J120"/>
     <mergeCell ref="G107:J107"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="E134:J134"/>
+    <mergeCell ref="A168:J168"/>
     <mergeCell ref="G93:J93"/>
     <mergeCell ref="A37:J37"/>
     <mergeCell ref="G69:J69"/>
-    <mergeCell ref="E165:J165"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="G92:J92"/>
+    <mergeCell ref="E126:J126"/>
     <mergeCell ref="E141:J141"/>
     <mergeCell ref="A26:J26"/>
     <mergeCell ref="A57:J57"/>
-    <mergeCell ref="G124:J124"/>
-    <mergeCell ref="G133:J133"/>
-    <mergeCell ref="A185:J185"/>
+    <mergeCell ref="E135:J135"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Clarify Spectrum Coordination meeting close in plain English
Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Carrier_Aggregation_Deployment.xlsx
+++ b/Carrier_Aggregation_Deployment.xlsx
@@ -27511,7 +27511,7 @@
       <c r="I174" s="7" t="inlineStr"/>
       <c r="J174" s="7" t="inlineStr"/>
     </row>
-    <row r="175" ht="40" customHeight="1">
+    <row r="175" ht="52" customHeight="1">
       <c r="A175" s="35" t="inlineStr">
         <is>
           <t>What it is (10 s)</t>
@@ -27531,7 +27531,7 @@
       <c r="I175" s="10" t="n"/>
       <c r="J175" s="11" t="n"/>
     </row>
-    <row r="176" ht="41" customHeight="1">
+    <row r="176" ht="52" customHeight="1">
       <c r="A176" s="35" t="inlineStr">
         <is>
           <t>Benefit (1–2 lines)</t>
@@ -27551,7 +27551,7 @@
       <c r="I176" s="10" t="n"/>
       <c r="J176" s="11" t="n"/>
     </row>
-    <row r="177" ht="40" customHeight="1">
+    <row r="177" ht="52" customHeight="1">
       <c r="A177" s="35" t="inlineStr">
         <is>
           <t>Trigger</t>
@@ -27571,7 +27571,7 @@
       <c r="I177" s="10" t="n"/>
       <c r="J177" s="11" t="n"/>
     </row>
-    <row r="178" ht="39" customHeight="1">
+    <row r="178" ht="52" customHeight="1">
       <c r="A178" s="35" t="inlineStr">
         <is>
           <t>Leave / after HO</t>
@@ -27591,7 +27591,7 @@
       <c r="I178" s="10" t="n"/>
       <c r="J178" s="11" t="n"/>
     </row>
-    <row r="179" ht="37" customHeight="1">
+    <row r="179" ht="52" customHeight="1">
       <c r="A179" s="35" t="inlineStr">
         <is>
           <t>Must-on conditions</t>
@@ -27611,7 +27611,7 @@
       <c r="I179" s="10" t="n"/>
       <c r="J179" s="11" t="n"/>
     </row>
-    <row r="180" ht="37" customHeight="1">
+    <row r="180" ht="52" customHeight="1">
       <c r="A180" s="35" t="inlineStr">
         <is>
           <t>Applicable case</t>
@@ -27631,7 +27631,7 @@
       <c r="I180" s="10" t="n"/>
       <c r="J180" s="11" t="n"/>
     </row>
-    <row r="181" ht="40" customHeight="1">
+    <row r="181" ht="52" customHeight="1">
       <c r="A181" s="35" t="inlineStr">
         <is>
           <t>UL / DL CA limitation</t>
@@ -27651,7 +27651,7 @@
       <c r="I181" s="10" t="n"/>
       <c r="J181" s="11" t="n"/>
     </row>
-    <row r="182" ht="39" customHeight="1">
+    <row r="182" ht="52" customHeight="1">
       <c r="A182" s="35" t="inlineStr">
         <is>
           <t>GPS required?</t>
@@ -27671,7 +27671,7 @@
       <c r="I182" s="10" t="n"/>
       <c r="J182" s="11" t="n"/>
     </row>
-    <row r="183" ht="38" customHeight="1">
+    <row r="183" ht="52" customHeight="1">
       <c r="A183" s="35" t="inlineStr">
         <is>
           <t>License (if asked)</t>
@@ -27691,7 +27691,7 @@
       <c r="I183" s="10" t="n"/>
       <c r="J183" s="11" t="n"/>
     </row>
-    <row r="184" ht="38" customHeight="1">
+    <row r="184" ht="52" customHeight="1">
       <c r="A184" s="35" t="inlineStr">
         <is>
           <t>How we know it is working</t>
@@ -27711,7 +27711,7 @@
       <c r="I184" s="10" t="n"/>
       <c r="J184" s="11" t="n"/>
     </row>
-    <row r="185" ht="41" customHeight="1">
+    <row r="185" ht="52" customHeight="1">
       <c r="A185" s="35" t="inlineStr">
         <is>
           <t>Do not mix / watch-outs</t>
@@ -27731,15 +27731,19 @@
       <c r="I185" s="10" t="n"/>
       <c r="J185" s="11" t="n"/>
     </row>
-    <row r="186" ht="38" customHeight="1">
+    <row r="186" ht="118" customHeight="1">
       <c r="A186" s="35" t="inlineStr">
         <is>
-          <t>One-line close</t>
+          <t>Plain-English close  (read this if the jargon is heavy)</t>
         </is>
       </c>
       <c r="B186" s="9" t="inlineStr">
         <is>
-          <t>Turn it on only after CA is green on a high/low pair; it does not create CA, it only swaps PCell on poor UL SINR so cell-edge CA UEs keep high-band DL.</t>
+          <t>1) First make normal Carrier Aggregation work between one high-frequency cell and one low-frequency cell (same site, overlapping coverage). If CA is not working, do not turn Spectrum Coordination on.
+2) Spectrum Coordination does not join two carriers by itself. CA already joined them. This feature only changes which of those two cells is the PCell (the cell that carries the uplink).
+3) When the UE is near the cell edge, uplink on the high band is weak (poor UL SINR). The eNodeB then makes the low-band cell the PCell so the UE transmits uplink on the low band (better coverage).
+4) The high-band cell is kept as an SCell, so downlink data can still use both bands. That is the gain: cell-edge users keep high-band download speed even when their upload cannot stay on the high band.
+5) Short version: CA = two pipes for download. Spectrum Coordination = move the upload pipe to the low band at the edge, without throwing away the high-band download pipe.</t>
         </is>
       </c>
       <c r="C186" s="10" t="n"/>

</xml_diff>

<commit_message>
Explain PCell swap: existing SCell target vs multi-SCell pick, UL vs DL
Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Carrier_Aggregation_Deployment.xlsx
+++ b/Carrier_Aggregation_Deployment.xlsx
@@ -23050,7 +23050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -27519,7 +27519,7 @@
       </c>
       <c r="B175" s="29" t="inlineStr">
         <is>
-          <t>LTE Spectrum Coordination is a CA companion: when a CA UE sits at the high-band UL edge, the eNodeB HOs the PCell to a better low-band SCell and keeps the old PCell as SCell, so DL still uses both bands while UL rides the coverage layer. Feature IDs: LCOFD-131312 (FDD) / TDLCOFD-131312 (TDD). Same for FDD and TDD.</t>
+          <t>The UE is already in CA: PCell = high band (upload + download), SCell = low band (download extra). If upload on the high-band PCell becomes too weak, the eNodeB does an inter-frequency handover: the low-band SCell becomes the new PCell, and the old high-band PCell is immediately kept as an SCell. Feature IDs: LCOFD-131312 (FDD) / TDLCOFD-131312 (TDD). Same for FDD and TDD.</t>
         </is>
       </c>
       <c r="C175" s="10" t="n"/>
@@ -27534,12 +27534,12 @@
     <row r="176" ht="52" customHeight="1">
       <c r="A176" s="35" t="inlineStr">
         <is>
-          <t>Benefit (1–2 lines)</t>
+          <t>Q1. Is the low-band SCell already configured with this PCell?</t>
         </is>
       </c>
       <c r="B176" s="9" t="inlineStr">
         <is>
-          <t>It lifts DL usage of CA UEs at the high-frequency UL coverage edge. Best when high/low gap is large. Scenario 1 (both bands already on): PUSCH MCS 0–3 &gt;10% on high band, low-minus-high UL interference &lt;5 dB, CA UE penetration &gt;25% → network User DL Average Throughput up. Scenario 2 (adding a new low band under an existing high band) → both User DL and User UL Average Throughput up.</t>
+          <t>YES. The FPD starts from a UE already in the CA state. The eNodeB only looks at that UE’s existing downlink SCells — it does not add a new neighbor from outside CA at this step. Example in Figure 4-1: before the swap, PCell is already 2600 MHz and SCell is already 850 MHz.</t>
         </is>
       </c>
       <c r="C176" s="10" t="n"/>
@@ -27554,12 +27554,12 @@
     <row r="177" ht="52" customHeight="1">
       <c r="A177" s="35" t="inlineStr">
         <is>
-          <t>Trigger</t>
+          <t>Q2. If the UE has several SCells, which one becomes the new PCell?</t>
         </is>
       </c>
       <c r="B177" s="29" t="inlineStr">
         <is>
-          <t>CA UE already aggregating. UL SINR used in scheduling (initial MCS) &lt; SpectrumCoordSinrThld (doc MML −2 dB). Then a DL SCell must pass A4 AND be stronger than all its intra-freq neighbours, and must be allowed as PCell. Target pick: PCell/PCC priority → largest BW → lowest EARFCN (or DL air-interface capability first if intelligent selection is ON).</t>
+          <t>Only SCells that pass ALL of: (a) better uplink than the current PCell, (b) DL RSRP reaches CA event A4, (c) stronger than all intra-frequency neighbors of that SCell, (d) allowed to be a PCell. If only one SCell passes → HO to that one. If two or more pass → pick by rule: highest PCell/PCC priority, then largest bandwidth, then lowest EARFCN. If intelligent selection is ON, DL air-interface capability is used first, then the same ties. UL SCells are never chosen as the target.</t>
         </is>
       </c>
       <c r="C177" s="10" t="n"/>
@@ -27571,15 +27571,19 @@
       <c r="I177" s="10" t="n"/>
       <c r="J177" s="11" t="n"/>
     </row>
-    <row r="178" ht="52" customHeight="1">
+    <row r="178" ht="118" customHeight="1">
       <c r="A178" s="35" t="inlineStr">
         <is>
-          <t>Leave / after HO</t>
+          <t>What “DL still uses both bands, UL rides the coverage layer” means</t>
         </is>
       </c>
       <c r="B178" s="9" t="inlineStr">
         <is>
-          <t>After HO, original SCell = new PCell and original PCell = SCell. In adaptive CA, SCell A2 then manages the old high band (SccA2RsrpThldExtendedOfs; doc −10). Operator off: SpectrumCoordinationSwitch-0. Not a coverage HO; extra HOs raise count, can cut DRX UEs and may drop VoLTE MOS.</t>
+          <t>Coverage layer = low frequency (better uplink reach). Capacity layer = high frequency (more downlink speed, weaker uplink at the edge).
+In normal LTE CA without UL CA, upload (PUSCH/PUCCH) is only on the PCell. Download can use PCell + SCell.
+BEFORE swap: PCell=high band → upload is on high band (often too weak at the edge); download = high + low.
+AFTER swap: PCell=low band → upload is on low band (coverage layer, stronger); the high band is still an SCell so download is still high + low.
+So download does not lose the high band. Only the upload home cell changes. That is why cell-edge users can keep high-band download while their upload survives.</t>
         </is>
       </c>
       <c r="C178" s="10" t="n"/>
@@ -27594,12 +27598,12 @@
     <row r="179" ht="52" customHeight="1">
       <c r="A179" s="35" t="inlineStr">
         <is>
-          <t>Must-on conditions</t>
+          <t>Benefit (1–2 lines)</t>
         </is>
       </c>
       <c r="B179" s="29" t="inlineStr">
         <is>
-          <t>HoAdmitSwitch OFF; HoWithSccCfgSwitch ON; SpectrumCoordinationSwitch ON. After enable also ON: CaEnhancedPreAllocSwitch, Dl2CCAckResShareSw, SccA2RmvSwitch. UE must support CA. CA already live (DL 2–8 CC).</t>
+          <t>It lifts DL usage of CA UEs at the high-frequency UL coverage edge. Best when high/low gap is large. Scenario 1 (both bands already on): PUSCH MCS 0–3 &gt;10% on high band, low-minus-high UL interference &lt;5 dB, CA UE penetration &gt;25% → network User DL Average Throughput up. Scenario 2 (adding a new low band under an existing high band) → both User DL and User UL Average Throughput up.</t>
         </is>
       </c>
       <c r="C179" s="10" t="n"/>
@@ -27614,12 +27618,12 @@
     <row r="180" ht="52" customHeight="1">
       <c r="A180" s="35" t="inlineStr">
         <is>
-          <t>Applicable case</t>
+          <t>Trigger</t>
         </is>
       </c>
       <c r="B180" s="9" t="inlineStr">
         <is>
-          <t>Multi-band CA cluster with overlapping high + low (FPD example 2600 + 850 MHz). Intra-eNodeB. Macro 3900/5900; TDD also LampSite. Not LBBPc.</t>
+          <t>CA UE already aggregating. UL SINR used in scheduling (initial MCS) &lt; SpectrumCoordSinrThld (doc MML −2 dB). Then a DL SCell must pass A4 AND be stronger than all its intra-freq neighbours, and must be allowed as PCell. Target pick: PCell/PCC priority → largest BW → lowest EARFCN (or DL air-interface capability first if intelligent selection is ON).</t>
         </is>
       </c>
       <c r="C180" s="10" t="n"/>
@@ -27634,12 +27638,12 @@
     <row r="181" ht="52" customHeight="1">
       <c r="A181" s="35" t="inlineStr">
         <is>
-          <t>UL / DL CA limitation</t>
+          <t>Leave / after HO</t>
         </is>
       </c>
       <c r="B181" s="29" t="inlineStr">
         <is>
-          <t>Compatible with DL 2CC–8CC. Does NOT take effect if the UE has 2 CC in UL and 2 CC in DL (UL SCells are never SC targets). If UL is 2 CC and DL is 3–8 CC, it does take effect. This is not UL CA; it only moves which cell is PCell so UL uses the low band.</t>
+          <t>After HO, original SCell = new PCell and original PCell = SCell. In adaptive CA, SCell A2 then manages the old high band (SccA2RsrpThldExtendedOfs; doc −10). Operator off: SpectrumCoordinationSwitch-0. Not a coverage HO; extra HOs raise count, can cut DRX UEs and may drop VoLTE MOS.</t>
         </is>
       </c>
       <c r="C181" s="10" t="n"/>
@@ -27654,12 +27658,12 @@
     <row r="182" ht="52" customHeight="1">
       <c r="A182" s="35" t="inlineStr">
         <is>
-          <t>GPS required?</t>
+          <t>Must-on conditions</t>
         </is>
       </c>
       <c r="B182" s="9" t="inlineStr">
         <is>
-          <t>No extra GPS requirement in this FPD. SC is an intra-eNodeB PCell change + CA SCell keep. Site sync stays whatever LTE already needs (TDD still needs the site’s existing GPS/1588/sync; SC does not add a GPS license or a new sync feature).</t>
+          <t>HoAdmitSwitch OFF; HoWithSccCfgSwitch ON; SpectrumCoordinationSwitch ON. After enable also ON: CaEnhancedPreAllocSwitch, Dl2CCAckResShareSw, SccA2RmvSwitch. UE must support CA. CA already live (DL 2–8 CC).</t>
         </is>
       </c>
       <c r="C182" s="10" t="n"/>
@@ -27674,12 +27678,12 @@
     <row r="183" ht="52" customHeight="1">
       <c r="A183" s="35" t="inlineStr">
         <is>
-          <t>License (if asked)</t>
+          <t>Applicable case</t>
         </is>
       </c>
       <c r="B183" s="29" t="inlineStr">
         <is>
-          <t>FDD LCOFD-131312 model LT1SUNPLTE00 per cell; TDD TDLCOFD-131312 model LT1SLTESPC00 per cell. Enhancement uses the same license. CA licenses still required. License shortage can block ACT CELL.</t>
+          <t>Multi-band CA cluster with overlapping high + low (FPD example 2600 + 850 MHz). Intra-eNodeB. Macro 3900/5900; TDD also LampSite. Not LBBPc.</t>
         </is>
       </c>
       <c r="C183" s="10" t="n"/>
@@ -27694,12 +27698,12 @@
     <row r="184" ht="52" customHeight="1">
       <c r="A184" s="35" t="inlineStr">
         <is>
-          <t>How we know it is working</t>
+          <t>UL / DL CA limitation</t>
         </is>
       </c>
       <c r="B184" s="9" t="inlineStr">
         <is>
-          <t>L.HHO.InterFreq.ULquality.Prep/Exec/Succ (1526729994 / 9996 / 9998) increase. Also watch CA PCell/SCell users and bits, CA UE DL rate, SCell add success (tied to HO success).</t>
+          <t>Compatible with DL 2CC–8CC. Does NOT take effect if the UE has 2 CC in UL and 2 CC in DL (UL SCells are never SC targets). If UL is 2 CC and DL is 3–8 CC, it does take effect. This is not UL CA; it only moves which cell is PCell so UL uses the low band.</t>
         </is>
       </c>
       <c r="C184" s="10" t="n"/>
@@ -27714,12 +27718,12 @@
     <row r="185" ht="52" customHeight="1">
       <c r="A185" s="35" t="inlineStr">
         <is>
-          <t>Do not mix / watch-outs</t>
+          <t>GPS required?</t>
         </is>
       </c>
       <c r="B185" s="29" t="inlineStr">
         <is>
-          <t>Not DSS, not GSM/UMTS spectrum sharing, not NR UL/DL decoupling. DSS / SUL DSS cut LTE UL RBs → fewer UEs get SC. NSA: may HO PCC off an NSA anchor — deselect SPCT_COORD_INTER_FREQ_HO_SW to exempt NSA UEs. Enhancement (WBB/RRN) is a different bit (WbbCaMultiCarrierCoordSw); NSA PCC anchoring wins over it. SCC coverage-threshold adaptation kills SC carrier management. More HOs; CQI/KPI move with the new PCell quality.</t>
+          <t>No extra GPS requirement in this FPD. SC is an intra-eNodeB PCell change + CA SCell keep. Site sync stays whatever LTE already needs (TDD still needs the site’s existing GPS/1588/sync; SC does not add a GPS license or a new sync feature).</t>
         </is>
       </c>
       <c r="C185" s="10" t="n"/>
@@ -27731,19 +27735,15 @@
       <c r="I185" s="10" t="n"/>
       <c r="J185" s="11" t="n"/>
     </row>
-    <row r="186" ht="118" customHeight="1">
+    <row r="186" ht="52" customHeight="1">
       <c r="A186" s="35" t="inlineStr">
         <is>
-          <t>Plain-English close  (read this if the jargon is heavy)</t>
+          <t>License (if asked)</t>
         </is>
       </c>
       <c r="B186" s="9" t="inlineStr">
         <is>
-          <t>1) First make normal Carrier Aggregation work between one high-frequency cell and one low-frequency cell (same site, overlapping coverage). If CA is not working, do not turn Spectrum Coordination on.
-2) Spectrum Coordination does not join two carriers by itself. CA already joined them. This feature only changes which of those two cells is the PCell (the cell that carries the uplink).
-3) When the UE is near the cell edge, uplink on the high band is weak (poor UL SINR). The eNodeB then makes the low-band cell the PCell so the UE transmits uplink on the low band (better coverage).
-4) The high-band cell is kept as an SCell, so downlink data can still use both bands. That is the gain: cell-edge users keep high-band download speed even when their upload cannot stay on the high band.
-5) Short version: CA = two pipes for download. Spectrum Coordination = move the upload pipe to the low band at the edge, without throwing away the high-band download pipe.</t>
+          <t>FDD LCOFD-131312 model LT1SUNPLTE00 per cell; TDD TDLCOFD-131312 model LT1SLTESPC00 per cell. Enhancement uses the same license. CA licenses still required. License shortage can block ACT CELL.</t>
         </is>
       </c>
       <c r="C186" s="10" t="n"/>
@@ -27755,8 +27755,72 @@
       <c r="I186" s="10" t="n"/>
       <c r="J186" s="11" t="n"/>
     </row>
+    <row r="187" ht="52" customHeight="1">
+      <c r="A187" s="35" t="inlineStr">
+        <is>
+          <t>How we know it is working</t>
+        </is>
+      </c>
+      <c r="B187" s="29" t="inlineStr">
+        <is>
+          <t>L.HHO.InterFreq.ULquality.Prep/Exec/Succ (1526729994 / 9996 / 9998) increase. Also watch CA PCell/SCell users and bits, CA UE DL rate, SCell add success (tied to HO success).</t>
+        </is>
+      </c>
+      <c r="C187" s="10" t="n"/>
+      <c r="D187" s="10" t="n"/>
+      <c r="E187" s="10" t="n"/>
+      <c r="F187" s="10" t="n"/>
+      <c r="G187" s="10" t="n"/>
+      <c r="H187" s="10" t="n"/>
+      <c r="I187" s="10" t="n"/>
+      <c r="J187" s="11" t="n"/>
+    </row>
+    <row r="188" ht="52" customHeight="1">
+      <c r="A188" s="35" t="inlineStr">
+        <is>
+          <t>Do not mix / watch-outs</t>
+        </is>
+      </c>
+      <c r="B188" s="9" t="inlineStr">
+        <is>
+          <t>Not DSS, not GSM/UMTS spectrum sharing, not NR UL/DL decoupling. DSS / SUL DSS cut LTE UL RBs → fewer UEs get SC. NSA: may HO PCC off an NSA anchor — deselect SPCT_COORD_INTER_FREQ_HO_SW to exempt NSA UEs. Enhancement (WBB/RRN) is a different bit (WbbCaMultiCarrierCoordSw); NSA PCC anchoring wins over it. SCC coverage-threshold adaptation kills SC carrier management. More HOs; CQI/KPI move with the new PCell quality.</t>
+        </is>
+      </c>
+      <c r="C188" s="10" t="n"/>
+      <c r="D188" s="10" t="n"/>
+      <c r="E188" s="10" t="n"/>
+      <c r="F188" s="10" t="n"/>
+      <c r="G188" s="10" t="n"/>
+      <c r="H188" s="10" t="n"/>
+      <c r="I188" s="10" t="n"/>
+      <c r="J188" s="11" t="n"/>
+    </row>
+    <row r="189" ht="118" customHeight="1">
+      <c r="A189" s="35" t="inlineStr">
+        <is>
+          <t>Plain-English close  (read this if the jargon is heavy)</t>
+        </is>
+      </c>
+      <c r="B189" s="29" t="inlineStr">
+        <is>
+          <t>1) First make normal Carrier Aggregation work between one high-frequency cell and one low-frequency cell (same site, overlapping coverage). If CA is not working, do not turn Spectrum Coordination on.
+2) Spectrum Coordination does not join two carriers by itself. CA already joined them. This feature only changes which of those two cells is the PCell (the cell that carries the uplink).
+3) When the UE is near the cell edge, uplink on the high band is weak (poor UL SINR). The eNodeB then makes the low-band cell the PCell so the UE transmits uplink on the low band (better coverage).
+4) The high-band cell is kept as an SCell, so downlink data can still use both bands. That is the gain: cell-edge users keep high-band download speed even when their upload cannot stay on the high band.
+5) Short version: CA = two pipes for download. Spectrum Coordination = move the upload pipe to the low band at the edge, without throwing away the high-band download pipe.</t>
+        </is>
+      </c>
+      <c r="C189" s="10" t="n"/>
+      <c r="D189" s="10" t="n"/>
+      <c r="E189" s="10" t="n"/>
+      <c r="F189" s="10" t="n"/>
+      <c r="G189" s="10" t="n"/>
+      <c r="H189" s="10" t="n"/>
+      <c r="I189" s="10" t="n"/>
+      <c r="J189" s="11" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="163">
+  <mergeCells count="166">
     <mergeCell ref="E138:J138"/>
     <mergeCell ref="E143:J143"/>
     <mergeCell ref="G109:J109"/>
@@ -27858,13 +27922,16 @@
     <mergeCell ref="A59:J59"/>
     <mergeCell ref="G115:J115"/>
     <mergeCell ref="E119:J119"/>
+    <mergeCell ref="B187:J187"/>
     <mergeCell ref="A64:J64"/>
     <mergeCell ref="A169:J169"/>
     <mergeCell ref="A51:J51"/>
     <mergeCell ref="E25:J25"/>
     <mergeCell ref="A61:J61"/>
+    <mergeCell ref="B189:J189"/>
     <mergeCell ref="A162:J162"/>
     <mergeCell ref="E146:J146"/>
+    <mergeCell ref="B188:J188"/>
     <mergeCell ref="A54:J54"/>
     <mergeCell ref="E121:J121"/>
     <mergeCell ref="G103:J103"/>

</xml_diff>

<commit_message>
Name CA Event A4 and intelligent-selection params in the workbook
Replace informal “event A4” / “DL capability” wording with FPD MOs:
PCellA4RsrpThd/PccA4RsrpThd for SC target, CarrAggrA4ThdRsrp for SCell add,
CaSmartSelectionSwitch and MinDlAvgToBeScheduledUeNum for pick order.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Carrier_Aggregation_Deployment.xlsx
+++ b/Carrier_Aggregation_Deployment.xlsx
@@ -4486,7 +4486,7 @@
       <c r="I137" s="7" t="inlineStr"/>
       <c r="J137" s="7" t="inlineStr"/>
     </row>
-    <row r="138" ht="42" customHeight="1">
+    <row r="138" ht="56" customHeight="1">
       <c r="A138" s="9" t="inlineStr">
         <is>
           <t>A1</t>
@@ -4514,7 +4514,7 @@
       <c r="I138" s="10" t="n"/>
       <c r="J138" s="11" t="n"/>
     </row>
-    <row r="139" ht="42" customHeight="1">
+    <row r="139" ht="56" customHeight="1">
       <c r="A139" s="12" t="inlineStr">
         <is>
           <t>A2</t>
@@ -4542,7 +4542,7 @@
       <c r="I139" s="10" t="n"/>
       <c r="J139" s="11" t="n"/>
     </row>
-    <row r="140" ht="42" customHeight="1">
+    <row r="140" ht="56" customHeight="1">
       <c r="A140" s="9" t="inlineStr">
         <is>
           <t>A3</t>
@@ -4570,7 +4570,7 @@
       <c r="I140" s="10" t="n"/>
       <c r="J140" s="11" t="n"/>
     </row>
-    <row r="141" ht="42" customHeight="1">
+    <row r="141" ht="56" customHeight="1">
       <c r="A141" s="12" t="inlineStr">
         <is>
           <t>A4</t>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="D141" s="12" t="inlineStr">
         <is>
-          <t>SCell add (measurement-based). Threshold = CarrAggrA4ThdRsrp + SCell/SCC A4 offset [+ extended Ofs]</t>
+          <t>Three different A4 MOs: (1) CA SCell-add = CaMgtCfg.CarrAggrA4ThdRsrp + CaGroupSCellCfg.SCellA4Offset or SccFreqCfg.SccA4Offset [+ SccA2RsrpThldExtendedOfs]; (2) SC/PCC-anchor target = CaGroupCell.PCellA4RsrpThd or PccFreqCfg.PccA4RsrpThd; (3) coverage HO = InterFreqHoGroup.InterFreqHoA4ThdRsrp</t>
         </is>
       </c>
       <c r="E141" s="10" t="n"/>
@@ -4598,7 +4598,7 @@
       <c r="I141" s="10" t="n"/>
       <c r="J141" s="11" t="n"/>
     </row>
-    <row r="142" ht="42" customHeight="1">
+    <row r="142" ht="56" customHeight="1">
       <c r="A142" s="9" t="inlineStr">
         <is>
           <t>A5</t>
@@ -4626,7 +4626,7 @@
       <c r="I142" s="10" t="n"/>
       <c r="J142" s="11" t="n"/>
     </row>
-    <row r="143" ht="42" customHeight="1">
+    <row r="143" ht="56" customHeight="1">
       <c r="A143" s="12" t="inlineStr">
         <is>
           <t>A6</t>
@@ -4903,7 +4903,7 @@
       <c r="I4" s="7" t="inlineStr"/>
       <c r="J4" s="7" t="inlineStr"/>
     </row>
-    <row r="5" ht="52" customHeight="1">
+    <row r="5" ht="64" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
         <is>
           <t>How enabled</t>
@@ -4935,7 +4935,7 @@
       <c r="I5" s="10" t="n"/>
       <c r="J5" s="11" t="n"/>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>What you define</t>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Best DL 2–5 / UL 2 combination from load, coverage, UE capability</t>
+          <t>CaSmartSelectionSwitch ON: first use highest DL air interface capability (CaMgtCfg.MinDlAvgToBeScheduledUeNum: P×SF×SE−G or (P×SF×SE−G)/N)</t>
         </is>
       </c>
       <c r="F6" s="10" t="n"/>
@@ -4967,7 +4967,7 @@
       <c r="I6" s="10" t="n"/>
       <c r="J6" s="11" t="n"/>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Who can aggregate</t>
@@ -4999,7 +4999,7 @@
       <c r="I7" s="10" t="n"/>
       <c r="J7" s="11" t="n"/>
     </row>
-    <row r="8" ht="52" customHeight="1">
+    <row r="8" ht="64" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Blind SCell</t>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>SmartCaFastSccCfgSwitch tries blind add during intelligent selection</t>
+          <t>SmartCaFastSccCfgSwitch tries blind add while CaSmartSelectionSwitch is ON</t>
         </is>
       </c>
       <c r="F8" s="10" t="n"/>
@@ -5031,7 +5031,7 @@
       <c r="I8" s="10" t="n"/>
       <c r="J8" s="11" t="n"/>
     </row>
-    <row r="9" ht="52" customHeight="1">
+    <row r="9" ht="64" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Route / capacity</t>
@@ -5063,7 +5063,7 @@
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="11" t="n"/>
     </row>
-    <row r="10" ht="52" customHeight="1">
+    <row r="10" ht="64" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
           <t>License character</t>
@@ -5095,7 +5095,7 @@
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="11" t="n"/>
     </row>
-    <row r="11" ht="52" customHeight="1">
+    <row r="11" ht="64" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>When to use</t>
@@ -5295,10 +5295,10 @@
       <c r="I41" s="6" t="n"/>
       <c r="J41" s="6" t="n"/>
     </row>
-    <row r="42" ht="41" customHeight="1">
+    <row r="42" ht="110" customHeight="1">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>Ch.12: the eNodeB selects DL combinations (2–5 CC) and UL combinations (2 CC) using triggers (traffic / measurement), UE capability, coverage overlap and load — rather than a static priority list alone. Requires CaSmartSelectionSwitch. When this switch is ON, PCC frequency count is capped at 9. SmartCaFastSccCfgSwitch (CaAlgoExtSwitch) can try blind SCell configuration to shorten time-to-CA; it requires CaSmartSelectionSwitch ON. Does not take effect together with some PCC-anchoring enhancements (e.g. UlCaCapbBasedPccSelectionSw).</t>
+          <t>Ch.12: the eNodeB selects DL combinations (2–5 CC) and UL combinations (2 CC) using triggers (traffic / measurement), UE capability, coverage overlap and load — rather than a static priority list alone. Switch: ENodeBAlgoSwitch.CaAlgoSwitch / CaSmartSelectionSwitch. When ON, PCC frequency count is capped at 9, and the first pick among candidate serving cells is highest downlink air interface capability: if CaMgtCfg.MinDlAvgToBeScheduledUeNum=0 then P×SF×SE−G, else (P×SF×SE−G)/N (P=L.ChMeas.PRB.DL.Avail, SF=CellMLB.CellCapacityScaleFactor, G=GBR bandwidth, SE=spectral efficiency, N=active UEs with floor=MinDlAvgToBeScheduledUeNum). Then PreferredPCellPriority/PreferredPccPriority, bandwidth, EARFCN. SmartCaFastSccCfgSwitch (CaAlgoExtSwitch) can try blind SCell configuration to shorten time-to-CA; it requires CaSmartSelectionSwitch ON. Does not take effect together with some PCC-anchoring enhancements (e.g. UlCaCapbBasedPccSelectionSw).</t>
         </is>
       </c>
       <c r="B42" s="19" t="n"/>
@@ -9341,7 +9341,7 @@
       <c r="I336" s="7" t="inlineStr"/>
       <c r="J336" s="7" t="inlineStr"/>
     </row>
-    <row r="337" ht="28" customHeight="1">
+    <row r="337" ht="40" customHeight="1">
       <c r="A337" s="34" t="n">
         <v>47</v>
       </c>
@@ -9367,7 +9367,7 @@
       </c>
       <c r="F337" s="31" t="inlineStr">
         <is>
-          <t>Base RSRP threshold for CA event A4 (SCell add).</t>
+          <t>Base RSRP threshold for CA SCell-add event A4 (CaMgtCfg.CarrAggrA4ThdRsrp). Not the SC/PCC-anchor A4 (PCellA4RsrpThd/PccA4RsrpThd) and not coverage HO A4 (InterFreqHoA4ThdRsrp).</t>
         </is>
       </c>
       <c r="G337" s="31" t="inlineStr">
@@ -23050,7 +23050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J189"/>
+  <dimension ref="A1:J190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -23418,7 +23418,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>Trigger is uplink SINR used in scheduling (initial MCS selection), compared with CaMgtCfg.SpectrumCoordSinrThld.  Doc optimization MML sets SpectrumCoordSinrThld = −2 on every original PCell.  This is NOT CA event A1–A6 as the trigger (A4/A2 are used afterwards to pick the target SCell and to manage SCells).</t>
+          <t>Trigger is uplink SINR used in scheduling (initial MCS selection), compared with CaMgtCfg.SpectrumCoordSinrThld.  Doc optimization MML sets SpectrumCoordSinrThld = −2 on every original PCell.  This is NOT CA event A1–A6 as the trigger. After the SINR trigger, target SCell suitability uses PCellA4RsrpThd/PccA4RsrpThd; post-HO SCell leave uses CarrAggrA2ThdRsrp + SccA2Offset [+ SccA2RsrpThldExtendedOfs].</t>
         </is>
       </c>
       <c r="B33" s="17" t="n"/>
@@ -23503,10 +23503,10 @@
       <c r="I37" s="22" t="n"/>
       <c r="J37" s="22" t="n"/>
     </row>
-    <row r="38" ht="130" customHeight="1">
+    <row r="38" ht="155" customHeight="1">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>•  Downlink signal strength of that SCell reaches the RSRP threshold for event A4  AND  is higher than all of its intra-frequency neighboring cells. If either fails, the SCell is not a target.
+          <t>•  Downlink RSRP of that SCell reaches CaGroupCell.PCellA4RsrpThd (group) or PccFreqCfg.PccA4RsrpThd (adaptive)  AND  is higher than all of its intra-frequency neighboring cells. If either fails, the SCell is not a target. This is NOT CaMgtCfg.CarrAggrA4ThdRsrp (that is CA SCell-add A4).
 •  Recommendation (Ch.4.1): CaGroupCell.PCellA4RsrpThd (group) or PccFreqCfg.PccA4RsrpThd (adaptive)  &gt;  InterFreqHoGroup.InterFreqHoA4ThdRsrp, to prevent a decrease in handover success rate.
 •  The SCell must also meet PCell conditions (see Carrier Aggregation FPD — this workbook Step1).
 •  If no downlink SCell meets the conditions: eNodeB does not initiate an inter-frequency handover.
@@ -23528,7 +23528,7 @@
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
         <is>
-          <t>B2 worked example  —  is this SCell a legal SC target?  (A4 + strongest intra-freq)</t>
+          <t>B2 worked example  —  is this SCell a legal SC target?  (PCellA4RsrpThd/PccA4RsrpThd + strongest intra-freq)</t>
         </is>
       </c>
       <c r="B39" s="6" t="n"/>
@@ -23541,13 +23541,13 @@
       <c r="I39" s="6" t="n"/>
       <c r="J39" s="6" t="n"/>
     </row>
-    <row r="40" ht="76" customHeight="1">
+    <row r="40" ht="80" customHeight="1">
       <c r="A40" s="27" t="inlineStr">
         <is>
           <t>3GPP / Huawei condition:
-SCell is suitable iff  (SCell RSRP reaches CA event A4)  AND  (SCell RSRP &gt; every intra-frequency neighbor of that SCell).
-CA A4 entering (this workbook / CA FPD Ch.4.3):  Mn + Ofn + Ocn − Hys  &gt;  Thresh
-Thresh = CarrAggrA4ThdRsrp + SCellA4Offset/SccA4Offset  (offsets 0 in the CA FPD MML examples).</t>
+SCell is suitable iff  (SCell RSRP reaches CaGroupCell.PCellA4RsrpThd [group] or PccFreqCfg.PccA4RsrpThd [adaptive])  AND  (SCell RSRP &gt; every intra-frequency neighbor of that SCell).
+Keep PCellA4RsrpThd/PccA4RsrpThd &gt; InterFreqHoGroup.InterFreqHoA4ThdRsrp so SC HO does not steal coverage HO.
+CA SCell-add A4 (used later for carrier management) is separate: CaMgtCfg.CarrAggrA4ThdRsrp + CaGroupSCellCfg.SCellA4Offset (group) or SccFreqCfg.SccA4Offset (adaptive).</t>
         </is>
       </c>
       <c r="B40" s="28" t="n"/>
@@ -23604,12 +23604,12 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Intelligent selection OFF (CaSmartSelectionSwitch)</t>
+          <t>CaSmartSelectionSwitch OFF</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Intelligent selection ON</t>
+          <t>CaSmartSelectionSwitch ON</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
@@ -23620,7 +23620,7 @@
       <c r="I43" s="7" t="inlineStr"/>
       <c r="J43" s="7" t="inlineStr"/>
     </row>
-    <row r="44" ht="40" customHeight="1">
+    <row r="44" ht="56" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
           <t>1</t>
@@ -23628,12 +23628,12 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>Highest PCell priority (CaGroupCell.PreferredPCellPriority) or PCC priority (PccFreqCfg.PreferredPccPriority)</t>
+          <t>Highest CaGroupCell.PreferredPCellPriority (group) or PccFreqCfg.PreferredPccPriority (adaptive)</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Highest downlink air interface capability (see CA FPD)</t>
+          <t>Highest DL air interface capability (CA FPD Ch.12). CaMgtCfg.MinDlAvgToBeScheduledUeNum=0 → P×SF×SE−G; else (P×SF×SE−G)/N. P=L.ChMeas.PRB.DL.Avail, SF=CellMLB.CellCapacityScaleFactor, G=GBR BW, SE=spectral efficiency, N=active UEs (floor=MinDlAvgToBeScheduledUeNum)</t>
         </is>
       </c>
       <c r="D44" s="10" t="n"/>
@@ -23644,7 +23644,7 @@
       <c r="I44" s="10" t="n"/>
       <c r="J44" s="11" t="n"/>
     </row>
-    <row r="45" ht="40" customHeight="1">
+    <row r="45" ht="56" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
           <t>2</t>
@@ -23652,12 +23652,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>If still tied: largest bandwidth</t>
+          <t>If still tied: largest cell bandwidth</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>If still tied: highest PCell / PCC priority (same MOs as left)</t>
+          <t>If still tied: highest PreferredPCellPriority / PreferredPccPriority</t>
         </is>
       </c>
       <c r="D45" s="10" t="n"/>
@@ -23668,7 +23668,7 @@
       <c r="I45" s="10" t="n"/>
       <c r="J45" s="11" t="n"/>
     </row>
-    <row r="46" ht="40" customHeight="1">
+    <row r="46" ht="56" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
           <t>3</t>
@@ -23676,12 +23676,12 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>If still tied: lowest center frequency</t>
+          <t>If still tied: lowest center frequency (EARFCN)</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>If still tied: larger bandwidth; then lowest center frequency</t>
+          <t>If still tied: larger bandwidth, then lowest EARFCN</t>
         </is>
       </c>
       <c r="D46" s="10" t="n"/>
@@ -23711,8 +23711,8 @@
     <row r="48" ht="88" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Doc 3CC optimization MML uses three downlink EARFCNs 123 / 567 / 890 as PCC/SCC pairs. Sample (intelligent selection OFF):
-UE PCell = high-frequency cell on EARFCN 890, UL SINR = −3 dB &lt; −2 dB → SC starts. Two DL SCells both pass A4+strongest:
+          <t>Doc 3CC optimization MML uses three downlink EARFCNs 123 / 567 / 890 as PCC/SCC pairs. Sample (ENodeBAlgoSwitch.CaAlgoSwitch / CaSmartSelectionSwitch OFF):
+UE PCell = high-frequency cell on EARFCN 890, UL SINR = −3 dB &lt; −2 dB → SC starts. Two DL SCells both pass PCellA4RsrpThd/PccA4RsrpThd + strongest:
   Cell A  EARFCN 123, PreferredPccPriority=2, BW=10 MHz
   Cell B  EARFCN 567, PreferredPccPriority=2, BW=20 MHz
 Same PCC priority → pick largest bandwidth → Cell B. After HO: PCell = Cell B, original 890-cell becomes SCell. If both had BW=20 MHz, pick the lower EARFCN (123).</t>
@@ -23795,7 +23795,7 @@
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="26" t="inlineStr">
         <is>
-          <t>C2.  SccA2RsrpThldExtendedOfs ≠ 0  and intelligent selection ON  (Ch.4.1 steps i–iv)</t>
+          <t>C2.  SccA2RsrpThldExtendedOfs ≠ 0  and CaSmartSelectionSwitch ON  (Ch.4.1 steps i–iv)</t>
         </is>
       </c>
       <c r="B53" s="6" t="n"/>
@@ -23818,7 +23818,7 @@
 If RSRP meets the new condition → remove SCell (end).
 If not → delete previous A2 cfg; deliver new A2 cfg + A1 cfg for this SCell.
     A1 threshold  =  CarrAggrA4ThdRsrp + SccA4Offset
-Before further A2/A1, intelligent selection may pick a better SCell.
+Before further A2/A1, CaSmartSelectionSwitch may pick a better SCell using the Ch.12 DL air interface capability formula (MinDlAvgToBeScheduledUeNum).
 Further A2 containing this SCell → remove it.  A1 containing this SCell → release new A2, restore previous A2 (threshold back to CarrAggrA2ThdRsrp + SccA2Offset).</t>
         </is>
       </c>
@@ -23840,7 +23840,7 @@
 First A2 thresh = −115 dBm. New A2 thresh = −115 + 0 + (−10) = −125 dBm.
 SCell RSRP in the report = −118 dBm.
 −118 meets first A2 (below −115) but does NOT meet new A2 (need to be below −125).
-Result: SCell is NOT removed on the first A2. eNodeB switches to the extended A2 + A1 pair (A1 thresh = −105 dBm) and intelligent selection may replace the SCell. If a later A2 still contains this SCell, it is removed.</t>
+Result: SCell is NOT removed on the first A2. eNodeB switches to the extended A2 + A1 pair (A1 thresh = CarrAggrA4ThdRsrp + SccA4Offset = −105 dBm) and CaSmartSelectionSwitch may replace the SCell. If a later A2 still contains this SCell, it is removed.</t>
         </is>
       </c>
       <c r="B55" s="14" t="n"/>
@@ -23856,7 +23856,7 @@
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="21" t="inlineStr">
         <is>
-          <t>C3.  SccA2RsrpThldExtendedOfs ≠ 0  and intelligent selection OFF</t>
+          <t>C3.  SccA2RsrpThldExtendedOfs ≠ 0  and CaSmartSelectionSwitch OFF</t>
         </is>
       </c>
       <c r="B56" s="22" t="n"/>
@@ -25147,7 +25147,7 @@
       </c>
       <c r="F94" s="31" t="inlineStr">
         <is>
-          <t>First tie-break among multiple SC target SCells when intelligent selection is OFF (and second tie-break when ON).</t>
+          <t>First tie-break among multiple SC target SCells when CaSmartSelectionSwitch is OFF (and second tie-break when ON).</t>
         </is>
       </c>
       <c r="G94" s="31" t="inlineStr">
@@ -25159,7 +25159,7 @@
       <c r="I94" s="10" t="n"/>
       <c r="J94" s="11" t="n"/>
     </row>
-    <row r="95" ht="40" customHeight="1">
+    <row r="95" ht="64" customHeight="1">
       <c r="A95" s="34" t="n">
         <v>12</v>
       </c>
@@ -25185,7 +25185,7 @@
       </c>
       <c r="F95" s="31" t="inlineStr">
         <is>
-          <t>Intelligent selection of serving cell combinations. Changes B3 selection order and C2 vs C3 A2 handling.</t>
+          <t>ENodeBAlgoSwitch.CaAlgoSwitch bit CaSmartSelectionSwitch. ON: first pick among SC targets is highest DL air interface capability (CaMgtCfg.MinDlAvgToBeScheduledUeNum formula). OFF: first pick is PreferredPCellPriority/PreferredPccPriority. Also changes C2 vs C3 A2 handling.</t>
         </is>
       </c>
       <c r="G95" s="31" t="inlineStr">
@@ -27511,7 +27511,7 @@
       <c r="I174" s="7" t="inlineStr"/>
       <c r="J174" s="7" t="inlineStr"/>
     </row>
-    <row r="175" ht="52" customHeight="1">
+    <row r="175" ht="82" customHeight="1">
       <c r="A175" s="35" t="inlineStr">
         <is>
           <t>What it is (10 s)</t>
@@ -27531,7 +27531,7 @@
       <c r="I175" s="10" t="n"/>
       <c r="J175" s="11" t="n"/>
     </row>
-    <row r="176" ht="52" customHeight="1">
+    <row r="176" ht="72" customHeight="1">
       <c r="A176" s="35" t="inlineStr">
         <is>
           <t>Q1. Is the low-band SCell already configured with this PCell?</t>
@@ -27551,7 +27551,7 @@
       <c r="I176" s="10" t="n"/>
       <c r="J176" s="11" t="n"/>
     </row>
-    <row r="177" ht="52" customHeight="1">
+    <row r="177" ht="116" customHeight="1">
       <c r="A177" s="35" t="inlineStr">
         <is>
           <t>Q2. If the UE has several SCells, which one becomes the new PCell?</t>
@@ -27559,7 +27559,8 @@
       </c>
       <c r="B177" s="29" t="inlineStr">
         <is>
-          <t>Only SCells that pass ALL of: (a) better uplink than the current PCell, (b) DL RSRP reaches CA event A4, (c) stronger than all intra-frequency neighbors of that SCell, (d) allowed to be a PCell. If only one SCell passes → HO to that one. If two or more pass → pick by rule: highest PCell/PCC priority, then largest bandwidth, then lowest EARFCN. If intelligent selection is ON, DL air-interface capability is used first, then the same ties. UL SCells are never chosen as the target.</t>
+          <t>Only existing DL SCells that pass ALL of: (a) better uplink than the current PCell; (b) DL RSRP reaches CaGroupCell.PCellA4RsrpThd (group) or PccFreqCfg.PccA4RsrpThd (adaptive) — keep this &gt; InterFreqHoGroup.InterFreqHoA4ThdRsrp; do not confuse with CA SCell-add CaMgtCfg.CarrAggrA4ThdRsrp; (c) stronger than all intra-frequency neighbors of that SCell; (d) allowed to be a PCell. UL SCells are never the target (CaMgtCfg.CellCaAlgoSwitch / CaUl2CCSwitch UEs with UL2CC+DL2CC are excluded).
+One candidate → HO to it. Several candidates → see next row for the pick order.</t>
         </is>
       </c>
       <c r="C177" s="10" t="n"/>
@@ -27571,19 +27572,17 @@
       <c r="I177" s="10" t="n"/>
       <c r="J177" s="11" t="n"/>
     </row>
-    <row r="178" ht="118" customHeight="1">
+    <row r="178" ht="140" customHeight="1">
       <c r="A178" s="35" t="inlineStr">
         <is>
-          <t>What “DL still uses both bands, UL rides the coverage layer” means</t>
+          <t>How the eNodeB picks among several legal SCells</t>
         </is>
       </c>
       <c r="B178" s="9" t="inlineStr">
         <is>
-          <t>Coverage layer = low frequency (better uplink reach). Capacity layer = high frequency (more downlink speed, weaker uplink at the edge).
-In normal LTE CA without UL CA, upload (PUSCH/PUCCH) is only on the PCell. Download can use PCell + SCell.
-BEFORE swap: PCell=high band → upload is on high band (often too weak at the edge); download = high + low.
-AFTER swap: PCell=low band → upload is on low band (coverage layer, stronger); the high band is still an SCell so download is still high + low.
-So download does not lose the high band. Only the upload home cell changes. That is why cell-edge users can keep high-band download while their upload survives.</t>
+          <t>Switch: ENodeBAlgoSwitch.CaAlgoSwitch → CaSmartSelectionSwitch.
+OFF: 1) highest CaGroupCell.PreferredPCellPriority (group) or PccFreqCfg.PreferredPccPriority (adaptive)  2) largest cell bandwidth  3) lowest center frequency (EARFCN).
+ON: 1) highest downlink air interface capability of the cell, from CA FPD Ch.12: if CaMgtCfg.MinDlAvgToBeScheduledUeNum=0 then P×SF×SE−G, else (P×SF×SE−G)/N. P = L.ChMeas.PRB.DL.Avail; SF = CellMLB.CellCapacityScaleFactor; G = GBR bandwidth in the cell; SE = cell spectral efficiency; N = active UEs (floor = MinDlAvgToBeScheduledUeNum).  2) same PreferredPCellPriority / PreferredPccPriority  3) larger bandwidth  4) lowest EARFCN.</t>
         </is>
       </c>
       <c r="C178" s="10" t="n"/>
@@ -27595,15 +27594,19 @@
       <c r="I178" s="10" t="n"/>
       <c r="J178" s="11" t="n"/>
     </row>
-    <row r="179" ht="52" customHeight="1">
+    <row r="179" ht="168" customHeight="1">
       <c r="A179" s="35" t="inlineStr">
         <is>
-          <t>Benefit (1–2 lines)</t>
+          <t>What “DL still uses both bands, UL rides the coverage layer” means</t>
         </is>
       </c>
       <c r="B179" s="29" t="inlineStr">
         <is>
-          <t>It lifts DL usage of CA UEs at the high-frequency UL coverage edge. Best when high/low gap is large. Scenario 1 (both bands already on): PUSCH MCS 0–3 &gt;10% on high band, low-minus-high UL interference &lt;5 dB, CA UE penetration &gt;25% → network User DL Average Throughput up. Scenario 2 (adding a new low band under an existing high band) → both User DL and User UL Average Throughput up.</t>
+          <t>Coverage layer = low frequency (better uplink reach). Capacity layer = high frequency (more downlink speed, weaker uplink at the edge).
+In normal LTE CA without UL CA, upload (PUSCH/PUCCH) is only on the PCell. Download can use PCell + SCell.
+BEFORE swap: PCell=high band → upload is on high band (often too weak at the edge); download = high + low.
+AFTER swap: PCell=low band → upload is on low band (coverage layer, stronger); the high band is still an SCell so download is still high + low.
+So download does not lose the high band. Only the upload home cell changes. That is why cell-edge users can keep high-band download while their upload survives.</t>
         </is>
       </c>
       <c r="C179" s="10" t="n"/>
@@ -27615,15 +27618,15 @@
       <c r="I179" s="10" t="n"/>
       <c r="J179" s="11" t="n"/>
     </row>
-    <row r="180" ht="52" customHeight="1">
+    <row r="180" ht="82" customHeight="1">
       <c r="A180" s="35" t="inlineStr">
         <is>
-          <t>Trigger</t>
+          <t>Benefit (1–2 lines)</t>
         </is>
       </c>
       <c r="B180" s="9" t="inlineStr">
         <is>
-          <t>CA UE already aggregating. UL SINR used in scheduling (initial MCS) &lt; SpectrumCoordSinrThld (doc MML −2 dB). Then a DL SCell must pass A4 AND be stronger than all its intra-freq neighbours, and must be allowed as PCell. Target pick: PCell/PCC priority → largest BW → lowest EARFCN (or DL air-interface capability first if intelligent selection is ON).</t>
+          <t>It lifts DL usage of CA UEs at the high-frequency UL coverage edge. Best when high/low gap is large. Scenario 1 (both bands already on): PUSCH MCS 0–3 &gt;10% on high band, low-minus-high UL interference &lt;5 dB, CA UE penetration &gt;25% → network User DL Average Throughput up. Scenario 2 (adding a new low band under an existing high band) → both User DL and User UL Average Throughput up.</t>
         </is>
       </c>
       <c r="C180" s="10" t="n"/>
@@ -27635,15 +27638,15 @@
       <c r="I180" s="10" t="n"/>
       <c r="J180" s="11" t="n"/>
     </row>
-    <row r="181" ht="52" customHeight="1">
+    <row r="181" ht="122" customHeight="1">
       <c r="A181" s="35" t="inlineStr">
         <is>
-          <t>Leave / after HO</t>
+          <t>Trigger</t>
         </is>
       </c>
       <c r="B181" s="29" t="inlineStr">
         <is>
-          <t>After HO, original SCell = new PCell and original PCell = SCell. In adaptive CA, SCell A2 then manages the old high band (SccA2RsrpThldExtendedOfs; doc −10). Operator off: SpectrumCoordinationSwitch-0. Not a coverage HO; extra HOs raise count, can cut DRX UEs and may drop VoLTE MOS.</t>
+          <t>CA UE already aggregating. UL SINR used in scheduling (initial MCS) &lt; CaMgtCfg.SpectrumCoordSinrThld (doc MML −2 dB). Then a DL SCell must reach CaGroupCell.PCellA4RsrpThd (group) or PccFreqCfg.PccA4RsrpThd (adaptive), AND be stronger than all intra-freq neighbours, AND be allowed as PCell. Recommend PCellA4RsrpThd/PccA4RsrpThd &gt; InterFreqHoGroup.InterFreqHoA4ThdRsrp. Target pick: if ENodeBAlgoSwitch.CaAlgoSwitch / CaSmartSelectionSwitch OFF → CaGroupCell.PreferredPCellPriority or PccFreqCfg.PreferredPccPriority → largest BW → lowest EARFCN. If CaSmartSelectionSwitch ON → highest DL air interface capability first (CaMgtCfg.MinDlAvgToBeScheduledUeNum=0 → P×SF×SE−G else (P×SF×SE−G)/N; P=L.ChMeas.PRB.DL.Avail, SF=CellMLB.CellCapacityScaleFactor), then the same ties.</t>
         </is>
       </c>
       <c r="C181" s="10" t="n"/>
@@ -27655,15 +27658,15 @@
       <c r="I181" s="10" t="n"/>
       <c r="J181" s="11" t="n"/>
     </row>
-    <row r="182" ht="52" customHeight="1">
+    <row r="182" ht="72" customHeight="1">
       <c r="A182" s="35" t="inlineStr">
         <is>
-          <t>Must-on conditions</t>
+          <t>Leave / after HO</t>
         </is>
       </c>
       <c r="B182" s="9" t="inlineStr">
         <is>
-          <t>HoAdmitSwitch OFF; HoWithSccCfgSwitch ON; SpectrumCoordinationSwitch ON. After enable also ON: CaEnhancedPreAllocSwitch, Dl2CCAckResShareSw, SccA2RmvSwitch. UE must support CA. CA already live (DL 2–8 CC).</t>
+          <t>After HO, original SCell = new PCell and original PCell = SCell. In adaptive CA, SCell A2 then manages the old high band (SccA2RsrpThldExtendedOfs; doc −10). Operator off: SpectrumCoordinationSwitch-0. Not a coverage HO; extra HOs raise count, can cut DRX UEs and may drop VoLTE MOS.</t>
         </is>
       </c>
       <c r="C182" s="10" t="n"/>
@@ -27675,15 +27678,15 @@
       <c r="I182" s="10" t="n"/>
       <c r="J182" s="11" t="n"/>
     </row>
-    <row r="183" ht="52" customHeight="1">
+    <row r="183" ht="62" customHeight="1">
       <c r="A183" s="35" t="inlineStr">
         <is>
-          <t>Applicable case</t>
+          <t>Must-on conditions</t>
         </is>
       </c>
       <c r="B183" s="29" t="inlineStr">
         <is>
-          <t>Multi-band CA cluster with overlapping high + low (FPD example 2600 + 850 MHz). Intra-eNodeB. Macro 3900/5900; TDD also LampSite. Not LBBPc.</t>
+          <t>HoAdmitSwitch OFF; HoWithSccCfgSwitch ON; SpectrumCoordinationSwitch ON. After enable also ON: CaEnhancedPreAllocSwitch, Dl2CCAckResShareSw, SccA2RmvSwitch. UE must support CA. CA already live (DL 2–8 CC).</t>
         </is>
       </c>
       <c r="C183" s="10" t="n"/>
@@ -27698,12 +27701,12 @@
     <row r="184" ht="52" customHeight="1">
       <c r="A184" s="35" t="inlineStr">
         <is>
-          <t>UL / DL CA limitation</t>
+          <t>Applicable case</t>
         </is>
       </c>
       <c r="B184" s="9" t="inlineStr">
         <is>
-          <t>Compatible with DL 2CC–8CC. Does NOT take effect if the UE has 2 CC in UL and 2 CC in DL (UL SCells are never SC targets). If UL is 2 CC and DL is 3–8 CC, it does take effect. This is not UL CA; it only moves which cell is PCell so UL uses the low band.</t>
+          <t>Multi-band CA cluster with overlapping high + low (FPD example 2600 + 850 MHz). Intra-eNodeB. Macro 3900/5900; TDD also LampSite. Not LBBPc.</t>
         </is>
       </c>
       <c r="C184" s="10" t="n"/>
@@ -27715,15 +27718,15 @@
       <c r="I184" s="10" t="n"/>
       <c r="J184" s="11" t="n"/>
     </row>
-    <row r="185" ht="52" customHeight="1">
+    <row r="185" ht="62" customHeight="1">
       <c r="A185" s="35" t="inlineStr">
         <is>
-          <t>GPS required?</t>
+          <t>UL / DL CA limitation</t>
         </is>
       </c>
       <c r="B185" s="29" t="inlineStr">
         <is>
-          <t>No extra GPS requirement in this FPD. SC is an intra-eNodeB PCell change + CA SCell keep. Site sync stays whatever LTE already needs (TDD still needs the site’s existing GPS/1588/sync; SC does not add a GPS license or a new sync feature).</t>
+          <t>Compatible with DL 2CC–8CC. Does NOT take effect if the UE has 2 CC in UL and 2 CC in DL (UL SCells are never SC targets). If UL is 2 CC and DL is 3–8 CC, it does take effect. This is not UL CA; it only moves which cell is PCell so UL uses the low band.</t>
         </is>
       </c>
       <c r="C185" s="10" t="n"/>
@@ -27735,15 +27738,15 @@
       <c r="I185" s="10" t="n"/>
       <c r="J185" s="11" t="n"/>
     </row>
-    <row r="186" ht="52" customHeight="1">
+    <row r="186" ht="62" customHeight="1">
       <c r="A186" s="35" t="inlineStr">
         <is>
-          <t>License (if asked)</t>
+          <t>GPS required?</t>
         </is>
       </c>
       <c r="B186" s="9" t="inlineStr">
         <is>
-          <t>FDD LCOFD-131312 model LT1SUNPLTE00 per cell; TDD TDLCOFD-131312 model LT1SLTESPC00 per cell. Enhancement uses the same license. CA licenses still required. License shortage can block ACT CELL.</t>
+          <t>No extra GPS requirement in this FPD. SC is an intra-eNodeB PCell change + CA SCell keep. Site sync stays whatever LTE already needs (TDD still needs the site’s existing GPS/1588/sync; SC does not add a GPS license or a new sync feature).</t>
         </is>
       </c>
       <c r="C186" s="10" t="n"/>
@@ -27755,15 +27758,15 @@
       <c r="I186" s="10" t="n"/>
       <c r="J186" s="11" t="n"/>
     </row>
-    <row r="187" ht="52" customHeight="1">
+    <row r="187" ht="62" customHeight="1">
       <c r="A187" s="35" t="inlineStr">
         <is>
-          <t>How we know it is working</t>
+          <t>License (if asked)</t>
         </is>
       </c>
       <c r="B187" s="29" t="inlineStr">
         <is>
-          <t>L.HHO.InterFreq.ULquality.Prep/Exec/Succ (1526729994 / 9996 / 9998) increase. Also watch CA PCell/SCell users and bits, CA UE DL rate, SCell add success (tied to HO success).</t>
+          <t>FDD LCOFD-131312 model LT1SUNPLTE00 per cell; TDD TDLCOFD-131312 model LT1SLTESPC00 per cell. Enhancement uses the same license. CA licenses still required. License shortage can block ACT CELL.</t>
         </is>
       </c>
       <c r="C187" s="10" t="n"/>
@@ -27778,12 +27781,12 @@
     <row r="188" ht="52" customHeight="1">
       <c r="A188" s="35" t="inlineStr">
         <is>
-          <t>Do not mix / watch-outs</t>
+          <t>How we know it is working</t>
         </is>
       </c>
       <c r="B188" s="9" t="inlineStr">
         <is>
-          <t>Not DSS, not GSM/UMTS spectrum sharing, not NR UL/DL decoupling. DSS / SUL DSS cut LTE UL RBs → fewer UEs get SC. NSA: may HO PCC off an NSA anchor — deselect SPCT_COORD_INTER_FREQ_HO_SW to exempt NSA UEs. Enhancement (WBB/RRN) is a different bit (WbbCaMultiCarrierCoordSw); NSA PCC anchoring wins over it. SCC coverage-threshold adaptation kills SC carrier management. More HOs; CQI/KPI move with the new PCell quality.</t>
+          <t>L.HHO.InterFreq.ULquality.Prep/Exec/Succ (1526729994 / 9996 / 9998) increase. Also watch CA PCell/SCell users and bits, CA UE DL rate, SCell add success (tied to HO success).</t>
         </is>
       </c>
       <c r="C188" s="10" t="n"/>
@@ -27795,19 +27798,15 @@
       <c r="I188" s="10" t="n"/>
       <c r="J188" s="11" t="n"/>
     </row>
-    <row r="189" ht="118" customHeight="1">
+    <row r="189" ht="82" customHeight="1">
       <c r="A189" s="35" t="inlineStr">
         <is>
-          <t>Plain-English close  (read this if the jargon is heavy)</t>
+          <t>Do not mix / watch-outs</t>
         </is>
       </c>
       <c r="B189" s="29" t="inlineStr">
         <is>
-          <t>1) First make normal Carrier Aggregation work between one high-frequency cell and one low-frequency cell (same site, overlapping coverage). If CA is not working, do not turn Spectrum Coordination on.
-2) Spectrum Coordination does not join two carriers by itself. CA already joined them. This feature only changes which of those two cells is the PCell (the cell that carries the uplink).
-3) When the UE is near the cell edge, uplink on the high band is weak (poor UL SINR). The eNodeB then makes the low-band cell the PCell so the UE transmits uplink on the low band (better coverage).
-4) The high-band cell is kept as an SCell, so downlink data can still use both bands. That is the gain: cell-edge users keep high-band download speed even when their upload cannot stay on the high band.
-5) Short version: CA = two pipes for download. Spectrum Coordination = move the upload pipe to the low band at the edge, without throwing away the high-band download pipe.</t>
+          <t>Not DSS, not GSM/UMTS spectrum sharing, not NR UL/DL decoupling. DSS / SUL DSS cut LTE UL RBs → fewer UEs get SC. NSA: may HO PCC off an NSA anchor — deselect SPCT_COORD_INTER_FREQ_HO_SW to exempt NSA UEs. Enhancement (WBB/RRN) is a different bit (WbbCaMultiCarrierCoordSw); NSA PCC anchoring wins over it. SCC coverage-threshold adaptation kills SC carrier management. More HOs; CQI/KPI move with the new PCell quality.</t>
         </is>
       </c>
       <c r="C189" s="10" t="n"/>
@@ -27819,8 +27818,32 @@
       <c r="I189" s="10" t="n"/>
       <c r="J189" s="11" t="n"/>
     </row>
+    <row r="190" ht="180" customHeight="1">
+      <c r="A190" s="35" t="inlineStr">
+        <is>
+          <t>Plain-English close  (read this if the jargon is heavy)</t>
+        </is>
+      </c>
+      <c r="B190" s="9" t="inlineStr">
+        <is>
+          <t>1) First make normal Carrier Aggregation work between one high-frequency cell and one low-frequency cell (same site, overlapping coverage). If CA is not working, do not turn Spectrum Coordination on.
+2) Spectrum Coordination does not join two carriers by itself. CA already joined them. This feature only changes which of those two cells is the PCell (the cell that carries the uplink).
+3) When the UE is near the cell edge, uplink on the high band is weak (poor UL SINR). The eNodeB then makes the low-band cell the PCell so the UE transmits uplink on the low band (better coverage).
+4) The high-band cell is kept as an SCell, so downlink data can still use both bands. That is the gain: cell-edge users keep high-band download speed even when their upload cannot stay on the high band.
+5) Short version: CA = two pipes for download. Spectrum Coordination = move the upload pipe to the low band at the edge, without throwing away the high-band download pipe.</t>
+        </is>
+      </c>
+      <c r="C190" s="10" t="n"/>
+      <c r="D190" s="10" t="n"/>
+      <c r="E190" s="10" t="n"/>
+      <c r="F190" s="10" t="n"/>
+      <c r="G190" s="10" t="n"/>
+      <c r="H190" s="10" t="n"/>
+      <c r="I190" s="10" t="n"/>
+      <c r="J190" s="11" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="166">
+  <mergeCells count="167">
     <mergeCell ref="E138:J138"/>
     <mergeCell ref="E143:J143"/>
     <mergeCell ref="G109:J109"/>
@@ -27940,6 +27963,7 @@
     <mergeCell ref="E151:J151"/>
     <mergeCell ref="A164:J164"/>
     <mergeCell ref="G78:J78"/>
+    <mergeCell ref="B190:J190"/>
     <mergeCell ref="A56:J56"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="G87:J87"/>

</xml_diff>